<commit_message>
Fix band phrases that broke the sentences quoting them
Four risk blocks read as broken English once a real answer filled the slot.
"most of it of what a buyer would be paying for is you", because the band
already carried the words the sentence then repeated. Another stopped mid
thought at "the way you spend your week is partly".

Caught by rendering every flag raising option against every sentence that
quotes it, rather than reading the one that happened to show up on screen.

Sentence case is now applied after a slot is filled instead of being written
into the band by hand. Bands are written lower case so they read mid sentence,
and a block reworded later can put one at the start of a sentence without
anybody noticing. Doing it in the engine means that cannot come back.

Co-Authored-By: Claude Opus 5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01EA6msubCCPndLhAZDV4oLH
</commit_message>
<xml_diff>
--- a/diagnostic/Business-Diagnostic-Spec.xlsx
+++ b/diagnostic/Business-Diagnostic-Spec.xlsx
@@ -13282,7 +13282,7 @@
       </c>
       <c r="F233" s="7" t="inlineStr">
         <is>
-          <t>most of it</t>
+          <t>Most</t>
         </is>
       </c>
       <c r="G233" s="5" t="inlineStr"/>
@@ -13315,7 +13315,7 @@
       </c>
       <c r="F234" s="7" t="inlineStr">
         <is>
-          <t>some of it</t>
+          <t>Some</t>
         </is>
       </c>
       <c r="G234" s="5" t="inlineStr"/>
@@ -13352,7 +13352,7 @@
       </c>
       <c r="F235" s="7" t="inlineStr">
         <is>
-          <t>almost none of it</t>
+          <t>Almost none</t>
         </is>
       </c>
       <c r="G235" s="5" t="inlineStr"/>
@@ -13533,7 +13533,7 @@
       </c>
       <c r="F240" s="7" t="inlineStr">
         <is>
-          <t>not at all</t>
+          <t>next to never</t>
         </is>
       </c>
       <c r="G240" s="5" t="inlineStr"/>
@@ -13751,7 +13751,7 @@
       </c>
       <c r="F246" s="7" t="inlineStr">
         <is>
-          <t>almost none of it</t>
+          <t>almost none</t>
         </is>
       </c>
       <c r="G246" s="5" t="inlineStr"/>
@@ -13784,7 +13784,7 @@
       </c>
       <c r="F247" s="7" t="inlineStr">
         <is>
-          <t>some of it</t>
+          <t>some</t>
         </is>
       </c>
       <c r="G247" s="5" t="inlineStr"/>
@@ -13821,7 +13821,7 @@
       </c>
       <c r="F248" s="7" t="inlineStr">
         <is>
-          <t>most of it</t>
+          <t>most</t>
         </is>
       </c>
       <c r="G248" s="5" t="inlineStr"/>
@@ -13858,7 +13858,7 @@
       </c>
       <c r="F249" s="7" t="inlineStr">
         <is>
-          <t>all of it</t>
+          <t>all</t>
         </is>
       </c>
       <c r="G249" s="5" t="inlineStr"/>
@@ -13932,7 +13932,7 @@
       </c>
       <c r="F251" s="7" t="inlineStr">
         <is>
-          <t>written down</t>
+          <t>a written plan</t>
         </is>
       </c>
       <c r="G251" s="5" t="inlineStr"/>
@@ -14076,7 +14076,7 @@
       </c>
       <c r="F255" s="7" t="inlineStr">
         <is>
-          <t>nothing</t>
+          <t>none</t>
         </is>
       </c>
       <c r="G255" s="5" t="inlineStr"/>
@@ -14253,7 +14253,7 @@
       </c>
       <c r="F260" s="7" t="inlineStr">
         <is>
-          <t>partly</t>
+          <t>only partly a match for what you wanted</t>
         </is>
       </c>
       <c r="G260" s="5" t="inlineStr"/>
@@ -16959,7 +16959,7 @@
       </c>
       <c r="D12" s="7" t="inlineStr">
         <is>
-          <t>You've got {q46.band} of how the work gets done written down. Every new hire takes longer than it should, quality moves depending on who's on the job, and nothing can be handed over cleanly.</t>
+          <t>{q46.band} of how the work gets done is written down. Every new hire takes longer than it should, quality moves depending on who's on the job, and nothing can be handed over cleanly.</t>
         </is>
       </c>
       <c r="E12" s="7" t="inlineStr"/>

</xml_diff>

<commit_message>
Show which variables a block uses and where each one lands
The report tabs now carry a variables column, so somebody rewriting a block can
see what data they have to work with rather than going hunting for it. Taken
from the authoring template Ryan had from the planning chat, which had the idea
and nothing else in it.

The Data slots tab goes further and lists every phrase a variable can print,
which answers drop it, and the report blocks that quote it. Changing a band on
the Answer options tab now has a visible blast radius, which is the check that
would have caught the band phrases that broke the sentences quoting them.

It also flags an exact figure prompt that no block quotes. All nine currently
in the tool are used, so nothing is asking for a number for no reason.

Co-Authored-By: Claude Opus 5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01EA6msubCCPndLhAZDV4oLH
</commit_message>
<xml_diff>
--- a/diagnostic/Business-Diagnostic-Spec.xlsx
+++ b/diagnostic/Business-Diagnostic-Spec.xlsx
@@ -26,16 +26,16 @@
     <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="1">'Questions'!$A$2:$I$54</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="2" hidden="1">'Answer options'!$A$2:$I$262</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="3" hidden="1">'Constraints and order'!$A$2:$G$9</definedName>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="4" hidden="1">'Report, constraint'!$A$2:$D$96</definedName>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="5" hidden="1">'Report, minor'!$A$2:$C$9</definedName>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="6" hidden="1">'Report, risk flags'!$A$2:$G$18</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="4" hidden="1">'Report, constraint'!$A$2:$E$96</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="5" hidden="1">'Report, minor'!$A$2:$D$9</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="6" hidden="1">'Report, risk flags'!$A$2:$H$18</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="7" hidden="1">'Report, risk framing'!$A$2:$E$6</definedName>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="8" hidden="1">'Report, compound'!$A$2:$D$19</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="8" hidden="1">'Report, compound'!$A$2:$E$19</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="9" hidden="1">'Report, don''t do yet'!$A$2:$C$44</definedName>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="10" hidden="1">'Report, open and close'!$A$2:$D$12</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="10" hidden="1">'Report, open and close'!$A$2:$E$12</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="11" hidden="1">'Thresholds'!$A$2:$C$10</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="12" hidden="1">'Logic'!$A$1:$B$14</definedName>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="13" hidden="1">'Data slots'!$A$2:$G$36</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="13" hidden="1">'Data slots'!$A$2:$F$47</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
@@ -129,7 +129,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="9">
+  <cellXfs count="10">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment vertical="center" wrapText="1"/>
@@ -154,6 +154,9 @@
     </xf>
     <xf numFmtId="0" fontId="2" fillId="4" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment vertical="top"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="3" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment vertical="top" wrapText="1"/>
     </xf>
   </cellXfs>
   <cellStyles count="1">
@@ -520,7 +523,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:B25"/>
+  <dimension ref="A1:B26"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="26" customWidth="1" min="1" max="1"/>
@@ -575,227 +578,239 @@
       </c>
       <c r="B5" s="3" t="inlineStr">
         <is>
-          <t>Ids the engine matches on. Changing one breaks the link between a question, its answer and the report line that quotes it.</t>
+          <t>Ids the engine matches on, and columns it works out for you. Changing one breaks the link between a question, its answer and the report line that quotes it.</t>
         </is>
       </c>
     </row>
     <row r="6">
       <c r="A6" s="2" t="inlineStr">
         <is>
+          <t>Variables</t>
+        </is>
+      </c>
+      <c r="B6" s="3" t="inlineStr">
+        <is>
+          <t>Anything in {curly braces} is filled in from the answers. Write band phrases lower case, because sentence case is applied after a variable is filled in, so one landing at the start of a sentence gets capitalised for you.</t>
+        </is>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" s="2" t="inlineStr">
+        <is>
           <t>White cells</t>
         </is>
       </c>
-      <c r="B6" s="3" t="inlineStr">
+      <c r="B7" s="3" t="inlineStr">
         <is>
           <t>Numbers and settings. Safe to change, and the Thresholds tab explains what each one does.</t>
         </is>
       </c>
     </row>
-    <row r="7">
-      <c r="A7" s="2" t="inlineStr"/>
-      <c r="B7" s="3" t="inlineStr"/>
-    </row>
     <row r="8">
-      <c r="A8" s="2" t="inlineStr">
-        <is>
-          <t>The one rule</t>
-        </is>
-      </c>
-      <c r="B8" s="3" t="inlineStr">
-        <is>
-          <t>The report names one constraint. Not a list. If an edit starts adding a second finding, it is working against the tool.</t>
-        </is>
-      </c>
+      <c r="A8" s="2" t="inlineStr"/>
+      <c r="B8" s="3" t="inlineStr"/>
     </row>
     <row r="9">
       <c r="A9" s="2" t="inlineStr">
         <is>
-          <t>The second rule</t>
+          <t>The one rule</t>
         </is>
       </c>
       <c r="B9" s="3" t="inlineStr">
         <is>
-          <t>No scores, no grades, no dollar figures, no timeframes. None of those can be defended from banded answers.</t>
+          <t>The report names one constraint. Not a list. If an edit starts adding a second finding, it is working against the tool.</t>
         </is>
       </c>
     </row>
     <row r="10">
       <c r="A10" s="2" t="inlineStr">
         <is>
+          <t>The second rule</t>
+        </is>
+      </c>
+      <c r="B10" s="3" t="inlineStr">
+        <is>
+          <t>No scores, no grades, no dollar figures, no timeframes. None of those can be defended from banded answers.</t>
+        </is>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" s="2" t="inlineStr">
+        <is>
           <t>Voice</t>
         </is>
       </c>
-      <c r="B10" s="3" t="inlineStr">
+      <c r="B11" s="3" t="inlineStr">
         <is>
           <t>No dashes of any kind. No colons except before a list. Australian spelling. Contractions throughout.</t>
         </is>
       </c>
     </row>
-    <row r="11">
-      <c r="A11" s="2" t="inlineStr"/>
-      <c r="B11" s="3" t="inlineStr"/>
-    </row>
     <row r="12">
-      <c r="A12" s="2" t="inlineStr">
-        <is>
-          <t>Tabs, in order</t>
-        </is>
-      </c>
+      <c r="A12" s="2" t="inlineStr"/>
       <c r="B12" s="3" t="inlineStr"/>
     </row>
     <row r="13">
       <c r="A13" s="2" t="inlineStr">
         <is>
-          <t>Questions</t>
-        </is>
-      </c>
-      <c r="B13" s="3" t="inlineStr">
-        <is>
-          <t>All 52 questions. Wording, help text, which block each one feeds, how heavily it counts.</t>
-        </is>
-      </c>
+          <t>Tabs, in order</t>
+        </is>
+      </c>
+      <c r="B13" s="3" t="inlineStr"/>
     </row>
     <row r="14">
       <c r="A14" s="2" t="inlineStr">
         <is>
-          <t>Answer options</t>
+          <t>Questions</t>
         </is>
       </c>
       <c r="B14" s="3" t="inlineStr">
         <is>
-          <t>Every option under every question. This is where the bands live, and the band phrase is what gets quoted in the report.</t>
+          <t>All 52 questions. Wording, help text, which block each one feeds, how heavily it counts.</t>
         </is>
       </c>
     </row>
     <row r="15">
       <c r="A15" s="2" t="inlineStr">
         <is>
-          <t>Constraints and order</t>
+          <t>Answer options</t>
         </is>
       </c>
       <c r="B15" s="3" t="inlineStr">
         <is>
-          <t>The seven constraints, the fixed order they are checked in, and what suppresses what.</t>
+          <t>Every option under every question. This is where the bands live, and the band phrase is what gets quoted in the report.</t>
         </is>
       </c>
     </row>
     <row r="16">
       <c r="A16" s="2" t="inlineStr">
         <is>
-          <t>Report, constraint</t>
+          <t>Constraints and order</t>
         </is>
       </c>
       <c r="B16" s="3" t="inlineStr">
         <is>
-          <t>The constraint blocks. Opening line, evidence clauses, closing line, and the fix actions.</t>
+          <t>The seven constraints, the fixed order they are checked in, and what suppresses what.</t>
         </is>
       </c>
     </row>
     <row r="17">
       <c r="A17" s="2" t="inlineStr">
         <is>
-          <t>Report, minor</t>
+          <t>Report, constraint</t>
         </is>
       </c>
       <c r="B17" s="3" t="inlineStr">
         <is>
-          <t>The one line that prints when a second constraint is loud but downstream.</t>
+          <t>The constraint blocks. Opening line, evidence clauses, closing line, and the fix actions.</t>
         </is>
       </c>
     </row>
     <row r="18">
       <c r="A18" s="2" t="inlineStr">
         <is>
-          <t>Report, risk flags</t>
+          <t>Report, minor</t>
         </is>
       </c>
       <c r="B18" s="3" t="inlineStr">
         <is>
-          <t>All 16 risk flags. Definition, the version used when the answer was Not sure, and the fix.</t>
+          <t>The one line that prints when a second constraint is loud but downstream.</t>
         </is>
       </c>
     </row>
     <row r="19">
       <c r="A19" s="2" t="inlineStr">
         <is>
-          <t>Report, risk framing</t>
+          <t>Report, risk flags</t>
         </is>
       </c>
       <c r="B19" s="3" t="inlineStr">
         <is>
-          <t>The three family blocks and the minor risk lines.</t>
+          <t>All 16 risk flags. Definition, the version used when the answer was Not sure, and the fix.</t>
         </is>
       </c>
     </row>
     <row r="20">
       <c r="A20" s="2" t="inlineStr">
         <is>
-          <t>Report, compound</t>
+          <t>Report, risk framing</t>
         </is>
       </c>
       <c r="B20" s="3" t="inlineStr">
         <is>
-          <t>The blocks that fire when a risk and the constraint are the same problem seen twice.</t>
+          <t>The three family blocks and the minor risk lines.</t>
         </is>
       </c>
     </row>
     <row r="21">
       <c r="A21" s="2" t="inlineStr">
         <is>
-          <t>Report, don't do yet</t>
+          <t>Report, compound</t>
         </is>
       </c>
       <c r="B21" s="3" t="inlineStr">
         <is>
-          <t>The closing section. What not to touch until the constraint is fixed.</t>
+          <t>The blocks that fire when a risk and the constraint are the same problem seen twice.</t>
         </is>
       </c>
     </row>
     <row r="22">
       <c r="A22" s="2" t="inlineStr">
         <is>
-          <t>Report, open and close</t>
+          <t>Report, don't do yet</t>
         </is>
       </c>
       <c r="B22" s="3" t="inlineStr">
         <is>
-          <t>The opening and closing of the report, including the three opening variants.</t>
+          <t>The closing section. What not to touch until the constraint is fixed.</t>
         </is>
       </c>
     </row>
     <row r="23">
       <c r="A23" s="2" t="inlineStr">
         <is>
-          <t>Thresholds</t>
+          <t>Report, open and close</t>
         </is>
       </c>
       <c r="B23" s="3" t="inlineStr">
         <is>
-          <t>Every tunable number, and what moving it does.</t>
+          <t>The opening and closing of the report, including the three opening variants.</t>
         </is>
       </c>
     </row>
     <row r="24">
       <c r="A24" s="2" t="inlineStr">
         <is>
-          <t>Logic</t>
+          <t>Thresholds</t>
         </is>
       </c>
       <c r="B24" s="3" t="inlineStr">
         <is>
-          <t>How the engine picks the primary, the minor, and the risks. Read this before changing a threshold.</t>
+          <t>Every tunable number, and what moving it does.</t>
         </is>
       </c>
     </row>
     <row r="25">
       <c r="A25" s="2" t="inlineStr">
         <is>
+          <t>Logic</t>
+        </is>
+      </c>
+      <c r="B25" s="3" t="inlineStr">
+        <is>
+          <t>How the engine picks the primary, the minor, and the risks. Read this before changing a threshold.</t>
+        </is>
+      </c>
+    </row>
+    <row r="26">
+      <c r="A26" s="2" t="inlineStr">
+        <is>
           <t>Data slots</t>
         </is>
       </c>
-      <c r="B25" s="3" t="inlineStr">
-        <is>
-          <t>Which questions can be quoted in the report, and how.</t>
+      <c r="B26" s="3" t="inlineStr">
+        <is>
+          <t>Every variable, every phrase it can print, and which report blocks quote it. Check here before changing a band phrase, because it shows you the sentences that band lands in.</t>
         </is>
       </c>
     </row>
@@ -1571,13 +1586,14 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:D12"/>
+  <dimension ref="A1:E12"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="11" customWidth="1" min="1" max="1"/>
     <col width="13" customWidth="1" min="2" max="2"/>
-    <col width="52" customWidth="1" min="3" max="3"/>
-    <col width="108" customWidth="1" min="4" max="4"/>
+    <col width="48" customWidth="1" min="3" max="3"/>
+    <col width="98" customWidth="1" min="4" max="4"/>
+    <col width="24" customWidth="1" min="5" max="5"/>
   </cols>
   <sheetData>
     <row r="1" ht="30" customHeight="1">
@@ -1608,6 +1624,11 @@
           <t>Wording</t>
         </is>
       </c>
+      <c r="E2" s="1" t="inlineStr">
+        <is>
+          <t>Variables in this row</t>
+        </is>
+      </c>
     </row>
     <row r="3">
       <c r="A3" s="5" t="inlineStr">
@@ -1631,6 +1652,7 @@
 It names one constraint. There'll be other things wrong, there always are. They're not in here because the order you fix them in matters more than the list.</t>
         </is>
       </c>
+      <c r="E3" s="9" t="inlineStr"/>
     </row>
     <row r="4">
       <c r="A4" s="5" t="inlineStr">
@@ -1654,6 +1676,7 @@
 What follows is the tightest thing in the business rather than a problem. Treat it as where the next bit of growth will come from, not something to fix.</t>
         </is>
       </c>
+      <c r="E4" s="9" t="inlineStr"/>
     </row>
     <row r="5">
       <c r="A5" s="5" t="inlineStr">
@@ -1677,6 +1700,7 @@
 What follows is the tightest thing in the business right now rather than something that's failing outright. Treat it as the next thing to work on, not an emergency.</t>
         </is>
       </c>
+      <c r="E5" s="9" t="inlineStr"/>
     </row>
     <row r="6">
       <c r="A6" s="5" t="inlineStr">
@@ -1700,6 +1724,7 @@
 The finding below is the best available reading of what you did tell us. The bigger issue is that the business isn't visible to you, and that's covered in the risk section. Come back and run this again once you can answer the numbers.</t>
         </is>
       </c>
+      <c r="E6" s="9" t="inlineStr"/>
     </row>
     <row r="7">
       <c r="A7" s="5" t="inlineStr">
@@ -1722,6 +1747,11 @@
           <t>Nothing in here is failing, so there's no evidence to walk you through. What you've got is {d.primaryShort} sitting as the tightest of the seven right now, which makes it the likeliest place the next bit of growth comes from. The actions below are worth doing and none of them are urgent.</t>
         </is>
       </c>
+      <c r="E7" s="9" t="inlineStr">
+        <is>
+          <t>{d.primaryShort}</t>
+        </is>
+      </c>
     </row>
     <row r="8">
       <c r="A8" s="5" t="inlineStr">
@@ -1745,6 +1775,11 @@
 The risk section is the part of this report to take seriously. Not being able to answer the questions is the finding, and it's the one worth acting on first.</t>
         </is>
       </c>
+      <c r="E8" s="9" t="inlineStr">
+        <is>
+          <t>{d.primaryShort}</t>
+        </is>
+      </c>
     </row>
     <row r="9">
       <c r="A9" s="5" t="inlineStr">
@@ -1768,6 +1803,7 @@
 Work the constraint and check back in ninety days. That's long enough for it to move and short enough that you'll still remember what you changed.</t>
         </is>
       </c>
+      <c r="E9" s="9" t="inlineStr"/>
     </row>
     <row r="10">
       <c r="A10" s="5" t="inlineStr">
@@ -1791,6 +1827,7 @@
 Run this again in ninety days, or whenever something material changes. The constraint moves as the business grows, and the answer you get next time probably won't be this one.</t>
         </is>
       </c>
+      <c r="E10" s="9" t="inlineStr"/>
     </row>
     <row r="11">
       <c r="A11" s="5" t="inlineStr">
@@ -1814,6 +1851,7 @@
 Get the numbers visible, then run this again. The second time through it will be worth something.</t>
         </is>
       </c>
+      <c r="E11" s="9" t="inlineStr"/>
     </row>
     <row r="12">
       <c r="A12" s="5" t="inlineStr">
@@ -1832,11 +1870,12 @@
         </is>
       </c>
       <c r="D12" s="7" t="inlineStr"/>
+      <c r="E12" s="9" t="inlineStr"/>
     </row>
   </sheetData>
-  <autoFilter ref="A2:D12"/>
+  <autoFilter ref="A2:E12"/>
   <mergeCells count="1">
-    <mergeCell ref="A1:D1"/>
+    <mergeCell ref="A1:E1"/>
   </mergeCells>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
@@ -2186,1156 +2225,1406 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:G36"/>
+  <dimension ref="A1:F47"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
-    <col width="5" customWidth="1" min="1" max="1"/>
-    <col width="7" customWidth="1" min="2" max="2"/>
-    <col width="66" customWidth="1" min="3" max="3"/>
-    <col width="15" customWidth="1" min="4" max="4"/>
-    <col width="15" customWidth="1" min="5" max="5"/>
-    <col width="14" customWidth="1" min="6" max="6"/>
-    <col width="10" customWidth="1" min="7" max="7"/>
+    <col width="17" customWidth="1" min="1" max="1"/>
+    <col width="5" customWidth="1" min="2" max="2"/>
+    <col width="54" customWidth="1" min="3" max="3"/>
+    <col width="70" customWidth="1" min="4" max="4"/>
+    <col width="52" customWidth="1" min="5" max="5"/>
+    <col width="60" customWidth="1" min="6" max="6"/>
   </cols>
   <sheetData>
     <row r="1" ht="30" customHeight="1">
       <c r="A1" s="4" t="inlineStr">
         <is>
-          <t>An exact figure is only offered on questions whose answer actually reaches the report prose, not on all fifty two. Asking for a number the report never uses is friction for nothing.</t>
+          <t>An exact figure is only offered on questions whose answer actually reaches the report prose, not on all fifty two. Asking for a number the report never uses is friction for nothing. Sentence case is applied after a variable is filled in, so write band phrases lower case and let the engine capitalise the ones that land at the start of a sentence.</t>
         </is>
       </c>
     </row>
     <row r="2" ht="30" customHeight="1">
       <c r="A2" s="1" t="inlineStr">
         <is>
+          <t>Variable</t>
+        </is>
+      </c>
+      <c r="B2" s="1" t="inlineStr">
+        <is>
           <t>Q#</t>
         </is>
       </c>
-      <c r="B2" s="1" t="inlineStr">
-        <is>
-          <t>q id</t>
-        </is>
-      </c>
       <c r="C2" s="1" t="inlineStr">
         <is>
-          <t>Question</t>
+          <t>Question it comes from</t>
         </is>
       </c>
       <c r="D2" s="1" t="inlineStr">
         <is>
-          <t>Band quoted in the report</t>
+          <t>Every phrase it can print</t>
         </is>
       </c>
       <c r="E2" s="1" t="inlineStr">
         <is>
-          <t>Offers an exact figure</t>
+          <t>When it does not resolve</t>
         </is>
       </c>
       <c r="F2" s="1" t="inlineStr">
         <is>
-          <t>Exact figure quoted</t>
-        </is>
-      </c>
-      <c r="G2" s="1" t="inlineStr">
-        <is>
-          <t>Unit</t>
+          <t>Report blocks that quote it</t>
         </is>
       </c>
     </row>
     <row r="3">
-      <c r="A3" s="5" t="n">
+      <c r="A3" s="6" t="inlineStr">
+        <is>
+          <t>{q6.band}</t>
+        </is>
+      </c>
+      <c r="B3" s="5" t="n">
         <v>6</v>
       </c>
-      <c r="B3" s="6" t="inlineStr">
-        <is>
-          <t>q6</t>
-        </is>
-      </c>
       <c r="C3" s="3" t="inlineStr">
         <is>
-          <t xml:space="preserve">In the last 6 months, how often have you delayed paying a supplier, a </t>
-        </is>
-      </c>
-      <c r="D3" s="5" t="inlineStr">
-        <is>
-          <t>yes</t>
-        </is>
-      </c>
-      <c r="E3" s="5" t="inlineStr">
-        <is>
-          <t>no</t>
-        </is>
-      </c>
-      <c r="F3" s="5" t="inlineStr">
-        <is>
-          <t>no</t>
-        </is>
-      </c>
-      <c r="G3" s="5" t="inlineStr"/>
+          <t>In the last 6 months, how often have you delayed paying a supplier, a bill or yourself because the money hadn't landed yet?</t>
+        </is>
+      </c>
+      <c r="D3" s="3" t="inlineStr">
+        <is>
+          <t>never | once or twice | most months | every month</t>
+        </is>
+      </c>
+      <c r="E3" s="3" t="inlineStr">
+        <is>
+          <t>clause is dropped on: Not sure</t>
+        </is>
+      </c>
+      <c r="F3" s="3" t="inlineStr">
+        <is>
+          <t>constraintDef / cashflow / evidence [2] / banded</t>
+        </is>
+      </c>
     </row>
     <row r="4">
-      <c r="A4" s="5" t="n">
+      <c r="A4" s="6" t="inlineStr">
+        <is>
+          <t>{q7.band}</t>
+        </is>
+      </c>
+      <c r="B4" s="5" t="n">
         <v>7</v>
       </c>
-      <c r="B4" s="6" t="inlineStr">
-        <is>
-          <t>q7</t>
-        </is>
-      </c>
       <c r="C4" s="3" t="inlineStr">
         <is>
-          <t xml:space="preserve">From finishing a job to the money hitting your account, how long does </t>
-        </is>
-      </c>
-      <c r="D4" s="5" t="inlineStr">
-        <is>
-          <t>yes</t>
-        </is>
-      </c>
-      <c r="E4" s="5" t="inlineStr">
-        <is>
-          <t>yes</t>
-        </is>
-      </c>
-      <c r="F4" s="5" t="inlineStr">
-        <is>
-          <t>yes</t>
-        </is>
-      </c>
-      <c r="G4" s="5" t="inlineStr">
-        <is>
-          <t>days</t>
+          <t>From finishing a job to the money hitting your account, how long does it usually take?</t>
+        </is>
+      </c>
+      <c r="D4" s="3" t="inlineStr">
+        <is>
+          <t>upfront or on the day | inside a fortnight | in the 15 to 30 day range | in the 31 to 60 day range | beyond 60 days</t>
+        </is>
+      </c>
+      <c r="E4" s="3" t="inlineStr">
+        <is>
+          <t>clause is dropped on: Not sure</t>
+        </is>
+      </c>
+      <c r="F4" s="3" t="inlineStr">
+        <is>
+          <t>constraintDef / cashflow / evidence [1] / banded</t>
         </is>
       </c>
     </row>
     <row r="5">
-      <c r="A5" s="5" t="n">
+      <c r="A5" s="6" t="inlineStr">
+        <is>
+          <t>{q7.exact}</t>
+        </is>
+      </c>
+      <c r="B5" s="5" t="n">
+        <v>7</v>
+      </c>
+      <c r="C5" s="3" t="inlineStr">
+        <is>
+          <t>From finishing a job to the money hitting your account, how long does it usually take?</t>
+        </is>
+      </c>
+      <c r="D5" s="3" t="inlineStr">
+        <is>
+          <t>the number they typed, in days</t>
+        </is>
+      </c>
+      <c r="E5" s="3" t="inlineStr">
+        <is>
+          <t>optional, so the precise wording only prints when it was filled in</t>
+        </is>
+      </c>
+      <c r="F5" s="3" t="inlineStr">
+        <is>
+          <t>constraintDef / cashflow / evidence [1] / precise</t>
+        </is>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" s="6" t="inlineStr">
+        <is>
+          <t>{q8.band}</t>
+        </is>
+      </c>
+      <c r="B6" s="5" t="n">
         <v>8</v>
       </c>
-      <c r="B5" s="6" t="inlineStr">
-        <is>
-          <t>q8</t>
-        </is>
-      </c>
-      <c r="C5" s="3" t="inlineStr">
-        <is>
-          <t xml:space="preserve">If revenue stopped tomorrow, how long could you cover wages and fixed </t>
-        </is>
-      </c>
-      <c r="D5" s="5" t="inlineStr">
-        <is>
-          <t>yes</t>
-        </is>
-      </c>
-      <c r="E5" s="5" t="inlineStr">
-        <is>
-          <t>no</t>
-        </is>
-      </c>
-      <c r="F5" s="5" t="inlineStr">
-        <is>
-          <t>no</t>
-        </is>
-      </c>
-      <c r="G5" s="5" t="inlineStr"/>
-    </row>
-    <row r="6">
-      <c r="A6" s="5" t="n">
+      <c r="C6" s="3" t="inlineStr">
+        <is>
+          <t>If revenue stopped tomorrow, how long could you cover wages and fixed costs from the cash you have?</t>
+        </is>
+      </c>
+      <c r="D6" s="3" t="inlineStr">
+        <is>
+          <t>more than three months of cover | one to three months of cover | two to four weeks of cover | under a fortnight of cover</t>
+        </is>
+      </c>
+      <c r="E6" s="3" t="inlineStr">
+        <is>
+          <t>clause is dropped on: Not sure</t>
+        </is>
+      </c>
+      <c r="F6" s="3" t="inlineStr">
+        <is>
+          <t>constraintDef / cashflow / evidence [3] / banded  riskDef / no_buffer / banded</t>
+        </is>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" s="6" t="inlineStr">
+        <is>
+          <t>{q9.band}</t>
+        </is>
+      </c>
+      <c r="B7" s="5" t="n">
         <v>9</v>
       </c>
-      <c r="B6" s="6" t="inlineStr">
-        <is>
-          <t>q9</t>
-        </is>
-      </c>
-      <c r="C6" s="3" t="inlineStr">
-        <is>
-          <t>In the last 12 months, have you turned down or delayed work because yo</t>
-        </is>
-      </c>
-      <c r="D6" s="5" t="inlineStr">
-        <is>
-          <t>yes</t>
-        </is>
-      </c>
-      <c r="E6" s="5" t="inlineStr">
-        <is>
-          <t>no</t>
-        </is>
-      </c>
-      <c r="F6" s="5" t="inlineStr">
-        <is>
-          <t>no</t>
-        </is>
-      </c>
-      <c r="G6" s="5" t="inlineStr"/>
-    </row>
-    <row r="7">
-      <c r="A7" s="5" t="n">
+      <c r="C7" s="3" t="inlineStr">
+        <is>
+          <t>In the last 12 months, have you turned down or delayed work because you couldn't fund the upfront cost of it?</t>
+        </is>
+      </c>
+      <c r="D7" s="3" t="inlineStr">
+        <is>
+          <t>never | once | a few times | regularly</t>
+        </is>
+      </c>
+      <c r="E7" s="3" t="inlineStr">
+        <is>
+          <t>clause is dropped on: Not sure</t>
+        </is>
+      </c>
+      <c r="F7" s="3" t="inlineStr">
+        <is>
+          <t>constraintDef / cashflow / evidence [4] / banded</t>
+        </is>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" s="6" t="inlineStr">
+        <is>
+          <t>{q12.band}</t>
+        </is>
+      </c>
+      <c r="B8" s="5" t="n">
         <v>12</v>
       </c>
-      <c r="B7" s="6" t="inlineStr">
-        <is>
-          <t>q12</t>
-        </is>
-      </c>
-      <c r="C7" s="3" t="inlineStr">
+      <c r="C8" s="3" t="inlineStr">
         <is>
           <t>If you were uncontactable for a month, what happens to the business?</t>
         </is>
       </c>
-      <c r="D7" s="5" t="inlineStr">
-        <is>
-          <t>yes</t>
-        </is>
-      </c>
-      <c r="E7" s="5" t="inlineStr">
-        <is>
-          <t>no</t>
-        </is>
-      </c>
-      <c r="F7" s="5" t="inlineStr">
-        <is>
-          <t>no</t>
-        </is>
-      </c>
-      <c r="G7" s="5" t="inlineStr"/>
-    </row>
-    <row r="8">
-      <c r="A8" s="5" t="n">
+      <c r="D8" s="3" t="inlineStr">
+        <is>
+          <t>runs fine without you | runs, but the decisions wait for you | degrades quickly without you | stops without you</t>
+        </is>
+      </c>
+      <c r="E8" s="3" t="inlineStr">
+        <is>
+          <t>clause is dropped on: Not sure</t>
+        </is>
+      </c>
+      <c r="F8" s="3" t="inlineStr">
+        <is>
+          <t>constraintDef / talent / evidence [2] / banded</t>
+        </is>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" s="6" t="inlineStr">
+        <is>
+          <t>{q13.band}</t>
+        </is>
+      </c>
+      <c r="B9" s="5" t="n">
         <v>13</v>
       </c>
-      <c r="B8" s="6" t="inlineStr">
-        <is>
-          <t>q13</t>
-        </is>
-      </c>
-      <c r="C8" s="3" t="inlineStr">
+      <c r="C9" s="3" t="inlineStr">
         <is>
           <t>How much of your week goes to work someone a level below you could do?</t>
         </is>
       </c>
-      <c r="D8" s="5" t="inlineStr">
-        <is>
-          <t>yes</t>
-        </is>
-      </c>
-      <c r="E8" s="5" t="inlineStr">
-        <is>
-          <t>no</t>
-        </is>
-      </c>
-      <c r="F8" s="5" t="inlineStr">
-        <is>
-          <t>no</t>
-        </is>
-      </c>
-      <c r="G8" s="5" t="inlineStr"/>
-    </row>
-    <row r="9">
-      <c r="A9" s="5" t="n">
+      <c r="D9" s="3" t="inlineStr">
+        <is>
+          <t>almost none of your week | about a quarter of your week | about half your week | most of your week</t>
+        </is>
+      </c>
+      <c r="E9" s="3" t="inlineStr">
+        <is>
+          <t>clause is dropped on: Not sure</t>
+        </is>
+      </c>
+      <c r="F9" s="3" t="inlineStr">
+        <is>
+          <t>constraintDef / talent / evidence [1] / banded</t>
+        </is>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" s="6" t="inlineStr">
+        <is>
+          <t>{q14.band}</t>
+        </is>
+      </c>
+      <c r="B10" s="5" t="n">
         <v>14</v>
       </c>
-      <c r="B9" s="6" t="inlineStr">
-        <is>
-          <t>q14</t>
-        </is>
-      </c>
-      <c r="C9" s="3" t="inlineStr">
-        <is>
-          <t>In the last 12 months, has something you wanted to grow stalled becaus</t>
-        </is>
-      </c>
-      <c r="D9" s="5" t="inlineStr">
-        <is>
-          <t>yes</t>
-        </is>
-      </c>
-      <c r="E9" s="5" t="inlineStr">
-        <is>
-          <t>no</t>
-        </is>
-      </c>
-      <c r="F9" s="5" t="inlineStr">
-        <is>
-          <t>no</t>
-        </is>
-      </c>
-      <c r="G9" s="5" t="inlineStr"/>
-    </row>
-    <row r="10">
-      <c r="A10" s="5" t="n">
+      <c r="C10" s="3" t="inlineStr">
+        <is>
+          <t>In the last 12 months, has something you wanted to grow stalled because there was nobody to hand it to?</t>
+        </is>
+      </c>
+      <c r="D10" s="3" t="inlineStr">
+        <is>
+          <t>never | once | a few times | as a matter of routine</t>
+        </is>
+      </c>
+      <c r="E10" s="3" t="inlineStr">
+        <is>
+          <t>clause is dropped on: Not sure</t>
+        </is>
+      </c>
+      <c r="F10" s="3" t="inlineStr">
+        <is>
+          <t>constraintDef / talent / evidence [3] / banded</t>
+        </is>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" s="6" t="inlineStr">
+        <is>
+          <t>{q16.band}</t>
+        </is>
+      </c>
+      <c r="B11" s="5" t="n">
         <v>16</v>
       </c>
-      <c r="B10" s="6" t="inlineStr">
-        <is>
-          <t>q16</t>
-        </is>
-      </c>
-      <c r="C10" s="3" t="inlineStr">
+      <c r="C11" s="3" t="inlineStr">
         <is>
           <t>How booked is your delivery capacity for the next 30 days?</t>
         </is>
       </c>
-      <c r="D10" s="5" t="inlineStr">
-        <is>
-          <t>yes</t>
-        </is>
-      </c>
-      <c r="E10" s="5" t="inlineStr">
-        <is>
-          <t>yes</t>
-        </is>
-      </c>
-      <c r="F10" s="5" t="inlineStr">
-        <is>
-          <t>yes</t>
-        </is>
-      </c>
-      <c r="G10" s="5" t="inlineStr">
-        <is>
-          <t>%</t>
-        </is>
-      </c>
-    </row>
-    <row r="11">
-      <c r="A11" s="5" t="n">
+      <c r="D11" s="3" t="inlineStr">
+        <is>
+          <t>under half full | around two thirds full | at or near full | full, with people waiting | over capacity and behind</t>
+        </is>
+      </c>
+      <c r="E11" s="3" t="inlineStr">
+        <is>
+          <t>clause is dropped on: Not sure</t>
+        </is>
+      </c>
+      <c r="F11" s="3" t="inlineStr">
+        <is>
+          <t>constraintDef / fulfilment / evidence [1] / banded</t>
+        </is>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" s="6" t="inlineStr">
+        <is>
+          <t>{q16.exact}</t>
+        </is>
+      </c>
+      <c r="B12" s="5" t="n">
+        <v>16</v>
+      </c>
+      <c r="C12" s="3" t="inlineStr">
+        <is>
+          <t>How booked is your delivery capacity for the next 30 days?</t>
+        </is>
+      </c>
+      <c r="D12" s="3" t="inlineStr">
+        <is>
+          <t>the number they typed, in %</t>
+        </is>
+      </c>
+      <c r="E12" s="3" t="inlineStr">
+        <is>
+          <t>optional, so the precise wording only prints when it was filled in</t>
+        </is>
+      </c>
+      <c r="F12" s="3" t="inlineStr">
+        <is>
+          <t>constraintDef / fulfilment / evidence [1] / precise</t>
+        </is>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" s="6" t="inlineStr">
+        <is>
+          <t>{q17.band}</t>
+        </is>
+      </c>
+      <c r="B13" s="5" t="n">
         <v>17</v>
       </c>
-      <c r="B11" s="6" t="inlineStr">
-        <is>
-          <t>q17</t>
-        </is>
-      </c>
-      <c r="C11" s="3" t="inlineStr">
-        <is>
-          <t xml:space="preserve">In the last 6 months, have you turned work away or pushed out a start </t>
-        </is>
-      </c>
-      <c r="D11" s="5" t="inlineStr">
-        <is>
-          <t>yes</t>
-        </is>
-      </c>
-      <c r="E11" s="5" t="inlineStr">
-        <is>
-          <t>no</t>
-        </is>
-      </c>
-      <c r="F11" s="5" t="inlineStr">
-        <is>
-          <t>no</t>
-        </is>
-      </c>
-      <c r="G11" s="5" t="inlineStr"/>
-    </row>
-    <row r="12">
-      <c r="A12" s="5" t="n">
+      <c r="C13" s="3" t="inlineStr">
+        <is>
+          <t>In the last 6 months, have you turned work away or pushed out a start date because you couldn't fit it in?</t>
+        </is>
+      </c>
+      <c r="D13" s="3" t="inlineStr">
+        <is>
+          <t>never | once or twice | most months | constantly</t>
+        </is>
+      </c>
+      <c r="E13" s="3" t="inlineStr">
+        <is>
+          <t>clause is dropped on: Not sure</t>
+        </is>
+      </c>
+      <c r="F13" s="3" t="inlineStr">
+        <is>
+          <t>constraintDef / fulfilment / evidence [2] / banded</t>
+        </is>
+      </c>
+    </row>
+    <row r="14">
+      <c r="A14" s="6" t="inlineStr">
+        <is>
+          <t>{q18.band}</t>
+        </is>
+      </c>
+      <c r="B14" s="5" t="n">
         <v>18</v>
       </c>
-      <c r="B12" s="6" t="inlineStr">
-        <is>
-          <t>q18</t>
-        </is>
-      </c>
-      <c r="C12" s="3" t="inlineStr">
+      <c r="C14" s="3" t="inlineStr">
         <is>
           <t>What's happened to your lead time in the last 12 months?</t>
         </is>
       </c>
-      <c r="D12" s="5" t="inlineStr">
-        <is>
-          <t>yes</t>
-        </is>
-      </c>
-      <c r="E12" s="5" t="inlineStr">
-        <is>
-          <t>no</t>
-        </is>
-      </c>
-      <c r="F12" s="5" t="inlineStr">
-        <is>
-          <t>no</t>
-        </is>
-      </c>
-      <c r="G12" s="5" t="inlineStr"/>
-    </row>
-    <row r="13">
-      <c r="A13" s="5" t="n">
+      <c r="D14" s="3" t="inlineStr">
+        <is>
+          <t>come down | held steady | stretched out | blown out</t>
+        </is>
+      </c>
+      <c r="E14" s="3" t="inlineStr">
+        <is>
+          <t>clause is dropped on: Not sure</t>
+        </is>
+      </c>
+      <c r="F14" s="3" t="inlineStr">
+        <is>
+          <t>constraintDef / fulfilment / evidence [3] / banded</t>
+        </is>
+      </c>
+    </row>
+    <row r="15">
+      <c r="A15" s="6" t="inlineStr">
+        <is>
+          <t>{q19.band}</t>
+        </is>
+      </c>
+      <c r="B15" s="5" t="n">
         <v>19</v>
       </c>
-      <c r="B13" s="6" t="inlineStr">
-        <is>
-          <t>q19</t>
-        </is>
-      </c>
-      <c r="C13" s="3" t="inlineStr">
+      <c r="C15" s="3" t="inlineStr">
         <is>
           <t>How often does delivery slip past what you promised the customer?</t>
         </is>
       </c>
-      <c r="D13" s="5" t="inlineStr">
-        <is>
-          <t>yes</t>
-        </is>
-      </c>
-      <c r="E13" s="5" t="inlineStr">
-        <is>
-          <t>no</t>
-        </is>
-      </c>
-      <c r="F13" s="5" t="inlineStr">
-        <is>
-          <t>no</t>
-        </is>
-      </c>
-      <c r="G13" s="5" t="inlineStr"/>
-    </row>
-    <row r="14">
-      <c r="A14" s="5" t="n">
+      <c r="D15" s="3" t="inlineStr">
+        <is>
+          <t>rarely | occasionally | regularly | on most jobs</t>
+        </is>
+      </c>
+      <c r="E15" s="3" t="inlineStr">
+        <is>
+          <t>clause is dropped on: Not sure</t>
+        </is>
+      </c>
+      <c r="F15" s="3" t="inlineStr">
+        <is>
+          <t>constraintDef / fulfilment / evidence [4] / banded</t>
+        </is>
+      </c>
+    </row>
+    <row r="16">
+      <c r="A16" s="6" t="inlineStr">
+        <is>
+          <t>{q21.band}</t>
+        </is>
+      </c>
+      <c r="B16" s="5" t="n">
         <v>21</v>
       </c>
-      <c r="B14" s="6" t="inlineStr">
-        <is>
-          <t>q21</t>
-        </is>
-      </c>
-      <c r="C14" s="3" t="inlineStr">
-        <is>
-          <t>Of the customers who bought from you a year ago, roughly how many stil</t>
-        </is>
-      </c>
-      <c r="D14" s="5" t="inlineStr">
-        <is>
-          <t>yes</t>
-        </is>
-      </c>
-      <c r="E14" s="5" t="inlineStr">
-        <is>
-          <t>yes</t>
-        </is>
-      </c>
-      <c r="F14" s="5" t="inlineStr">
-        <is>
-          <t>yes</t>
-        </is>
-      </c>
-      <c r="G14" s="5" t="inlineStr">
-        <is>
-          <t>%</t>
-        </is>
-      </c>
-    </row>
-    <row r="15">
-      <c r="A15" s="5" t="n">
+      <c r="C16" s="3" t="inlineStr">
+        <is>
+          <t>Of the customers who bought from you a year ago, roughly how many still buy from you?</t>
+        </is>
+      </c>
+      <c r="D16" s="3" t="inlineStr">
+        <is>
+          <t>above 70% | around half | under a third | close to none | one off by design</t>
+        </is>
+      </c>
+      <c r="E16" s="3" t="inlineStr">
+        <is>
+          <t>clause is dropped on: Not sure</t>
+        </is>
+      </c>
+      <c r="F16" s="3" t="inlineStr">
+        <is>
+          <t>constraintDef / value / evidence [1] / banded</t>
+        </is>
+      </c>
+    </row>
+    <row r="17">
+      <c r="A17" s="6" t="inlineStr">
+        <is>
+          <t>{q21.exact}</t>
+        </is>
+      </c>
+      <c r="B17" s="5" t="n">
+        <v>21</v>
+      </c>
+      <c r="C17" s="3" t="inlineStr">
+        <is>
+          <t>Of the customers who bought from you a year ago, roughly how many still buy from you?</t>
+        </is>
+      </c>
+      <c r="D17" s="3" t="inlineStr">
+        <is>
+          <t>the number they typed, in %</t>
+        </is>
+      </c>
+      <c r="E17" s="3" t="inlineStr">
+        <is>
+          <t>optional, so the precise wording only prints when it was filled in</t>
+        </is>
+      </c>
+      <c r="F17" s="3" t="inlineStr">
+        <is>
+          <t>constraintDef / value / evidence [1] / precise</t>
+        </is>
+      </c>
+    </row>
+    <row r="18">
+      <c r="A18" s="6" t="inlineStr">
+        <is>
+          <t>{q22.band}</t>
+        </is>
+      </c>
+      <c r="B18" s="5" t="n">
         <v>22</v>
       </c>
-      <c r="B15" s="6" t="inlineStr">
-        <is>
-          <t>q22</t>
-        </is>
-      </c>
-      <c r="C15" s="3" t="inlineStr">
-        <is>
-          <t>How often do customers come back and buy again without you chasing the</t>
-        </is>
-      </c>
-      <c r="D15" s="5" t="inlineStr">
-        <is>
-          <t>yes</t>
-        </is>
-      </c>
-      <c r="E15" s="5" t="inlineStr">
-        <is>
-          <t>no</t>
-        </is>
-      </c>
-      <c r="F15" s="5" t="inlineStr">
-        <is>
-          <t>no</t>
-        </is>
-      </c>
-      <c r="G15" s="5" t="inlineStr"/>
-    </row>
-    <row r="16">
-      <c r="A16" s="5" t="n">
+      <c r="C18" s="3" t="inlineStr">
+        <is>
+          <t>How often do customers come back and buy again without you chasing them?</t>
+        </is>
+      </c>
+      <c r="D18" s="3" t="inlineStr">
+        <is>
+          <t>usually | sometimes | rarely | never</t>
+        </is>
+      </c>
+      <c r="E18" s="3" t="inlineStr">
+        <is>
+          <t>clause is dropped on: Not sure</t>
+        </is>
+      </c>
+      <c r="F18" s="3" t="inlineStr">
+        <is>
+          <t>constraintDef / value / evidence [2] / banded</t>
+        </is>
+      </c>
+    </row>
+    <row r="19">
+      <c r="A19" s="6" t="inlineStr">
+        <is>
+          <t>{q23.band}</t>
+        </is>
+      </c>
+      <c r="B19" s="5" t="n">
         <v>23</v>
       </c>
-      <c r="B16" s="6" t="inlineStr">
-        <is>
-          <t>q23</t>
-        </is>
-      </c>
-      <c r="C16" s="3" t="inlineStr">
-        <is>
-          <t>How many of your new customers arrive through a referral from an exist</t>
-        </is>
-      </c>
-      <c r="D16" s="5" t="inlineStr">
-        <is>
-          <t>yes</t>
-        </is>
-      </c>
-      <c r="E16" s="5" t="inlineStr">
-        <is>
-          <t>no</t>
-        </is>
-      </c>
-      <c r="F16" s="5" t="inlineStr">
-        <is>
-          <t>no</t>
-        </is>
-      </c>
-      <c r="G16" s="5" t="inlineStr"/>
-    </row>
-    <row r="17">
-      <c r="A17" s="5" t="n">
+      <c r="C19" s="3" t="inlineStr">
+        <is>
+          <t>How many of your new customers arrive through a referral from an existing one?</t>
+        </is>
+      </c>
+      <c r="D19" s="3" t="inlineStr">
+        <is>
+          <t>most of them | about half | a few | almost none</t>
+        </is>
+      </c>
+      <c r="E19" s="3" t="inlineStr">
+        <is>
+          <t>clause is dropped on: Not sure</t>
+        </is>
+      </c>
+      <c r="F19" s="3" t="inlineStr">
+        <is>
+          <t>constraintDef / value / evidence [3] / banded</t>
+        </is>
+      </c>
+    </row>
+    <row r="20">
+      <c r="A20" s="6" t="inlineStr">
+        <is>
+          <t>{q26.band}</t>
+        </is>
+      </c>
+      <c r="B20" s="5" t="n">
         <v>26</v>
       </c>
-      <c r="B17" s="6" t="inlineStr">
-        <is>
-          <t>q26</t>
-        </is>
-      </c>
-      <c r="C17" s="3" t="inlineStr">
-        <is>
-          <t>Of the people who enquire and get a quote or a proposal, how many go a</t>
-        </is>
-      </c>
-      <c r="D17" s="5" t="inlineStr">
-        <is>
-          <t>yes</t>
-        </is>
-      </c>
-      <c r="E17" s="5" t="inlineStr">
-        <is>
-          <t>yes</t>
-        </is>
-      </c>
-      <c r="F17" s="5" t="inlineStr">
-        <is>
-          <t>yes</t>
-        </is>
-      </c>
-      <c r="G17" s="5" t="inlineStr">
-        <is>
-          <t>%</t>
-        </is>
-      </c>
-    </row>
-    <row r="18">
-      <c r="A18" s="5" t="n">
+      <c r="C20" s="3" t="inlineStr">
+        <is>
+          <t>Of the people who enquire and get a quote or a proposal, how many go ahead?</t>
+        </is>
+      </c>
+      <c r="D20" s="3" t="inlineStr">
+        <is>
+          <t>above 50% | in the 25 to 50% range | in the 10 to 25% range | under 10%</t>
+        </is>
+      </c>
+      <c r="E20" s="3" t="inlineStr">
+        <is>
+          <t>clause is dropped on: Not sure</t>
+        </is>
+      </c>
+      <c r="F20" s="3" t="inlineStr">
+        <is>
+          <t>constraintDef / offer / evidence [1] / banded</t>
+        </is>
+      </c>
+    </row>
+    <row r="21">
+      <c r="A21" s="6" t="inlineStr">
+        <is>
+          <t>{q26.exact}</t>
+        </is>
+      </c>
+      <c r="B21" s="5" t="n">
+        <v>26</v>
+      </c>
+      <c r="C21" s="3" t="inlineStr">
+        <is>
+          <t>Of the people who enquire and get a quote or a proposal, how many go ahead?</t>
+        </is>
+      </c>
+      <c r="D21" s="3" t="inlineStr">
+        <is>
+          <t>the number they typed, in %</t>
+        </is>
+      </c>
+      <c r="E21" s="3" t="inlineStr">
+        <is>
+          <t>optional, so the precise wording only prints when it was filled in</t>
+        </is>
+      </c>
+      <c r="F21" s="3" t="inlineStr">
+        <is>
+          <t>constraintDef / offer / evidence [1] / precise</t>
+        </is>
+      </c>
+    </row>
+    <row r="22">
+      <c r="A22" s="6" t="inlineStr">
+        <is>
+          <t>{q27.band}</t>
+        </is>
+      </c>
+      <c r="B22" s="5" t="n">
         <v>27</v>
       </c>
-      <c r="B18" s="6" t="inlineStr">
-        <is>
-          <t>q27</t>
-        </is>
-      </c>
-      <c r="C18" s="3" t="inlineStr">
+      <c r="C22" s="3" t="inlineStr">
         <is>
           <t>When you lose a deal, what's the most common reason?</t>
         </is>
       </c>
-      <c r="D18" s="5" t="inlineStr">
-        <is>
-          <t>yes</t>
-        </is>
-      </c>
-      <c r="E18" s="5" t="inlineStr">
-        <is>
-          <t>no</t>
-        </is>
-      </c>
-      <c r="F18" s="5" t="inlineStr">
-        <is>
-          <t>no</t>
-        </is>
-      </c>
-      <c r="G18" s="5" t="inlineStr"/>
-    </row>
-    <row r="19">
-      <c r="A19" s="5" t="n">
+      <c r="D22" s="3" t="inlineStr">
+        <is>
+          <t>price | timing | a competitor | inaction | unknown</t>
+        </is>
+      </c>
+      <c r="E22" s="3" t="inlineStr">
+        <is>
+          <t>clause is dropped on: Not sure</t>
+        </is>
+      </c>
+      <c r="F22" s="3" t="inlineStr">
+        <is>
+          <t>constraintDef / offer / evidence [2] / banded</t>
+        </is>
+      </c>
+    </row>
+    <row r="23">
+      <c r="A23" s="6" t="inlineStr">
+        <is>
+          <t>{q28.band}</t>
+        </is>
+      </c>
+      <c r="B23" s="5" t="n">
         <v>28</v>
       </c>
-      <c r="B19" s="6" t="inlineStr">
-        <is>
-          <t>q28</t>
-        </is>
-      </c>
-      <c r="C19" s="3" t="inlineStr">
-        <is>
-          <t xml:space="preserve">How often do you have to explain what you do twice, or get asked what </t>
-        </is>
-      </c>
-      <c r="D19" s="5" t="inlineStr">
-        <is>
-          <t>yes</t>
-        </is>
-      </c>
-      <c r="E19" s="5" t="inlineStr">
-        <is>
-          <t>no</t>
-        </is>
-      </c>
-      <c r="F19" s="5" t="inlineStr">
-        <is>
-          <t>no</t>
-        </is>
-      </c>
-      <c r="G19" s="5" t="inlineStr"/>
-    </row>
-    <row r="20">
-      <c r="A20" s="5" t="n">
+      <c r="C23" s="3" t="inlineStr">
+        <is>
+          <t>How often do you have to explain what you do twice, or get asked what exactly you sell?</t>
+        </is>
+      </c>
+      <c r="D23" s="3" t="inlineStr">
+        <is>
+          <t>rarely | sometimes | often | in most conversations</t>
+        </is>
+      </c>
+      <c r="E23" s="3" t="inlineStr">
+        <is>
+          <t>clause is dropped on: Not sure</t>
+        </is>
+      </c>
+      <c r="F23" s="3" t="inlineStr">
+        <is>
+          <t>constraintDef / offer / evidence [3] / banded</t>
+        </is>
+      </c>
+    </row>
+    <row r="24">
+      <c r="A24" s="6" t="inlineStr">
+        <is>
+          <t>{q31.band}</t>
+        </is>
+      </c>
+      <c r="B24" s="5" t="n">
         <v>31</v>
       </c>
-      <c r="B20" s="6" t="inlineStr">
-        <is>
-          <t>q31</t>
-        </is>
-      </c>
-      <c r="C20" s="3" t="inlineStr">
+      <c r="C24" s="3" t="inlineStr">
         <is>
           <t>How many new enquiries does the business get in a typical month?</t>
         </is>
       </c>
-      <c r="D20" s="5" t="inlineStr">
-        <is>
-          <t>yes</t>
-        </is>
-      </c>
-      <c r="E20" s="5" t="inlineStr">
-        <is>
-          <t>yes</t>
-        </is>
-      </c>
-      <c r="F20" s="5" t="inlineStr">
-        <is>
-          <t>yes</t>
-        </is>
-      </c>
-      <c r="G20" s="5" t="inlineStr">
-        <is>
-          <t>a month</t>
-        </is>
-      </c>
-    </row>
-    <row r="21">
-      <c r="A21" s="5" t="n">
+      <c r="D24" s="3" t="inlineStr">
+        <is>
+          <t>a handful at most | in the 3 to 10 range | in the 11 to 30 range | in the 31 to 100 range | above 100</t>
+        </is>
+      </c>
+      <c r="E24" s="3" t="inlineStr">
+        <is>
+          <t>clause is dropped on: Not sure</t>
+        </is>
+      </c>
+      <c r="F24" s="3" t="inlineStr">
+        <is>
+          <t>constraintDef / demand / evidence [1] / banded</t>
+        </is>
+      </c>
+    </row>
+    <row r="25">
+      <c r="A25" s="6" t="inlineStr">
+        <is>
+          <t>{q31.exact}</t>
+        </is>
+      </c>
+      <c r="B25" s="5" t="n">
+        <v>31</v>
+      </c>
+      <c r="C25" s="3" t="inlineStr">
+        <is>
+          <t>How many new enquiries does the business get in a typical month?</t>
+        </is>
+      </c>
+      <c r="D25" s="3" t="inlineStr">
+        <is>
+          <t>the number they typed, in a month</t>
+        </is>
+      </c>
+      <c r="E25" s="3" t="inlineStr">
+        <is>
+          <t>optional, so the precise wording only prints when it was filled in</t>
+        </is>
+      </c>
+      <c r="F25" s="3" t="inlineStr">
+        <is>
+          <t>constraintDef / demand / evidence [1] / precise</t>
+        </is>
+      </c>
+    </row>
+    <row r="26">
+      <c r="A26" s="6" t="inlineStr">
+        <is>
+          <t>{q33.band}</t>
+        </is>
+      </c>
+      <c r="B26" s="5" t="n">
         <v>33</v>
       </c>
-      <c r="B21" s="6" t="inlineStr">
-        <is>
-          <t>q33</t>
-        </is>
-      </c>
-      <c r="C21" s="3" t="inlineStr">
+      <c r="C26" s="3" t="inlineStr">
         <is>
           <t>Has enquiry volume changed in the last 12 months?</t>
         </is>
       </c>
-      <c r="D21" s="5" t="inlineStr">
-        <is>
-          <t>yes</t>
-        </is>
-      </c>
-      <c r="E21" s="5" t="inlineStr">
-        <is>
-          <t>no</t>
-        </is>
-      </c>
-      <c r="F21" s="5" t="inlineStr">
-        <is>
-          <t>no</t>
-        </is>
-      </c>
-      <c r="G21" s="5" t="inlineStr"/>
-    </row>
-    <row r="22">
-      <c r="A22" s="5" t="n">
+      <c r="D26" s="3" t="inlineStr">
+        <is>
+          <t>grown | stayed flat | fallen | fallen sharply</t>
+        </is>
+      </c>
+      <c r="E26" s="3" t="inlineStr">
+        <is>
+          <t>clause is dropped on: Not sure</t>
+        </is>
+      </c>
+      <c r="F26" s="3" t="inlineStr">
+        <is>
+          <t>constraintDef / demand / evidence [2] / banded</t>
+        </is>
+      </c>
+    </row>
+    <row r="27">
+      <c r="A27" s="6" t="inlineStr">
+        <is>
+          <t>{q35.band}</t>
+        </is>
+      </c>
+      <c r="B27" s="5" t="n">
         <v>35</v>
       </c>
-      <c r="B22" s="6" t="inlineStr">
-        <is>
-          <t>q35</t>
-        </is>
-      </c>
-      <c r="C22" s="3" t="inlineStr">
+      <c r="C27" s="3" t="inlineStr">
         <is>
           <t>Are you doing anything right now to generate new enquiries?</t>
         </is>
       </c>
-      <c r="D22" s="5" t="inlineStr">
-        <is>
-          <t>yes</t>
-        </is>
-      </c>
-      <c r="E22" s="5" t="inlineStr">
-        <is>
-          <t>no</t>
-        </is>
-      </c>
-      <c r="F22" s="5" t="inlineStr">
-        <is>
-          <t>no</t>
-        </is>
-      </c>
-      <c r="G22" s="5" t="inlineStr"/>
-    </row>
-    <row r="23">
-      <c r="A23" s="5" t="n">
+      <c r="D27" s="3" t="inlineStr">
+        <is>
+          <t>consistently | on and off | nothing, it all comes to you</t>
+        </is>
+      </c>
+      <c r="E27" s="3" t="inlineStr">
+        <is>
+          <t>clause is dropped on: Not sure</t>
+        </is>
+      </c>
+      <c r="F27" s="3" t="inlineStr">
+        <is>
+          <t>constraintDef / demand / evidence [3] / banded</t>
+        </is>
+      </c>
+    </row>
+    <row r="28">
+      <c r="A28" s="6" t="inlineStr">
+        <is>
+          <t>{q36.band}</t>
+        </is>
+      </c>
+      <c r="B28" s="5" t="n">
         <v>36</v>
       </c>
-      <c r="B23" s="6" t="inlineStr">
-        <is>
-          <t>q36</t>
-        </is>
-      </c>
-      <c r="C23" s="3" t="inlineStr">
-        <is>
-          <t>On a typical job or sale, what's left after the direct cost of deliver</t>
-        </is>
-      </c>
-      <c r="D23" s="5" t="inlineStr">
-        <is>
-          <t>yes</t>
-        </is>
-      </c>
-      <c r="E23" s="5" t="inlineStr">
-        <is>
-          <t>yes</t>
-        </is>
-      </c>
-      <c r="F23" s="5" t="inlineStr">
-        <is>
-          <t>yes</t>
-        </is>
-      </c>
-      <c r="G23" s="5" t="inlineStr">
-        <is>
-          <t>%</t>
-        </is>
-      </c>
-    </row>
-    <row r="24">
-      <c r="A24" s="5" t="n">
+      <c r="C28" s="3" t="inlineStr">
+        <is>
+          <t>On a typical job or sale, what's left after the direct cost of delivering it?</t>
+        </is>
+      </c>
+      <c r="D28" s="3" t="inlineStr">
+        <is>
+          <t>above 50% | in the 30 to 50% range | in the 15 to 30% range | under 15%</t>
+        </is>
+      </c>
+      <c r="E28" s="3" t="inlineStr">
+        <is>
+          <t>clause is dropped on: Not sure</t>
+        </is>
+      </c>
+      <c r="F28" s="3" t="inlineStr">
+        <is>
+          <t>constraintDef / margin / evidence [1] / banded</t>
+        </is>
+      </c>
+    </row>
+    <row r="29">
+      <c r="A29" s="6" t="inlineStr">
+        <is>
+          <t>{q36.exact}</t>
+        </is>
+      </c>
+      <c r="B29" s="5" t="n">
+        <v>36</v>
+      </c>
+      <c r="C29" s="3" t="inlineStr">
+        <is>
+          <t>On a typical job or sale, what's left after the direct cost of delivering it?</t>
+        </is>
+      </c>
+      <c r="D29" s="3" t="inlineStr">
+        <is>
+          <t>the number they typed, in %</t>
+        </is>
+      </c>
+      <c r="E29" s="3" t="inlineStr">
+        <is>
+          <t>optional, so the precise wording only prints when it was filled in</t>
+        </is>
+      </c>
+      <c r="F29" s="3" t="inlineStr">
+        <is>
+          <t>constraintDef / margin / evidence [1] / precise</t>
+        </is>
+      </c>
+    </row>
+    <row r="30">
+      <c r="A30" s="6" t="inlineStr">
+        <is>
+          <t>{q37.band}</t>
+        </is>
+      </c>
+      <c r="B30" s="5" t="n">
         <v>37</v>
       </c>
-      <c r="B24" s="6" t="inlineStr">
-        <is>
-          <t>q37</t>
-        </is>
-      </c>
-      <c r="C24" s="3" t="inlineStr">
-        <is>
-          <t>After everything, including paying yourself properly, what's left at t</t>
-        </is>
-      </c>
-      <c r="D24" s="5" t="inlineStr">
-        <is>
-          <t>yes</t>
-        </is>
-      </c>
-      <c r="E24" s="5" t="inlineStr">
-        <is>
-          <t>yes</t>
-        </is>
-      </c>
-      <c r="F24" s="5" t="inlineStr">
-        <is>
-          <t>yes</t>
-        </is>
-      </c>
-      <c r="G24" s="5" t="inlineStr">
-        <is>
-          <t>%</t>
-        </is>
-      </c>
-    </row>
-    <row r="25">
-      <c r="A25" s="5" t="n">
+      <c r="C30" s="3" t="inlineStr">
+        <is>
+          <t>After everything, including paying yourself properly, what's left at the end of a year?</t>
+        </is>
+      </c>
+      <c r="D30" s="3" t="inlineStr">
+        <is>
+          <t>above 20% | in the 10 to 20% range | in the 1 to 10% range | nothing, or a loss</t>
+        </is>
+      </c>
+      <c r="E30" s="3" t="inlineStr">
+        <is>
+          <t>clause is dropped on: Not sure</t>
+        </is>
+      </c>
+      <c r="F30" s="3" t="inlineStr">
+        <is>
+          <t>constraintDef / margin / evidence [2] / banded</t>
+        </is>
+      </c>
+    </row>
+    <row r="31">
+      <c r="A31" s="6" t="inlineStr">
+        <is>
+          <t>{q37.exact}</t>
+        </is>
+      </c>
+      <c r="B31" s="5" t="n">
+        <v>37</v>
+      </c>
+      <c r="C31" s="3" t="inlineStr">
+        <is>
+          <t>After everything, including paying yourself properly, what's left at the end of a year?</t>
+        </is>
+      </c>
+      <c r="D31" s="3" t="inlineStr">
+        <is>
+          <t>the number they typed, in %</t>
+        </is>
+      </c>
+      <c r="E31" s="3" t="inlineStr">
+        <is>
+          <t>optional, so the precise wording only prints when it was filled in</t>
+        </is>
+      </c>
+      <c r="F31" s="3" t="inlineStr">
+        <is>
+          <t>constraintDef / margin / evidence [2] / precise</t>
+        </is>
+      </c>
+    </row>
+    <row r="32">
+      <c r="A32" s="6" t="inlineStr">
+        <is>
+          <t>{q38.band}</t>
+        </is>
+      </c>
+      <c r="B32" s="5" t="n">
         <v>38</v>
       </c>
-      <c r="B25" s="6" t="inlineStr">
-        <is>
-          <t>q38</t>
-        </is>
-      </c>
-      <c r="C25" s="3" t="inlineStr">
+      <c r="C32" s="3" t="inlineStr">
         <is>
           <t>When did you last raise your prices?</t>
         </is>
       </c>
-      <c r="D25" s="5" t="inlineStr">
-        <is>
-          <t>yes</t>
-        </is>
-      </c>
-      <c r="E25" s="5" t="inlineStr">
-        <is>
-          <t>no</t>
-        </is>
-      </c>
-      <c r="F25" s="5" t="inlineStr">
-        <is>
-          <t>no</t>
-        </is>
-      </c>
-      <c r="G25" s="5" t="inlineStr"/>
-    </row>
-    <row r="26">
-      <c r="A26" s="5" t="n">
+      <c r="D32" s="3" t="inlineStr">
+        <is>
+          <t>inside the last six months | in the last year | one to two years ago | more than two years ago | never</t>
+        </is>
+      </c>
+      <c r="E32" s="3" t="inlineStr">
+        <is>
+          <t>clause is dropped on: Not sure</t>
+        </is>
+      </c>
+      <c r="F32" s="3" t="inlineStr">
+        <is>
+          <t>constraintDef / margin / evidence [3] / banded</t>
+        </is>
+      </c>
+    </row>
+    <row r="33">
+      <c r="A33" s="6" t="inlineStr">
+        <is>
+          <t>{q39.band}</t>
+        </is>
+      </c>
+      <c r="B33" s="5" t="n">
         <v>39</v>
       </c>
-      <c r="B26" s="6" t="inlineStr">
-        <is>
-          <t>q39</t>
-        </is>
-      </c>
-      <c r="C26" s="3" t="inlineStr">
+      <c r="C33" s="3" t="inlineStr">
         <is>
           <t>How often does a job end up costing more to deliver than you quoted?</t>
         </is>
       </c>
-      <c r="D26" s="5" t="inlineStr">
-        <is>
-          <t>yes</t>
-        </is>
-      </c>
-      <c r="E26" s="5" t="inlineStr">
-        <is>
-          <t>no</t>
-        </is>
-      </c>
-      <c r="F26" s="5" t="inlineStr">
-        <is>
-          <t>no</t>
-        </is>
-      </c>
-      <c r="G26" s="5" t="inlineStr"/>
-    </row>
-    <row r="27">
-      <c r="A27" s="5" t="n">
+      <c r="D33" s="3" t="inlineStr">
+        <is>
+          <t>rarely | sometimes | often | on most jobs</t>
+        </is>
+      </c>
+      <c r="E33" s="3" t="inlineStr">
+        <is>
+          <t>clause is dropped on: Not sure</t>
+        </is>
+      </c>
+      <c r="F33" s="3" t="inlineStr">
+        <is>
+          <t>constraintDef / margin / evidence [4] / banded</t>
+        </is>
+      </c>
+    </row>
+    <row r="34">
+      <c r="A34" s="6" t="inlineStr">
+        <is>
+          <t>{q41.band}</t>
+        </is>
+      </c>
+      <c r="B34" s="5" t="n">
         <v>41</v>
       </c>
-      <c r="B27" s="6" t="inlineStr">
-        <is>
-          <t>q41</t>
-        </is>
-      </c>
-      <c r="C27" s="3" t="inlineStr">
+      <c r="C34" s="3" t="inlineStr">
         <is>
           <t>What share of your revenue comes from your single biggest customer?</t>
         </is>
       </c>
-      <c r="D27" s="5" t="inlineStr">
-        <is>
-          <t>yes</t>
-        </is>
-      </c>
-      <c r="E27" s="5" t="inlineStr">
-        <is>
-          <t>yes</t>
-        </is>
-      </c>
-      <c r="F27" s="5" t="inlineStr">
-        <is>
-          <t>yes</t>
-        </is>
-      </c>
-      <c r="G27" s="5" t="inlineStr">
-        <is>
-          <t>%</t>
-        </is>
-      </c>
-    </row>
-    <row r="28">
-      <c r="A28" s="5" t="n">
+      <c r="D34" s="3" t="inlineStr">
+        <is>
+          <t>under 10% | between 10 and 20% | between 20 and 30% | between 30 and 50% | more than half</t>
+        </is>
+      </c>
+      <c r="E34" s="3" t="inlineStr">
+        <is>
+          <t>clause is dropped on: Not sure</t>
+        </is>
+      </c>
+      <c r="F34" s="3" t="inlineStr">
+        <is>
+          <t>compound [15] / text  compound [17] / text  compound [4] / text  compound [5] / text  riskDef / key_client / banded</t>
+        </is>
+      </c>
+    </row>
+    <row r="35">
+      <c r="A35" s="6" t="inlineStr">
+        <is>
+          <t>{q41.exact}</t>
+        </is>
+      </c>
+      <c r="B35" s="5" t="n">
+        <v>41</v>
+      </c>
+      <c r="C35" s="3" t="inlineStr">
+        <is>
+          <t>What share of your revenue comes from your single biggest customer?</t>
+        </is>
+      </c>
+      <c r="D35" s="3" t="inlineStr">
+        <is>
+          <t>the number they typed, in %</t>
+        </is>
+      </c>
+      <c r="E35" s="3" t="inlineStr">
+        <is>
+          <t>optional, so the precise wording only prints when it was filled in</t>
+        </is>
+      </c>
+      <c r="F35" s="3" t="inlineStr">
+        <is>
+          <t>riskDef / key_client / precise</t>
+        </is>
+      </c>
+    </row>
+    <row r="36">
+      <c r="A36" s="6" t="inlineStr">
+        <is>
+          <t>{q42.band}</t>
+        </is>
+      </c>
+      <c r="B36" s="5" t="n">
         <v>42</v>
       </c>
-      <c r="B28" s="6" t="inlineStr">
-        <is>
-          <t>q42</t>
-        </is>
-      </c>
-      <c r="C28" s="3" t="inlineStr">
-        <is>
-          <t>What share of revenue comes from your single biggest product or servic</t>
-        </is>
-      </c>
-      <c r="D28" s="5" t="inlineStr">
-        <is>
-          <t>yes</t>
-        </is>
-      </c>
-      <c r="E28" s="5" t="inlineStr">
-        <is>
-          <t>yes</t>
-        </is>
-      </c>
-      <c r="F28" s="5" t="inlineStr">
-        <is>
-          <t>yes</t>
-        </is>
-      </c>
-      <c r="G28" s="5" t="inlineStr">
-        <is>
-          <t>%</t>
-        </is>
-      </c>
-    </row>
-    <row r="29">
-      <c r="A29" s="5" t="n">
+      <c r="C36" s="3" t="inlineStr">
+        <is>
+          <t>What share of revenue comes from your single biggest product or service line?</t>
+        </is>
+      </c>
+      <c r="D36" s="3" t="inlineStr">
+        <is>
+          <t>under a quarter | a quarter to a half | half to three quarters | more than three quarters</t>
+        </is>
+      </c>
+      <c r="E36" s="3" t="inlineStr">
+        <is>
+          <t>clause is dropped on: Not sure</t>
+        </is>
+      </c>
+      <c r="F36" s="3" t="inlineStr">
+        <is>
+          <t>riskDef / key_product / banded</t>
+        </is>
+      </c>
+    </row>
+    <row r="37">
+      <c r="A37" s="6" t="inlineStr">
+        <is>
+          <t>{q42.exact}</t>
+        </is>
+      </c>
+      <c r="B37" s="5" t="n">
+        <v>42</v>
+      </c>
+      <c r="C37" s="3" t="inlineStr">
+        <is>
+          <t>What share of revenue comes from your single biggest product or service line?</t>
+        </is>
+      </c>
+      <c r="D37" s="3" t="inlineStr">
+        <is>
+          <t>the number they typed, in %</t>
+        </is>
+      </c>
+      <c r="E37" s="3" t="inlineStr">
+        <is>
+          <t>optional, so the precise wording only prints when it was filled in</t>
+        </is>
+      </c>
+      <c r="F37" s="3" t="inlineStr">
+        <is>
+          <t>riskDef / key_product / precise</t>
+        </is>
+      </c>
+    </row>
+    <row r="38">
+      <c r="A38" s="6" t="inlineStr">
+        <is>
+          <t>{q43.band}</t>
+        </is>
+      </c>
+      <c r="B38" s="5" t="n">
         <v>43</v>
       </c>
-      <c r="B29" s="6" t="inlineStr">
-        <is>
-          <t>q43</t>
-        </is>
-      </c>
-      <c r="C29" s="3" t="inlineStr">
+      <c r="C38" s="3" t="inlineStr">
         <is>
           <t>How spread out are the places your new customers come from?</t>
         </is>
       </c>
-      <c r="D29" s="5" t="inlineStr">
-        <is>
-          <t>yes</t>
-        </is>
-      </c>
-      <c r="E29" s="5" t="inlineStr">
-        <is>
-          <t>no</t>
-        </is>
-      </c>
-      <c r="F29" s="5" t="inlineStr">
-        <is>
-          <t>no</t>
-        </is>
-      </c>
-      <c r="G29" s="5" t="inlineStr"/>
-    </row>
-    <row r="30">
-      <c r="A30" s="5" t="n">
+      <c r="D38" s="3" t="inlineStr">
+        <is>
+          <t>spread across several channels | carried by two channels | almost entirely one channel</t>
+        </is>
+      </c>
+      <c r="E38" s="3" t="inlineStr">
+        <is>
+          <t>clause is dropped on: Not sure</t>
+        </is>
+      </c>
+      <c r="F38" s="3" t="inlineStr">
+        <is>
+          <t>riskDef / key_channel / banded</t>
+        </is>
+      </c>
+    </row>
+    <row r="39">
+      <c r="A39" s="6" t="inlineStr">
+        <is>
+          <t>{q45.band}</t>
+        </is>
+      </c>
+      <c r="B39" s="5" t="n">
         <v>45</v>
       </c>
-      <c r="B30" s="6" t="inlineStr">
-        <is>
-          <t>q45</t>
-        </is>
-      </c>
-      <c r="C30" s="3" t="inlineStr">
+      <c r="C39" s="3" t="inlineStr">
         <is>
           <t>How is your work actually committed by the customer?</t>
         </is>
       </c>
-      <c r="D30" s="5" t="inlineStr">
-        <is>
-          <t>yes</t>
-        </is>
-      </c>
-      <c r="E30" s="5" t="inlineStr">
-        <is>
-          <t>no</t>
-        </is>
-      </c>
-      <c r="F30" s="5" t="inlineStr">
-        <is>
-          <t>no</t>
-        </is>
-      </c>
-      <c r="G30" s="5" t="inlineStr"/>
-    </row>
-    <row r="31">
-      <c r="A31" s="5" t="n">
+      <c r="D39" s="3" t="inlineStr">
+        <is>
+          <t>term contracts | job by job agreements | month to month | a handshake and an email</t>
+        </is>
+      </c>
+      <c r="E39" s="3" t="inlineStr">
+        <is>
+          <t>clause is dropped on: Not sure</t>
+        </is>
+      </c>
+      <c r="F39" s="3" t="inlineStr">
+        <is>
+          <t>riskDef / no_contracts / banded</t>
+        </is>
+      </c>
+    </row>
+    <row r="40">
+      <c r="A40" s="6" t="inlineStr">
+        <is>
+          <t>{q46.band}</t>
+        </is>
+      </c>
+      <c r="B40" s="5" t="n">
         <v>46</v>
       </c>
-      <c r="B31" s="6" t="inlineStr">
-        <is>
-          <t>q46</t>
-        </is>
-      </c>
-      <c r="C31" s="3" t="inlineStr">
-        <is>
-          <t>How much of how the work gets done is written down well enough for som</t>
-        </is>
-      </c>
-      <c r="D31" s="5" t="inlineStr">
-        <is>
-          <t>yes</t>
-        </is>
-      </c>
-      <c r="E31" s="5" t="inlineStr">
-        <is>
-          <t>no</t>
-        </is>
-      </c>
-      <c r="F31" s="5" t="inlineStr">
-        <is>
-          <t>no</t>
-        </is>
-      </c>
-      <c r="G31" s="5" t="inlineStr"/>
-    </row>
-    <row r="32">
-      <c r="A32" s="5" t="n">
+      <c r="C40" s="3" t="inlineStr">
+        <is>
+          <t>How much of how the work gets done is written down well enough for someone new to follow?</t>
+        </is>
+      </c>
+      <c r="D40" s="3" t="inlineStr">
+        <is>
+          <t>Most | Some | Almost none</t>
+        </is>
+      </c>
+      <c r="E40" s="3" t="inlineStr">
+        <is>
+          <t>clause is dropped on: Not sure</t>
+        </is>
+      </c>
+      <c r="F40" s="3" t="inlineStr">
+        <is>
+          <t>riskDef / no_process / banded</t>
+        </is>
+      </c>
+    </row>
+    <row r="41">
+      <c r="A41" s="6" t="inlineStr">
+        <is>
+          <t>{q47.band}</t>
+        </is>
+      </c>
+      <c r="B41" s="5" t="n">
         <v>47</v>
       </c>
-      <c r="B32" s="6" t="inlineStr">
-        <is>
-          <t>q47</t>
-        </is>
-      </c>
-      <c r="C32" s="3" t="inlineStr">
-        <is>
-          <t>How often do you look at numbers that tell you how the business is tra</t>
-        </is>
-      </c>
-      <c r="D32" s="5" t="inlineStr">
-        <is>
-          <t>yes</t>
-        </is>
-      </c>
-      <c r="E32" s="5" t="inlineStr">
-        <is>
-          <t>no</t>
-        </is>
-      </c>
-      <c r="F32" s="5" t="inlineStr">
-        <is>
-          <t>no</t>
-        </is>
-      </c>
-      <c r="G32" s="5" t="inlineStr"/>
-    </row>
-    <row r="33">
-      <c r="A33" s="5" t="n">
+      <c r="C41" s="3" t="inlineStr">
+        <is>
+          <t>How often do you look at numbers that tell you how the business is travelling?</t>
+        </is>
+      </c>
+      <c r="D41" s="3" t="inlineStr">
+        <is>
+          <t>weekly | monthly | once a year at tax time | next to never</t>
+        </is>
+      </c>
+      <c r="E41" s="3" t="inlineStr">
+        <is>
+          <t>clause is dropped on: Not sure</t>
+        </is>
+      </c>
+      <c r="F41" s="3" t="inlineStr">
+        <is>
+          <t>riskDef / no_data / banded</t>
+        </is>
+      </c>
+    </row>
+    <row r="42">
+      <c r="A42" s="6" t="inlineStr">
+        <is>
+          <t>{q49.band}</t>
+        </is>
+      </c>
+      <c r="B42" s="5" t="n">
         <v>49</v>
       </c>
-      <c r="B33" s="6" t="inlineStr">
-        <is>
-          <t>q49</t>
-        </is>
-      </c>
-      <c r="C33" s="3" t="inlineStr">
-        <is>
-          <t>If you sold the business tomorrow, how much of what the buyer is payin</t>
-        </is>
-      </c>
-      <c r="D33" s="5" t="inlineStr">
-        <is>
-          <t>yes</t>
-        </is>
-      </c>
-      <c r="E33" s="5" t="inlineStr">
-        <is>
-          <t>no</t>
-        </is>
-      </c>
-      <c r="F33" s="5" t="inlineStr">
-        <is>
-          <t>no</t>
-        </is>
-      </c>
-      <c r="G33" s="5" t="inlineStr"/>
-    </row>
-    <row r="34">
-      <c r="A34" s="5" t="n">
+      <c r="C42" s="3" t="inlineStr">
+        <is>
+          <t>If you sold the business tomorrow, how much of what the buyer is paying for is you personally?</t>
+        </is>
+      </c>
+      <c r="D42" s="3" t="inlineStr">
+        <is>
+          <t>almost none | some | most | all</t>
+        </is>
+      </c>
+      <c r="E42" s="3" t="inlineStr">
+        <is>
+          <t>clause is dropped on: Not sure</t>
+        </is>
+      </c>
+      <c r="F42" s="3" t="inlineStr">
+        <is>
+          <t>riskDef / owner_trapped / banded</t>
+        </is>
+      </c>
+    </row>
+    <row r="43">
+      <c r="A43" s="6" t="inlineStr">
+        <is>
+          <t>{q50.band}</t>
+        </is>
+      </c>
+      <c r="B43" s="5" t="n">
         <v>50</v>
       </c>
-      <c r="B34" s="6" t="inlineStr">
-        <is>
-          <t>q50</t>
-        </is>
-      </c>
-      <c r="C34" s="3" t="inlineStr">
-        <is>
-          <t xml:space="preserve">Is there a plan for what happens to the business if you stop, sell or </t>
-        </is>
-      </c>
-      <c r="D34" s="5" t="inlineStr">
-        <is>
-          <t>yes</t>
-        </is>
-      </c>
-      <c r="E34" s="5" t="inlineStr">
-        <is>
-          <t>no</t>
-        </is>
-      </c>
-      <c r="F34" s="5" t="inlineStr">
-        <is>
-          <t>no</t>
-        </is>
-      </c>
-      <c r="G34" s="5" t="inlineStr"/>
-    </row>
-    <row r="35">
-      <c r="A35" s="5" t="n">
+      <c r="C43" s="3" t="inlineStr">
+        <is>
+          <t>Is there a plan for what happens to the business if you stop, sell or step back?</t>
+        </is>
+      </c>
+      <c r="D43" s="3" t="inlineStr">
+        <is>
+          <t>a written plan | a rough idea | nothing</t>
+        </is>
+      </c>
+      <c r="E43" s="3" t="inlineStr">
+        <is>
+          <t>clause is dropped on: Not sure</t>
+        </is>
+      </c>
+      <c r="F43" s="3" t="inlineStr">
+        <is>
+          <t>riskDef / no_succession / banded</t>
+        </is>
+      </c>
+    </row>
+    <row r="44">
+      <c r="A44" s="6" t="inlineStr">
+        <is>
+          <t>{q51.band}</t>
+        </is>
+      </c>
+      <c r="B44" s="5" t="n">
         <v>51</v>
       </c>
-      <c r="B35" s="6" t="inlineStr">
-        <is>
-          <t>q51</t>
-        </is>
-      </c>
-      <c r="C35" s="3" t="inlineStr">
-        <is>
-          <t>Have you personally guaranteed any of the business's debt, leases or f</t>
-        </is>
-      </c>
-      <c r="D35" s="5" t="inlineStr">
-        <is>
-          <t>yes</t>
-        </is>
-      </c>
-      <c r="E35" s="5" t="inlineStr">
-        <is>
-          <t>no</t>
-        </is>
-      </c>
-      <c r="F35" s="5" t="inlineStr">
-        <is>
-          <t>no</t>
-        </is>
-      </c>
-      <c r="G35" s="5" t="inlineStr"/>
-    </row>
-    <row r="36">
-      <c r="A36" s="5" t="n">
+      <c r="C44" s="3" t="inlineStr">
+        <is>
+          <t>Have you personally guaranteed any of the business's debt, leases or facilities?</t>
+        </is>
+      </c>
+      <c r="D44" s="3" t="inlineStr">
+        <is>
+          <t>none | a small amount | a significant amount</t>
+        </is>
+      </c>
+      <c r="E44" s="3" t="inlineStr">
+        <is>
+          <t>clause is dropped on: Not sure</t>
+        </is>
+      </c>
+      <c r="F44" s="3" t="inlineStr">
+        <is>
+          <t>riskDef / personal_guarantee / banded</t>
+        </is>
+      </c>
+    </row>
+    <row r="45">
+      <c r="A45" s="6" t="inlineStr">
+        <is>
+          <t>{q52.band}</t>
+        </is>
+      </c>
+      <c r="B45" s="5" t="n">
         <v>52</v>
       </c>
-      <c r="B36" s="6" t="inlineStr">
-        <is>
-          <t>q52</t>
-        </is>
-      </c>
-      <c r="C36" s="3" t="inlineStr">
-        <is>
-          <t>How well does the way you spend your week match what you wanted out of</t>
-        </is>
-      </c>
-      <c r="D36" s="5" t="inlineStr">
-        <is>
-          <t>yes</t>
-        </is>
-      </c>
-      <c r="E36" s="5" t="inlineStr">
-        <is>
-          <t>no</t>
-        </is>
-      </c>
-      <c r="F36" s="5" t="inlineStr">
-        <is>
-          <t>no</t>
-        </is>
-      </c>
-      <c r="G36" s="5" t="inlineStr"/>
+      <c r="C45" s="3" t="inlineStr">
+        <is>
+          <t>How well does the way you spend your week match what you wanted out of this business?</t>
+        </is>
+      </c>
+      <c r="D45" s="3" t="inlineStr">
+        <is>
+          <t>close to what you signed up for | only partly a match for what you wanted | the opposite of what you wanted</t>
+        </is>
+      </c>
+      <c r="E45" s="3" t="inlineStr">
+        <is>
+          <t>clause is dropped on: Not sure</t>
+        </is>
+      </c>
+      <c r="F45" s="3" t="inlineStr">
+        <is>
+          <t>riskDef / model_misfit / banded</t>
+        </is>
+      </c>
+    </row>
+    <row r="46">
+      <c r="A46" s="6" t="inlineStr">
+        <is>
+          <t>{d.primaryShort}</t>
+        </is>
+      </c>
+      <c r="B46" s="5" t="inlineStr"/>
+      <c r="C46" s="3" t="inlineStr">
+        <is>
+          <t>derived, not a question</t>
+        </is>
+      </c>
+      <c r="D46" s="3" t="inlineStr">
+        <is>
+          <t>the primary constraint's short name, lower case</t>
+        </is>
+      </c>
+      <c r="E46" s="3" t="inlineStr">
+        <is>
+          <t>always resolves</t>
+        </is>
+      </c>
+      <c r="F46" s="3" t="inlineStr">
+        <is>
+          <t>looseBody  minorConstraint / cashflow  minorConstraint / demand  minorConstraint / fulfilment  minorConstraint / margin  minorConstraint / offer  minorConstraint / talent  minorConstraint / value  unsureBody</t>
+        </is>
+      </c>
+    </row>
+    <row r="47">
+      <c r="A47" s="6" t="inlineStr">
+        <is>
+          <t>{d.unownedLayers}</t>
+        </is>
+      </c>
+      <c r="B47" s="5" t="inlineStr"/>
+      <c r="C47" s="3" t="inlineStr">
+        <is>
+          <t>derived, not a question</t>
+        </is>
+      </c>
+      <c r="D47" s="3" t="inlineStr">
+        <is>
+          <t>a sentence naming which layers sit with the owner</t>
+        </is>
+      </c>
+      <c r="E47" s="3" t="inlineStr">
+        <is>
+          <t>always resolves</t>
+        </is>
+      </c>
+      <c r="F47" s="3" t="inlineStr">
+        <is>
+          <t>constraintDef / talent / open</t>
+        </is>
+      </c>
     </row>
   </sheetData>
-  <autoFilter ref="A2:G36"/>
+  <autoFilter ref="A2:F47"/>
   <mergeCells count="1">
-    <mergeCell ref="A1:G1"/>
+    <mergeCell ref="A1:F1"/>
   </mergeCells>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
@@ -14669,13 +14958,14 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:D96"/>
+  <dimension ref="A1:E96"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="13" customWidth="1" min="1" max="1"/>
     <col width="22" customWidth="1" min="2" max="2"/>
-    <col width="92" customWidth="1" min="3" max="3"/>
-    <col width="78" customWidth="1" min="4" max="4"/>
+    <col width="82" customWidth="1" min="3" max="3"/>
+    <col width="68" customWidth="1" min="4" max="4"/>
+    <col width="26" customWidth="1" min="5" max="5"/>
   </cols>
   <sheetData>
     <row r="1" ht="30" customHeight="1">
@@ -14706,6 +14996,11 @@
           <t>Precise version, used only when they typed the figure</t>
         </is>
       </c>
+      <c r="E2" s="1" t="inlineStr">
+        <is>
+          <t>Variables in this row</t>
+        </is>
+      </c>
     </row>
     <row r="3">
       <c r="A3" s="6" t="inlineStr">
@@ -14724,6 +15019,7 @@
         </is>
       </c>
       <c r="D3" s="7" t="inlineStr"/>
+      <c r="E3" s="9" t="inlineStr"/>
     </row>
     <row r="4">
       <c r="A4" s="6" t="inlineStr">
@@ -14742,6 +15038,7 @@
         </is>
       </c>
       <c r="D4" s="7" t="inlineStr"/>
+      <c r="E4" s="9" t="inlineStr"/>
     </row>
     <row r="5">
       <c r="A5" s="6" t="inlineStr">
@@ -14760,6 +15057,7 @@
         </is>
       </c>
       <c r="D5" s="7" t="inlineStr"/>
+      <c r="E5" s="9" t="inlineStr"/>
     </row>
     <row r="6">
       <c r="A6" s="6" t="inlineStr">
@@ -14782,6 +15080,11 @@
           <t>money takes {q7.exact} days to arrive after the work is done</t>
         </is>
       </c>
+      <c r="E6" s="9" t="inlineStr">
+        <is>
+          <t>{q7.band}, {q7.exact}</t>
+        </is>
+      </c>
     </row>
     <row r="7">
       <c r="A7" s="6" t="inlineStr">
@@ -14800,6 +15103,11 @@
         </is>
       </c>
       <c r="D7" s="7" t="inlineStr"/>
+      <c r="E7" s="9" t="inlineStr">
+        <is>
+          <t>{q6.band}</t>
+        </is>
+      </c>
     </row>
     <row r="8">
       <c r="A8" s="6" t="inlineStr">
@@ -14818,6 +15126,11 @@
         </is>
       </c>
       <c r="D8" s="7" t="inlineStr"/>
+      <c r="E8" s="9" t="inlineStr">
+        <is>
+          <t>{q8.band}</t>
+        </is>
+      </c>
     </row>
     <row r="9">
       <c r="A9" s="6" t="inlineStr">
@@ -14836,6 +15149,11 @@
         </is>
       </c>
       <c r="D9" s="7" t="inlineStr"/>
+      <c r="E9" s="9" t="inlineStr">
+        <is>
+          <t>{q9.band}</t>
+        </is>
+      </c>
     </row>
     <row r="10">
       <c r="A10" s="6" t="inlineStr">
@@ -14854,6 +15172,7 @@
         </is>
       </c>
       <c r="D10" s="7" t="inlineStr"/>
+      <c r="E10" s="9" t="inlineStr"/>
     </row>
     <row r="11">
       <c r="A11" s="6" t="inlineStr">
@@ -14872,6 +15191,7 @@
         </is>
       </c>
       <c r="D11" s="7" t="inlineStr"/>
+      <c r="E11" s="9" t="inlineStr"/>
     </row>
     <row r="12">
       <c r="A12" s="6" t="inlineStr">
@@ -14890,6 +15210,7 @@
         </is>
       </c>
       <c r="D12" s="7" t="inlineStr"/>
+      <c r="E12" s="9" t="inlineStr"/>
     </row>
     <row r="13">
       <c r="A13" s="6" t="inlineStr">
@@ -14908,6 +15229,7 @@
         </is>
       </c>
       <c r="D13" s="7" t="inlineStr"/>
+      <c r="E13" s="9" t="inlineStr"/>
     </row>
     <row r="14">
       <c r="A14" s="6" t="inlineStr">
@@ -14926,6 +15248,7 @@
         </is>
       </c>
       <c r="D14" s="7" t="inlineStr"/>
+      <c r="E14" s="9" t="inlineStr"/>
     </row>
     <row r="15">
       <c r="A15" s="6" t="inlineStr">
@@ -14944,6 +15267,7 @@
         </is>
       </c>
       <c r="D15" s="7" t="inlineStr"/>
+      <c r="E15" s="9" t="inlineStr"/>
     </row>
     <row r="16">
       <c r="A16" s="6" t="inlineStr">
@@ -14962,6 +15286,7 @@
         </is>
       </c>
       <c r="D16" s="7" t="inlineStr"/>
+      <c r="E16" s="9" t="inlineStr"/>
     </row>
     <row r="17">
       <c r="A17" s="6" t="inlineStr">
@@ -14980,6 +15305,7 @@
         </is>
       </c>
       <c r="D17" s="7" t="inlineStr"/>
+      <c r="E17" s="9" t="inlineStr"/>
     </row>
     <row r="18">
       <c r="A18" s="6" t="inlineStr">
@@ -14998,6 +15324,7 @@
         </is>
       </c>
       <c r="D18" s="7" t="inlineStr"/>
+      <c r="E18" s="9" t="inlineStr"/>
     </row>
     <row r="19">
       <c r="A19" s="6" t="inlineStr">
@@ -15016,6 +15343,11 @@
         </is>
       </c>
       <c r="D19" s="7" t="inlineStr"/>
+      <c r="E19" s="9" t="inlineStr">
+        <is>
+          <t>{d.unownedLayers}</t>
+        </is>
+      </c>
     </row>
     <row r="20">
       <c r="A20" s="6" t="inlineStr">
@@ -15034,6 +15366,11 @@
         </is>
       </c>
       <c r="D20" s="7" t="inlineStr"/>
+      <c r="E20" s="9" t="inlineStr">
+        <is>
+          <t>{q13.band}</t>
+        </is>
+      </c>
     </row>
     <row r="21">
       <c r="A21" s="6" t="inlineStr">
@@ -15052,6 +15389,11 @@
         </is>
       </c>
       <c r="D21" s="7" t="inlineStr"/>
+      <c r="E21" s="9" t="inlineStr">
+        <is>
+          <t>{q12.band}</t>
+        </is>
+      </c>
     </row>
     <row r="22">
       <c r="A22" s="6" t="inlineStr">
@@ -15070,6 +15412,11 @@
         </is>
       </c>
       <c r="D22" s="7" t="inlineStr"/>
+      <c r="E22" s="9" t="inlineStr">
+        <is>
+          <t>{q14.band}</t>
+        </is>
+      </c>
     </row>
     <row r="23">
       <c r="A23" s="6" t="inlineStr">
@@ -15088,6 +15435,7 @@
         </is>
       </c>
       <c r="D23" s="7" t="inlineStr"/>
+      <c r="E23" s="9" t="inlineStr"/>
     </row>
     <row r="24">
       <c r="A24" s="6" t="inlineStr">
@@ -15106,6 +15454,7 @@
         </is>
       </c>
       <c r="D24" s="7" t="inlineStr"/>
+      <c r="E24" s="9" t="inlineStr"/>
     </row>
     <row r="25">
       <c r="A25" s="6" t="inlineStr">
@@ -15124,6 +15473,7 @@
         </is>
       </c>
       <c r="D25" s="7" t="inlineStr"/>
+      <c r="E25" s="9" t="inlineStr"/>
     </row>
     <row r="26">
       <c r="A26" s="6" t="inlineStr">
@@ -15142,6 +15492,7 @@
         </is>
       </c>
       <c r="D26" s="7" t="inlineStr"/>
+      <c r="E26" s="9" t="inlineStr"/>
     </row>
     <row r="27">
       <c r="A27" s="6" t="inlineStr">
@@ -15160,6 +15511,7 @@
         </is>
       </c>
       <c r="D27" s="7" t="inlineStr"/>
+      <c r="E27" s="9" t="inlineStr"/>
     </row>
     <row r="28">
       <c r="A28" s="6" t="inlineStr">
@@ -15178,6 +15530,7 @@
         </is>
       </c>
       <c r="D28" s="7" t="inlineStr"/>
+      <c r="E28" s="9" t="inlineStr"/>
     </row>
     <row r="29">
       <c r="A29" s="6" t="inlineStr">
@@ -15196,6 +15549,7 @@
         </is>
       </c>
       <c r="D29" s="7" t="inlineStr"/>
+      <c r="E29" s="9" t="inlineStr"/>
     </row>
     <row r="30">
       <c r="A30" s="6" t="inlineStr">
@@ -15214,6 +15568,7 @@
         </is>
       </c>
       <c r="D30" s="7" t="inlineStr"/>
+      <c r="E30" s="9" t="inlineStr"/>
     </row>
     <row r="31">
       <c r="A31" s="6" t="inlineStr">
@@ -15232,6 +15587,7 @@
         </is>
       </c>
       <c r="D31" s="7" t="inlineStr"/>
+      <c r="E31" s="9" t="inlineStr"/>
     </row>
     <row r="32">
       <c r="A32" s="6" t="inlineStr">
@@ -15250,6 +15606,7 @@
         </is>
       </c>
       <c r="D32" s="7" t="inlineStr"/>
+      <c r="E32" s="9" t="inlineStr"/>
     </row>
     <row r="33">
       <c r="A33" s="6" t="inlineStr">
@@ -15272,6 +15629,11 @@
           <t>you're running at {q16.exact}% booked</t>
         </is>
       </c>
+      <c r="E33" s="9" t="inlineStr">
+        <is>
+          <t>{q16.band}, {q16.exact}</t>
+        </is>
+      </c>
     </row>
     <row r="34">
       <c r="A34" s="6" t="inlineStr">
@@ -15290,6 +15652,11 @@
         </is>
       </c>
       <c r="D34" s="7" t="inlineStr"/>
+      <c r="E34" s="9" t="inlineStr">
+        <is>
+          <t>{q17.band}</t>
+        </is>
+      </c>
     </row>
     <row r="35">
       <c r="A35" s="6" t="inlineStr">
@@ -15308,6 +15675,11 @@
         </is>
       </c>
       <c r="D35" s="7" t="inlineStr"/>
+      <c r="E35" s="9" t="inlineStr">
+        <is>
+          <t>{q18.band}</t>
+        </is>
+      </c>
     </row>
     <row r="36">
       <c r="A36" s="6" t="inlineStr">
@@ -15326,6 +15698,11 @@
         </is>
       </c>
       <c r="D36" s="7" t="inlineStr"/>
+      <c r="E36" s="9" t="inlineStr">
+        <is>
+          <t>{q19.band}</t>
+        </is>
+      </c>
     </row>
     <row r="37">
       <c r="A37" s="6" t="inlineStr">
@@ -15344,6 +15721,7 @@
         </is>
       </c>
       <c r="D37" s="7" t="inlineStr"/>
+      <c r="E37" s="9" t="inlineStr"/>
     </row>
     <row r="38">
       <c r="A38" s="6" t="inlineStr">
@@ -15362,6 +15740,7 @@
         </is>
       </c>
       <c r="D38" s="7" t="inlineStr"/>
+      <c r="E38" s="9" t="inlineStr"/>
     </row>
     <row r="39">
       <c r="A39" s="6" t="inlineStr">
@@ -15380,6 +15759,7 @@
         </is>
       </c>
       <c r="D39" s="7" t="inlineStr"/>
+      <c r="E39" s="9" t="inlineStr"/>
     </row>
     <row r="40">
       <c r="A40" s="6" t="inlineStr">
@@ -15398,6 +15778,7 @@
         </is>
       </c>
       <c r="D40" s="7" t="inlineStr"/>
+      <c r="E40" s="9" t="inlineStr"/>
     </row>
     <row r="41">
       <c r="A41" s="6" t="inlineStr">
@@ -15416,6 +15797,7 @@
         </is>
       </c>
       <c r="D41" s="7" t="inlineStr"/>
+      <c r="E41" s="9" t="inlineStr"/>
     </row>
     <row r="42">
       <c r="A42" s="6" t="inlineStr">
@@ -15434,6 +15816,7 @@
         </is>
       </c>
       <c r="D42" s="7" t="inlineStr"/>
+      <c r="E42" s="9" t="inlineStr"/>
     </row>
     <row r="43">
       <c r="A43" s="6" t="inlineStr">
@@ -15452,6 +15835,7 @@
         </is>
       </c>
       <c r="D43" s="7" t="inlineStr"/>
+      <c r="E43" s="9" t="inlineStr"/>
     </row>
     <row r="44">
       <c r="A44" s="6" t="inlineStr">
@@ -15470,6 +15854,7 @@
         </is>
       </c>
       <c r="D44" s="7" t="inlineStr"/>
+      <c r="E44" s="9" t="inlineStr"/>
     </row>
     <row r="45">
       <c r="A45" s="6" t="inlineStr">
@@ -15488,6 +15873,7 @@
         </is>
       </c>
       <c r="D45" s="7" t="inlineStr"/>
+      <c r="E45" s="9" t="inlineStr"/>
     </row>
     <row r="46">
       <c r="A46" s="6" t="inlineStr">
@@ -15506,6 +15892,7 @@
         </is>
       </c>
       <c r="D46" s="7" t="inlineStr"/>
+      <c r="E46" s="9" t="inlineStr"/>
     </row>
     <row r="47">
       <c r="A47" s="6" t="inlineStr">
@@ -15528,6 +15915,11 @@
           <t>of the customers you had a year ago, {q21.exact}% still buy from you</t>
         </is>
       </c>
+      <c r="E47" s="9" t="inlineStr">
+        <is>
+          <t>{q21.band}, {q21.exact}</t>
+        </is>
+      </c>
     </row>
     <row r="48">
       <c r="A48" s="6" t="inlineStr">
@@ -15546,6 +15938,11 @@
         </is>
       </c>
       <c r="D48" s="7" t="inlineStr"/>
+      <c r="E48" s="9" t="inlineStr">
+        <is>
+          <t>{q22.band}</t>
+        </is>
+      </c>
     </row>
     <row r="49">
       <c r="A49" s="6" t="inlineStr">
@@ -15564,6 +15961,11 @@
         </is>
       </c>
       <c r="D49" s="7" t="inlineStr"/>
+      <c r="E49" s="9" t="inlineStr">
+        <is>
+          <t>{q23.band}</t>
+        </is>
+      </c>
     </row>
     <row r="50">
       <c r="A50" s="6" t="inlineStr">
@@ -15582,6 +15984,7 @@
         </is>
       </c>
       <c r="D50" s="7" t="inlineStr"/>
+      <c r="E50" s="9" t="inlineStr"/>
     </row>
     <row r="51">
       <c r="A51" s="6" t="inlineStr">
@@ -15600,6 +16003,7 @@
         </is>
       </c>
       <c r="D51" s="7" t="inlineStr"/>
+      <c r="E51" s="9" t="inlineStr"/>
     </row>
     <row r="52">
       <c r="A52" s="6" t="inlineStr">
@@ -15618,6 +16022,7 @@
         </is>
       </c>
       <c r="D52" s="7" t="inlineStr"/>
+      <c r="E52" s="9" t="inlineStr"/>
     </row>
     <row r="53">
       <c r="A53" s="6" t="inlineStr">
@@ -15636,6 +16041,7 @@
         </is>
       </c>
       <c r="D53" s="7" t="inlineStr"/>
+      <c r="E53" s="9" t="inlineStr"/>
     </row>
     <row r="54">
       <c r="A54" s="6" t="inlineStr">
@@ -15654,6 +16060,7 @@
         </is>
       </c>
       <c r="D54" s="7" t="inlineStr"/>
+      <c r="E54" s="9" t="inlineStr"/>
     </row>
     <row r="55">
       <c r="A55" s="6" t="inlineStr">
@@ -15672,6 +16079,7 @@
         </is>
       </c>
       <c r="D55" s="7" t="inlineStr"/>
+      <c r="E55" s="9" t="inlineStr"/>
     </row>
     <row r="56">
       <c r="A56" s="6" t="inlineStr">
@@ -15690,6 +16098,7 @@
         </is>
       </c>
       <c r="D56" s="7" t="inlineStr"/>
+      <c r="E56" s="9" t="inlineStr"/>
     </row>
     <row r="57">
       <c r="A57" s="6" t="inlineStr">
@@ -15708,6 +16117,7 @@
         </is>
       </c>
       <c r="D57" s="7" t="inlineStr"/>
+      <c r="E57" s="9" t="inlineStr"/>
     </row>
     <row r="58">
       <c r="A58" s="6" t="inlineStr">
@@ -15726,6 +16136,7 @@
         </is>
       </c>
       <c r="D58" s="7" t="inlineStr"/>
+      <c r="E58" s="9" t="inlineStr"/>
     </row>
     <row r="59">
       <c r="A59" s="6" t="inlineStr">
@@ -15744,6 +16155,7 @@
         </is>
       </c>
       <c r="D59" s="7" t="inlineStr"/>
+      <c r="E59" s="9" t="inlineStr"/>
     </row>
     <row r="60">
       <c r="A60" s="6" t="inlineStr">
@@ -15766,6 +16178,11 @@
           <t>your close rate sits at {q26.exact}%</t>
         </is>
       </c>
+      <c r="E60" s="9" t="inlineStr">
+        <is>
+          <t>{q26.band}, {q26.exact}</t>
+        </is>
+      </c>
     </row>
     <row r="61">
       <c r="A61" s="6" t="inlineStr">
@@ -15784,6 +16201,11 @@
         </is>
       </c>
       <c r="D61" s="7" t="inlineStr"/>
+      <c r="E61" s="9" t="inlineStr">
+        <is>
+          <t>{q27.band}</t>
+        </is>
+      </c>
     </row>
     <row r="62">
       <c r="A62" s="6" t="inlineStr">
@@ -15802,6 +16224,11 @@
         </is>
       </c>
       <c r="D62" s="7" t="inlineStr"/>
+      <c r="E62" s="9" t="inlineStr">
+        <is>
+          <t>{q28.band}</t>
+        </is>
+      </c>
     </row>
     <row r="63">
       <c r="A63" s="6" t="inlineStr">
@@ -15820,6 +16247,7 @@
         </is>
       </c>
       <c r="D63" s="7" t="inlineStr"/>
+      <c r="E63" s="9" t="inlineStr"/>
     </row>
     <row r="64">
       <c r="A64" s="6" t="inlineStr">
@@ -15838,6 +16266,7 @@
         </is>
       </c>
       <c r="D64" s="7" t="inlineStr"/>
+      <c r="E64" s="9" t="inlineStr"/>
     </row>
     <row r="65">
       <c r="A65" s="6" t="inlineStr">
@@ -15856,6 +16285,7 @@
         </is>
       </c>
       <c r="D65" s="7" t="inlineStr"/>
+      <c r="E65" s="9" t="inlineStr"/>
     </row>
     <row r="66">
       <c r="A66" s="6" t="inlineStr">
@@ -15874,6 +16304,7 @@
         </is>
       </c>
       <c r="D66" s="7" t="inlineStr"/>
+      <c r="E66" s="9" t="inlineStr"/>
     </row>
     <row r="67">
       <c r="A67" s="6" t="inlineStr">
@@ -15892,6 +16323,7 @@
         </is>
       </c>
       <c r="D67" s="7" t="inlineStr"/>
+      <c r="E67" s="9" t="inlineStr"/>
     </row>
     <row r="68">
       <c r="A68" s="6" t="inlineStr">
@@ -15910,6 +16342,7 @@
         </is>
       </c>
       <c r="D68" s="7" t="inlineStr"/>
+      <c r="E68" s="9" t="inlineStr"/>
     </row>
     <row r="69">
       <c r="A69" s="6" t="inlineStr">
@@ -15928,6 +16361,7 @@
         </is>
       </c>
       <c r="D69" s="7" t="inlineStr"/>
+      <c r="E69" s="9" t="inlineStr"/>
     </row>
     <row r="70">
       <c r="A70" s="6" t="inlineStr">
@@ -15946,6 +16380,7 @@
         </is>
       </c>
       <c r="D70" s="7" t="inlineStr"/>
+      <c r="E70" s="9" t="inlineStr"/>
     </row>
     <row r="71">
       <c r="A71" s="6" t="inlineStr">
@@ -15964,6 +16399,7 @@
         </is>
       </c>
       <c r="D71" s="7" t="inlineStr"/>
+      <c r="E71" s="9" t="inlineStr"/>
     </row>
     <row r="72">
       <c r="A72" s="6" t="inlineStr">
@@ -15982,6 +16418,7 @@
         </is>
       </c>
       <c r="D72" s="7" t="inlineStr"/>
+      <c r="E72" s="9" t="inlineStr"/>
     </row>
     <row r="73">
       <c r="A73" s="6" t="inlineStr">
@@ -16004,6 +16441,11 @@
           <t>enquiries run at about {q31.exact} a month</t>
         </is>
       </c>
+      <c r="E73" s="9" t="inlineStr">
+        <is>
+          <t>{q31.band}, {q31.exact}</t>
+        </is>
+      </c>
     </row>
     <row r="74">
       <c r="A74" s="6" t="inlineStr">
@@ -16022,6 +16464,11 @@
         </is>
       </c>
       <c r="D74" s="7" t="inlineStr"/>
+      <c r="E74" s="9" t="inlineStr">
+        <is>
+          <t>{q33.band}</t>
+        </is>
+      </c>
     </row>
     <row r="75">
       <c r="A75" s="6" t="inlineStr">
@@ -16040,6 +16487,11 @@
         </is>
       </c>
       <c r="D75" s="7" t="inlineStr"/>
+      <c r="E75" s="9" t="inlineStr">
+        <is>
+          <t>{q35.band}</t>
+        </is>
+      </c>
     </row>
     <row r="76">
       <c r="A76" s="6" t="inlineStr">
@@ -16058,6 +16510,7 @@
         </is>
       </c>
       <c r="D76" s="7" t="inlineStr"/>
+      <c r="E76" s="9" t="inlineStr"/>
     </row>
     <row r="77">
       <c r="A77" s="6" t="inlineStr">
@@ -16076,6 +16529,7 @@
         </is>
       </c>
       <c r="D77" s="7" t="inlineStr"/>
+      <c r="E77" s="9" t="inlineStr"/>
     </row>
     <row r="78">
       <c r="A78" s="6" t="inlineStr">
@@ -16094,6 +16548,7 @@
         </is>
       </c>
       <c r="D78" s="7" t="inlineStr"/>
+      <c r="E78" s="9" t="inlineStr"/>
     </row>
     <row r="79">
       <c r="A79" s="6" t="inlineStr">
@@ -16112,6 +16567,7 @@
         </is>
       </c>
       <c r="D79" s="7" t="inlineStr"/>
+      <c r="E79" s="9" t="inlineStr"/>
     </row>
     <row r="80">
       <c r="A80" s="6" t="inlineStr">
@@ -16130,6 +16586,7 @@
         </is>
       </c>
       <c r="D80" s="7" t="inlineStr"/>
+      <c r="E80" s="9" t="inlineStr"/>
     </row>
     <row r="81">
       <c r="A81" s="6" t="inlineStr">
@@ -16148,6 +16605,7 @@
         </is>
       </c>
       <c r="D81" s="7" t="inlineStr"/>
+      <c r="E81" s="9" t="inlineStr"/>
     </row>
     <row r="82">
       <c r="A82" s="6" t="inlineStr">
@@ -16166,6 +16624,7 @@
         </is>
       </c>
       <c r="D82" s="7" t="inlineStr"/>
+      <c r="E82" s="9" t="inlineStr"/>
     </row>
     <row r="83">
       <c r="A83" s="6" t="inlineStr">
@@ -16184,6 +16643,7 @@
         </is>
       </c>
       <c r="D83" s="7" t="inlineStr"/>
+      <c r="E83" s="9" t="inlineStr"/>
     </row>
     <row r="84">
       <c r="A84" s="6" t="inlineStr">
@@ -16202,6 +16662,7 @@
         </is>
       </c>
       <c r="D84" s="7" t="inlineStr"/>
+      <c r="E84" s="9" t="inlineStr"/>
     </row>
     <row r="85">
       <c r="A85" s="6" t="inlineStr">
@@ -16220,6 +16681,7 @@
         </is>
       </c>
       <c r="D85" s="7" t="inlineStr"/>
+      <c r="E85" s="9" t="inlineStr"/>
     </row>
     <row r="86">
       <c r="A86" s="6" t="inlineStr">
@@ -16242,6 +16704,11 @@
           <t>what's left after direct costs sits at {q36.exact}%</t>
         </is>
       </c>
+      <c r="E86" s="9" t="inlineStr">
+        <is>
+          <t>{q36.band}, {q36.exact}</t>
+        </is>
+      </c>
     </row>
     <row r="87">
       <c r="A87" s="6" t="inlineStr">
@@ -16264,6 +16731,11 @@
           <t>after everything it's {q37.exact}%</t>
         </is>
       </c>
+      <c r="E87" s="9" t="inlineStr">
+        <is>
+          <t>{q37.band}, {q37.exact}</t>
+        </is>
+      </c>
     </row>
     <row r="88">
       <c r="A88" s="6" t="inlineStr">
@@ -16282,6 +16754,11 @@
         </is>
       </c>
       <c r="D88" s="7" t="inlineStr"/>
+      <c r="E88" s="9" t="inlineStr">
+        <is>
+          <t>{q38.band}</t>
+        </is>
+      </c>
     </row>
     <row r="89">
       <c r="A89" s="6" t="inlineStr">
@@ -16300,6 +16777,11 @@
         </is>
       </c>
       <c r="D89" s="7" t="inlineStr"/>
+      <c r="E89" s="9" t="inlineStr">
+        <is>
+          <t>{q39.band}</t>
+        </is>
+      </c>
     </row>
     <row r="90">
       <c r="A90" s="6" t="inlineStr">
@@ -16318,6 +16800,7 @@
         </is>
       </c>
       <c r="D90" s="7" t="inlineStr"/>
+      <c r="E90" s="9" t="inlineStr"/>
     </row>
     <row r="91">
       <c r="A91" s="6" t="inlineStr">
@@ -16336,6 +16819,7 @@
         </is>
       </c>
       <c r="D91" s="7" t="inlineStr"/>
+      <c r="E91" s="9" t="inlineStr"/>
     </row>
     <row r="92">
       <c r="A92" s="6" t="inlineStr">
@@ -16354,6 +16838,7 @@
         </is>
       </c>
       <c r="D92" s="7" t="inlineStr"/>
+      <c r="E92" s="9" t="inlineStr"/>
     </row>
     <row r="93">
       <c r="A93" s="6" t="inlineStr">
@@ -16372,6 +16857,7 @@
         </is>
       </c>
       <c r="D93" s="7" t="inlineStr"/>
+      <c r="E93" s="9" t="inlineStr"/>
     </row>
     <row r="94">
       <c r="A94" s="6" t="inlineStr">
@@ -16390,6 +16876,7 @@
         </is>
       </c>
       <c r="D94" s="7" t="inlineStr"/>
+      <c r="E94" s="9" t="inlineStr"/>
     </row>
     <row r="95">
       <c r="A95" s="6" t="inlineStr">
@@ -16408,6 +16895,7 @@
         </is>
       </c>
       <c r="D95" s="7" t="inlineStr"/>
+      <c r="E95" s="9" t="inlineStr"/>
     </row>
     <row r="96">
       <c r="A96" s="6" t="inlineStr">
@@ -16426,11 +16914,12 @@
         </is>
       </c>
       <c r="D96" s="7" t="inlineStr"/>
+      <c r="E96" s="9" t="inlineStr"/>
     </row>
   </sheetData>
-  <autoFilter ref="A2:D96"/>
+  <autoFilter ref="A2:E96"/>
   <mergeCells count="1">
-    <mergeCell ref="A1:D1"/>
+    <mergeCell ref="A1:E1"/>
   </mergeCells>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
@@ -16442,12 +16931,13 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:C9"/>
+  <dimension ref="A1:D9"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="13" customWidth="1" min="1" max="1"/>
     <col width="24" customWidth="1" min="2" max="2"/>
-    <col width="110" customWidth="1" min="3" max="3"/>
+    <col width="100" customWidth="1" min="3" max="3"/>
+    <col width="24" customWidth="1" min="4" max="4"/>
   </cols>
   <sheetData>
     <row r="1" ht="30" customHeight="1">
@@ -16473,6 +16963,11 @@
           <t>The one line printed when this is a loud but downstream second finding</t>
         </is>
       </c>
+      <c r="D2" s="1" t="inlineStr">
+        <is>
+          <t>Variables in this row</t>
+        </is>
+      </c>
     </row>
     <row r="3">
       <c r="A3" s="6" t="inlineStr">
@@ -16490,6 +16985,11 @@
           <t>There's cash flow strain in your answers too. It sits downstream of the {d.primaryShort} problem and it should ease as that one moves.</t>
         </is>
       </c>
+      <c r="D3" s="9" t="inlineStr">
+        <is>
+          <t>{d.primaryShort}</t>
+        </is>
+      </c>
     </row>
     <row r="4">
       <c r="A4" s="6" t="inlineStr">
@@ -16507,6 +17007,11 @@
           <t>A talent gap shows up in your answers as well. It's downstream of the {d.primaryShort} problem, so it isn't the thing to work on first.</t>
         </is>
       </c>
+      <c r="D4" s="9" t="inlineStr">
+        <is>
+          <t>{d.primaryShort}</t>
+        </is>
+      </c>
     </row>
     <row r="5">
       <c r="A5" s="6" t="inlineStr">
@@ -16524,6 +17029,11 @@
           <t>You'll see fulfilment strain in here as well. That's downstream of the {d.primaryShort} problem, and it should settle once the layer above it is in place.</t>
         </is>
       </c>
+      <c r="D5" s="9" t="inlineStr">
+        <is>
+          <t>{d.primaryShort}</t>
+        </is>
+      </c>
     </row>
     <row r="6">
       <c r="A6" s="6" t="inlineStr">
@@ -16541,6 +17051,11 @@
           <t>Retention looks soft too. That's downstream of the {d.primaryShort} problem rather than a separate finding.</t>
         </is>
       </c>
+      <c r="D6" s="9" t="inlineStr">
+        <is>
+          <t>{d.primaryShort}</t>
+        </is>
+      </c>
     </row>
     <row r="7">
       <c r="A7" s="6" t="inlineStr">
@@ -16558,6 +17073,11 @@
           <t>The offer looks weak in places as well. Downstream of the {d.primaryShort} problem, and not worth touching yet.</t>
         </is>
       </c>
+      <c r="D7" s="9" t="inlineStr">
+        <is>
+          <t>{d.primaryShort}</t>
+        </is>
+      </c>
     </row>
     <row r="8">
       <c r="A8" s="6" t="inlineStr">
@@ -16575,6 +17095,11 @@
           <t>Demand reads thin too. It's downstream of the {d.primaryShort} problem, so leave it where it is.</t>
         </is>
       </c>
+      <c r="D8" s="9" t="inlineStr">
+        <is>
+          <t>{d.primaryShort}</t>
+        </is>
+      </c>
     </row>
     <row r="9">
       <c r="A9" s="6" t="inlineStr">
@@ -16592,11 +17117,16 @@
           <t>Margin looks tight as well. That's downstream of the {d.primaryShort} problem and it'll move when that does.</t>
         </is>
       </c>
+      <c r="D9" s="9" t="inlineStr">
+        <is>
+          <t>{d.primaryShort}</t>
+        </is>
+      </c>
     </row>
   </sheetData>
-  <autoFilter ref="A2:C9"/>
+  <autoFilter ref="A2:D9"/>
   <mergeCells count="1">
-    <mergeCell ref="A1:C1"/>
+    <mergeCell ref="A1:D1"/>
   </mergeCells>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
@@ -16608,16 +17138,17 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:G18"/>
+  <dimension ref="A1:H18"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="15" customWidth="1" min="1" max="1"/>
     <col width="19" customWidth="1" min="2" max="2"/>
     <col width="22" customWidth="1" min="3" max="3"/>
-    <col width="78" customWidth="1" min="4" max="4"/>
-    <col width="62" customWidth="1" min="5" max="5"/>
-    <col width="78" customWidth="1" min="6" max="6"/>
-    <col width="72" customWidth="1" min="7" max="7"/>
+    <col width="72" customWidth="1" min="4" max="4"/>
+    <col width="56" customWidth="1" min="5" max="5"/>
+    <col width="72" customWidth="1" min="6" max="6"/>
+    <col width="66" customWidth="1" min="7" max="7"/>
+    <col width="24" customWidth="1" min="8" max="8"/>
   </cols>
   <sheetData>
     <row r="1" ht="30" customHeight="1">
@@ -16663,6 +17194,11 @@
           <t>What to do</t>
         </is>
       </c>
+      <c r="H2" s="1" t="inlineStr">
+        <is>
+          <t>Variables in this row</t>
+        </is>
+      </c>
     </row>
     <row r="3">
       <c r="A3" s="5" t="inlineStr">
@@ -16696,6 +17232,11 @@
           <t>Set a ceiling, say twenty percent of revenue from any one customer, and treat crossing it as the trigger to go and win two more. Get them onto a term agreement in the meantime.</t>
         </is>
       </c>
+      <c r="H3" s="9" t="inlineStr">
+        <is>
+          <t>{q41.band}, {q41.exact}</t>
+        </is>
+      </c>
     </row>
     <row r="4">
       <c r="A4" s="5" t="inlineStr">
@@ -16727,6 +17268,11 @@
       <c r="G4" s="7" t="inlineStr">
         <is>
           <t>Build a second line and sell it to the customers you already have. It's cheaper than finding new customers for the line you've got.</t>
+        </is>
+      </c>
+      <c r="H4" s="9" t="inlineStr">
+        <is>
+          <t>{q42.band}, {q42.exact}</t>
         </is>
       </c>
     </row>
@@ -16758,6 +17304,11 @@
           <t>Stand up a second channel before you need it, and give it ninety days before you judge it. One channel is a decision somebody else gets to make on your behalf.</t>
         </is>
       </c>
+      <c r="H5" s="9" t="inlineStr">
+        <is>
+          <t>{q43.band}</t>
+        </is>
+      </c>
     </row>
     <row r="6">
       <c r="A6" s="5" t="inlineStr">
@@ -16787,6 +17338,7 @@
           <t>Qualify a second supplier and give them ten percent of your volume. A backup you've never actually bought from isn't a backup.</t>
         </is>
       </c>
+      <c r="H6" s="9" t="inlineStr"/>
     </row>
     <row r="7">
       <c r="A7" s="5" t="inlineStr">
@@ -16816,6 +17368,7 @@
           <t>Write down what they hold, then move one piece of it to somebody else this month. Repeat until nothing sits in one head.</t>
         </is>
       </c>
+      <c r="H7" s="9" t="inlineStr"/>
     </row>
     <row r="8">
       <c r="A8" s="5" t="inlineStr">
@@ -16845,6 +17398,7 @@
           <t>Have them document the work while they're still here, and pay them properly to do it. It's the cheapest insurance available to you.</t>
         </is>
       </c>
+      <c r="H8" s="9" t="inlineStr"/>
     </row>
     <row r="9">
       <c r="A9" s="5" t="inlineStr">
@@ -16874,6 +17428,7 @@
           <t>Take one thing you do well and sell it somewhere else, even at a small scale. Proving it travels is the whole exercise.</t>
         </is>
       </c>
+      <c r="H9" s="9" t="inlineStr"/>
     </row>
     <row r="10">
       <c r="A10" s="5" t="inlineStr">
@@ -16907,6 +17462,11 @@
           <t>Build to one month of fixed costs in a separate account, then three. Move a fixed percentage of every payment that comes in, automatically, so it isn't a decision you make each time.</t>
         </is>
       </c>
+      <c r="H10" s="9" t="inlineStr">
+        <is>
+          <t>{q8.band}</t>
+        </is>
+      </c>
     </row>
     <row r="11">
       <c r="A11" s="5" t="inlineStr">
@@ -16940,6 +17500,11 @@
           <t>Put a written agreement behind every piece of work, with terms, scope and a notice period. Start with your largest customers.</t>
         </is>
       </c>
+      <c r="H11" s="9" t="inlineStr">
+        <is>
+          <t>{q45.band}</t>
+        </is>
+      </c>
     </row>
     <row r="12">
       <c r="A12" s="5" t="inlineStr">
@@ -16973,6 +17538,11 @@
           <t>Record yourself doing the five things that go wrong most often, then turn each one into a one page checklist. Checklists beat manuals, because people actually use them.</t>
         </is>
       </c>
+      <c r="H12" s="9" t="inlineStr">
+        <is>
+          <t>{q46.band}</t>
+        </is>
+      </c>
     </row>
     <row r="13">
       <c r="A13" s="5" t="inlineStr">
@@ -17004,6 +17574,11 @@
       <c r="G13" s="7" t="inlineStr">
         <is>
           <t>Pick five numbers and look at them weekly. Cash in the bank, enquiries, close rate, jobs delivered, and margin on the last ten jobs. One page, same day every week.</t>
+        </is>
+      </c>
+      <c r="H13" s="9" t="inlineStr">
+        <is>
+          <t>{q47.band}</t>
         </is>
       </c>
     </row>
@@ -17035,6 +17610,7 @@
           <t>Name the person, tell them, and start handing over one area at a time with the decisions attached. A deputy who can't decide anything is a job title.</t>
         </is>
       </c>
+      <c r="H14" s="9" t="inlineStr"/>
     </row>
     <row r="15">
       <c r="A15" s="5" t="inlineStr">
@@ -17068,6 +17644,11 @@
           <t>Work out what only you can do and start moving everything else. The test is whether the business survives you taking a month off, so book the month and find out.</t>
         </is>
       </c>
+      <c r="H15" s="9" t="inlineStr">
+        <is>
+          <t>{q49.band}</t>
+        </is>
+      </c>
     </row>
     <row r="16">
       <c r="A16" s="5" t="inlineStr">
@@ -17101,6 +17682,11 @@
           <t>Write the one page version. Who runs it, what happens to the customers, what it's worth and who'd buy it. It doesn't need to be right, it needs to exist.</t>
         </is>
       </c>
+      <c r="H16" s="9" t="inlineStr">
+        <is>
+          <t>{q50.band}</t>
+        </is>
+      </c>
     </row>
     <row r="17">
       <c r="A17" s="5" t="inlineStr">
@@ -17134,6 +17720,11 @@
           <t>List every guarantee you've signed and put a date against each one to renegotiate or release it. Most get renewed on autopilot because nobody asks.</t>
         </is>
       </c>
+      <c r="H17" s="9" t="inlineStr">
+        <is>
+          <t>{q51.band}</t>
+        </is>
+      </c>
     </row>
     <row r="18">
       <c r="A18" s="5" t="inlineStr">
@@ -17167,11 +17758,16 @@
           <t>Write down what you actually wanted out of this, then hold your week up against it. The gap is the brief for the next twelve months.</t>
         </is>
       </c>
+      <c r="H18" s="9" t="inlineStr">
+        <is>
+          <t>{q52.band}</t>
+        </is>
+      </c>
     </row>
   </sheetData>
-  <autoFilter ref="A2:G18"/>
+  <autoFilter ref="A2:H18"/>
   <mergeCells count="1">
-    <mergeCell ref="A1:G1"/>
+    <mergeCell ref="A1:H1"/>
   </mergeCells>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
@@ -17342,13 +17938,14 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:D19"/>
+  <dimension ref="A1:E19"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="13" customWidth="1" min="1" max="1"/>
     <col width="20" customWidth="1" min="2" max="2"/>
     <col width="8" customWidth="1" min="3" max="3"/>
-    <col width="122" customWidth="1" min="4" max="4"/>
+    <col width="112" customWidth="1" min="4" max="4"/>
+    <col width="24" customWidth="1" min="5" max="5"/>
   </cols>
   <sheetData>
     <row r="1" ht="30" customHeight="1">
@@ -17379,6 +17976,11 @@
           <t>Block. Prints when both are present</t>
         </is>
       </c>
+      <c r="E2" s="1" t="inlineStr">
+        <is>
+          <t>Variables in this row</t>
+        </is>
+      </c>
     </row>
     <row r="3">
       <c r="A3" s="6" t="inlineStr">
@@ -17399,6 +18001,11 @@
           <t>Cash flow is your constraint and one customer carries {q41.band} of your revenue. That customer is also setting your payment terms, which means they're setting your cash position. Fixing terms with them is worth more than everything else on the list.</t>
         </is>
       </c>
+      <c r="E3" s="9" t="inlineStr">
+        <is>
+          <t>{q41.band}</t>
+        </is>
+      </c>
     </row>
     <row r="4">
       <c r="A4" s="6" t="inlineStr">
@@ -17419,6 +18026,7 @@
           <t>You're cash constrained and personally guaranteeing the business's obligations. That's the combination that follows people home. Get the buffer built before you take on another dollar of guaranteed debt.</t>
         </is>
       </c>
+      <c r="E4" s="9" t="inlineStr"/>
     </row>
     <row r="5">
       <c r="A5" s="6" t="inlineStr">
@@ -17439,6 +18047,7 @@
           <t>Cash flow is your constraint and your work isn't contracted. You're funding jobs upfront for customers who can walk without penalty. Deposits and written terms deal with both at once.</t>
         </is>
       </c>
+      <c r="E5" s="9" t="inlineStr"/>
     </row>
     <row r="6">
       <c r="A6" s="6" t="inlineStr">
@@ -17459,6 +18068,7 @@
           <t>You're cash constrained and you're not looking at the numbers often enough to see it coming. A thirteen week cash forecast, updated weekly, is the highest value hour in your month right now.</t>
         </is>
       </c>
+      <c r="E6" s="9" t="inlineStr"/>
     </row>
     <row r="7">
       <c r="A7" s="6" t="inlineStr">
@@ -17479,6 +18089,7 @@
           <t>You're demand constrained and the one channel you have isn't producing. A second channel is the fix and it's also the risk mitigation. Same move, two problems.</t>
         </is>
       </c>
+      <c r="E7" s="9" t="inlineStr"/>
     </row>
     <row r="8">
       <c r="A8" s="6" t="inlineStr">
@@ -17499,6 +18110,11 @@
           <t>You're quiet and one customer carries {q41.band} of your revenue. Together those mean the business is one phone call from a crisis. New demand is urgent here for reasons that have nothing to do with growth.</t>
         </is>
       </c>
+      <c r="E8" s="9" t="inlineStr">
+        <is>
+          <t>{q41.band}</t>
+        </is>
+      </c>
     </row>
     <row r="9">
       <c r="A9" s="6" t="inlineStr">
@@ -17519,6 +18135,7 @@
           <t>You're fulfilment constrained and almost nothing is written down. Those aren't two findings. Undocumented work is slow work, and it's why adding people hasn't given you the output you expected.</t>
         </is>
       </c>
+      <c r="E9" s="9" t="inlineStr"/>
     </row>
     <row r="10">
       <c r="A10" s="6" t="inlineStr">
@@ -17539,6 +18156,7 @@
           <t>You're at capacity and one person holds how the work actually gets done. Every hire you make is rate limited by the one person who has to train them. Getting that knowledge out of one head is what unlocks the capacity.</t>
         </is>
       </c>
+      <c r="E10" s="9" t="inlineStr"/>
     </row>
     <row r="11">
       <c r="A11" s="6" t="inlineStr">
@@ -17559,6 +18177,7 @@
           <t>You're at capacity and the business depends on one person to function. Adding work to that arrangement adds it to them. The capacity you're missing is currently locked in one diary.</t>
         </is>
       </c>
+      <c r="E11" s="9" t="inlineStr"/>
     </row>
     <row r="12">
       <c r="A12" s="6" t="inlineStr">
@@ -17579,6 +18198,7 @@
           <t>Margin is your constraint and you don't know which work makes money. You're almost certainly subsidising some customers with others, and until you can see which, every pricing decision you make is a guess.</t>
         </is>
       </c>
+      <c r="E12" s="9" t="inlineStr"/>
     </row>
     <row r="13">
       <c r="A13" s="6" t="inlineStr">
@@ -17599,6 +18219,11 @@
           <t>Margin is tight and one customer carries {q41.band} of your revenue. Big customers get big customer pricing, and yours is probably the one holding the margin down. Repricing them is the fastest lever you have, and it's the scariest, which is why it hasn't happened.</t>
         </is>
       </c>
+      <c r="E13" s="9" t="inlineStr">
+        <is>
+          <t>{q41.band}</t>
+        </is>
+      </c>
     </row>
     <row r="14">
       <c r="A14" s="6" t="inlineStr">
@@ -17619,6 +18244,7 @@
           <t>The offer is your constraint and nearly all your enquiries come through one channel. That's why this feels like a demand problem. The channel is working. The thing it's delivering people to isn't.</t>
         </is>
       </c>
+      <c r="E14" s="9" t="inlineStr"/>
     </row>
     <row r="15">
       <c r="A15" s="6" t="inlineStr">
@@ -17639,6 +18265,7 @@
           <t>Your constraint is talent and your key person risk is the same thing seen from the other side. The layer that doesn't exist is the reason everything routes through one person, so hiring the role deals with both. Treat it as one job rather than two.</t>
         </is>
       </c>
+      <c r="E15" s="9" t="inlineStr"/>
     </row>
     <row r="16">
       <c r="A16" s="6" t="inlineStr">
@@ -17659,6 +18286,7 @@
           <t>You're talent constrained and the business is close to unsellable, and both of those come from the same fact. The business runs on you. The role you haven't hired is also the thing standing between you and owning something a buyer would want.</t>
         </is>
       </c>
+      <c r="E16" s="9" t="inlineStr"/>
     </row>
     <row r="17">
       <c r="A17" s="6" t="inlineStr">
@@ -17679,6 +18307,7 @@
           <t>The missing layer and the missing second in command are one problem with two names. You don't need a succession plan and a hire. You need the hire, and the succession plan writes itself afterwards.</t>
         </is>
       </c>
+      <c r="E17" s="9" t="inlineStr"/>
     </row>
     <row r="18">
       <c r="A18" s="6" t="inlineStr">
@@ -17699,6 +18328,11 @@
           <t>You're carrying a talent gap and a single customer worth {q41.band} of revenue. Building the layer while one customer can end your year is the sequencing error we'd flag hardest. Get that customer onto a term agreement before you take on the salary.</t>
         </is>
       </c>
+      <c r="E18" s="9" t="inlineStr">
+        <is>
+          <t>{q41.band}</t>
+        </is>
+      </c>
     </row>
     <row r="19">
       <c r="A19" s="6" t="inlineStr">
@@ -17719,11 +18353,12 @@
           <t>Retention is your constraint and you don't know why customers leave. Those are the same sentence. Ten phone calls this week would find the leak, and nothing you do before those calls is anything but a guess.</t>
         </is>
       </c>
+      <c r="E19" s="9" t="inlineStr"/>
     </row>
   </sheetData>
-  <autoFilter ref="A2:D19"/>
+  <autoFilter ref="A2:E19"/>
   <mergeCells count="1">
-    <mergeCell ref="A1:D1"/>
+    <mergeCell ref="A1:E1"/>
   </mergeCells>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Diagnostic: Ryan's talent and fulfilment rewrites, plus an audit marker
Talent is a missing layer, not missing hands, so the opening says that and
none of the five fix actions reassign work to somebody already in the
business. The five steps are Ryan's sequence: list last week's tasks, name
the role that should own each, hire the role with the most against it,
give it responsibility and authority, train it yourself and give it ninety
days. The don't redraw the org chart line is gone.

Fulfilment is capacity, not capability. The fix order is refine what you
have, cut what isn't earning its capacity, then hire. Don't Do This Yet is
back to four blunt lines.

AUDIT-PROGRESS.md records that the read stops at value constrained and that
value and offer are blocked on Ryan picking how to split them.

Co-Authored-By: Claude Opus 5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01EA6msubCCPndLhAZDV4oLH
</commit_message>
<xml_diff>
--- a/diagnostic/Business-Diagnostic-Spec.xlsx
+++ b/diagnostic/Business-Diagnostic-Spec.xlsx
@@ -24,10 +24,10 @@
     <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="1">'Questions'!$A$2:$J$60</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="2" hidden="1">'Answer options'!$A$2:$I$305</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="3" hidden="1">'Constraints and order'!$A$2:$G$9</definedName>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="4" hidden="1">'Report, constraint'!$A$2:$E$108</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="4" hidden="1">'Report, constraint'!$A$2:$E$106</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="5" hidden="1">'Report, risk flags'!$A$2:$H$12</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="6" hidden="1">'Report, risk section'!$A$2:$B$3</definedName>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="7" hidden="1">'Report, don''t do yet'!$A$2:$C$44</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="7" hidden="1">'Report, don''t do yet'!$A$2:$C$42</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="8" hidden="1">'Report, open and close'!$A$2:$E$14</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="9" hidden="1">'Thresholds'!$A$2:$C$8</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="10" hidden="1">'Logic'!$A$1:$B$14</definedName>
@@ -15465,7 +15465,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E108"/>
+  <dimension ref="A1:E106"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="13" customWidth="1" min="1" max="1"/>
@@ -15935,7 +15935,7 @@
       </c>
       <c r="C22" s="7" t="inlineStr">
         <is>
-          <t>Talent here means a missing layer, not missing hands.</t>
+          <t>Being talent constrained means you're missing a layer in the business, not missing extra hands.</t>
         </is>
       </c>
       <c r="D22" s="7" t="inlineStr"/>
@@ -16088,7 +16088,7 @@
       </c>
       <c r="C29" s="7" t="inlineStr">
         <is>
-          <t>You need one role hired with the authority to actually run what you hand over, rather than another pair of hands underneath you.</t>
+          <t>Hire one role that owns a layer of the business, with the authority to run it. Not another pair of hands underneath you.</t>
         </is>
       </c>
       <c r="D29" s="7" t="inlineStr"/>
@@ -16107,13 +16107,13 @@
       </c>
       <c r="C30" s="7" t="inlineStr">
         <is>
-          <t>Every layer sits with you. Hire the one that would free the most of your week first, not the one that's easiest to fill.</t>
+          <t>Write down every task you did last week.</t>
         </is>
       </c>
       <c r="D30" s="7" t="inlineStr"/>
       <c r="E30" s="8" t="inlineStr">
         <is>
-          <t>q11 is n</t>
+          <t>always prints</t>
         </is>
       </c>
     </row>
@@ -16130,7 +16130,7 @@
       </c>
       <c r="C31" s="7" t="inlineStr">
         <is>
-          <t>List every task you touched last week. Against each one, write the name of the person who'd do it if you were away for a month. Any task with no name against it is the hire.</t>
+          <t>Against each one, write the role that should own it. A role, not a person already in the business.</t>
         </is>
       </c>
       <c r="D31" s="7" t="inlineStr"/>
@@ -16153,7 +16153,7 @@
       </c>
       <c r="C32" s="7" t="inlineStr">
         <is>
-          <t>Hire the layer rather than the hands. Another delivery person gives you more capacity. A person who runs delivery gives you your week back.</t>
+          <t>Whichever role has the most tasks against it, or the most hours, hire that role first.</t>
         </is>
       </c>
       <c r="D32" s="7" t="inlineStr"/>
@@ -16176,13 +16176,13 @@
       </c>
       <c r="C33" s="7" t="inlineStr">
         <is>
-          <t>You've got more direct reports than one person can run properly. The hire that fixes this sits between you and most of them.</t>
+          <t>Give them responsibility and the authority to go with it. One without the other doesn't work.</t>
         </is>
       </c>
       <c r="D33" s="7" t="inlineStr"/>
       <c r="E33" s="8" t="inlineStr">
         <is>
-          <t>q15 is d/e</t>
+          <t>always prints</t>
         </is>
       </c>
     </row>
@@ -16199,7 +16199,7 @@
       </c>
       <c r="C34" s="7" t="inlineStr">
         <is>
-          <t>Hand over one whole area with the decisions attached. Half a handover leaves you doing the work and them carrying the confusion.</t>
+          <t>Train them yourself, then give them ninety days to prove they're the one.</t>
         </is>
       </c>
       <c r="D34" s="7" t="inlineStr"/>
@@ -16212,25 +16212,21 @@
     <row r="35">
       <c r="A35" s="6" t="inlineStr">
         <is>
-          <t>talent</t>
+          <t>fulfilment</t>
         </is>
       </c>
       <c r="B35" s="6" t="inlineStr">
         <is>
-          <t>Fix action 6</t>
+          <t>Title</t>
         </is>
       </c>
       <c r="C35" s="7" t="inlineStr">
         <is>
-          <t>Give it ninety days before you judge it, and don't let yourself become the escalation point for what you handed over.</t>
+          <t>You are {c} constrained</t>
         </is>
       </c>
       <c r="D35" s="7" t="inlineStr"/>
-      <c r="E35" s="8" t="inlineStr">
-        <is>
-          <t>always prints</t>
-        </is>
-      </c>
+      <c r="E35" s="8" t="inlineStr"/>
     </row>
     <row r="36">
       <c r="A36" s="6" t="inlineStr">
@@ -16240,12 +16236,12 @@
       </c>
       <c r="B36" s="6" t="inlineStr">
         <is>
-          <t>Title</t>
+          <t>Title, nothing failing</t>
         </is>
       </c>
       <c r="C36" s="7" t="inlineStr">
         <is>
-          <t>You are {c} constrained</t>
+          <t>The tightest thing is {c}</t>
         </is>
       </c>
       <c r="D36" s="7" t="inlineStr"/>
@@ -16259,12 +16255,12 @@
       </c>
       <c r="B37" s="6" t="inlineStr">
         <is>
-          <t>Title, nothing failing</t>
+          <t>Opening</t>
         </is>
       </c>
       <c r="C37" s="7" t="inlineStr">
         <is>
-          <t>The tightest thing is {c}</t>
+          <t>This is capacity, not capability. You know how to do the work, but you can't do enough of it.</t>
         </is>
       </c>
       <c r="D37" s="7" t="inlineStr"/>
@@ -16278,16 +16274,24 @@
       </c>
       <c r="B38" s="6" t="inlineStr">
         <is>
-          <t>Opening</t>
+          <t>Evidence clause 1</t>
         </is>
       </c>
       <c r="C38" s="7" t="inlineStr">
         <is>
-          <t>This is capacity, not capability. You know how to do the work and you can't get enough hours of it out the door.</t>
-        </is>
-      </c>
-      <c r="D38" s="7" t="inlineStr"/>
-      <c r="E38" s="8" t="inlineStr"/>
+          <t>you're running {q16.band}</t>
+        </is>
+      </c>
+      <c r="D38" s="7" t="inlineStr">
+        <is>
+          <t>you're running at {q16.exact}% booked</t>
+        </is>
+      </c>
+      <c r="E38" s="8" t="inlineStr">
+        <is>
+          <t>{q16.band}, {q16.exact}</t>
+        </is>
+      </c>
     </row>
     <row r="39">
       <c r="A39" s="6" t="inlineStr">
@@ -16297,22 +16301,18 @@
       </c>
       <c r="B39" s="6" t="inlineStr">
         <is>
-          <t>Evidence clause 1</t>
+          <t>Evidence clause 2</t>
         </is>
       </c>
       <c r="C39" s="7" t="inlineStr">
         <is>
-          <t>you're running {q16.band}</t>
-        </is>
-      </c>
-      <c r="D39" s="7" t="inlineStr">
-        <is>
-          <t>you're running at {q16.exact}% booked</t>
-        </is>
-      </c>
+          <t>{q17.band}</t>
+        </is>
+      </c>
+      <c r="D39" s="7" t="inlineStr"/>
       <c r="E39" s="8" t="inlineStr">
         <is>
-          <t>{q16.band}, {q16.exact}</t>
+          <t>{q17.band}</t>
         </is>
       </c>
     </row>
@@ -16324,18 +16324,18 @@
       </c>
       <c r="B40" s="6" t="inlineStr">
         <is>
-          <t>Evidence clause 2</t>
+          <t>Evidence clause 3</t>
         </is>
       </c>
       <c r="C40" s="7" t="inlineStr">
         <is>
-          <t>{q17.band}</t>
+          <t>lead times have {q18.band}</t>
         </is>
       </c>
       <c r="D40" s="7" t="inlineStr"/>
       <c r="E40" s="8" t="inlineStr">
         <is>
-          <t>{q17.band}</t>
+          <t>{q18.band}</t>
         </is>
       </c>
     </row>
@@ -16347,18 +16347,18 @@
       </c>
       <c r="B41" s="6" t="inlineStr">
         <is>
-          <t>Evidence clause 3</t>
+          <t>Evidence clause 4</t>
         </is>
       </c>
       <c r="C41" s="7" t="inlineStr">
         <is>
-          <t>lead times have {q18.band}</t>
+          <t>a typical job is ready {q19.band}</t>
         </is>
       </c>
       <c r="D41" s="7" t="inlineStr"/>
       <c r="E41" s="8" t="inlineStr">
         <is>
-          <t>{q18.band}</t>
+          <t>{q19.band}</t>
         </is>
       </c>
     </row>
@@ -16370,20 +16370,16 @@
       </c>
       <c r="B42" s="6" t="inlineStr">
         <is>
-          <t>Evidence clause 4</t>
+          <t>Closing</t>
         </is>
       </c>
       <c r="C42" s="7" t="inlineStr">
         <is>
-          <t>a typical job is ready {q19.band}</t>
+          <t>Nothing at the front of the business needs attention until the back of it can breathe. Anything you do to bring in more work right now gets paid for by the customers you already have.</t>
         </is>
       </c>
       <c r="D42" s="7" t="inlineStr"/>
-      <c r="E42" s="8" t="inlineStr">
-        <is>
-          <t>{q19.band}</t>
-        </is>
-      </c>
+      <c r="E42" s="8" t="inlineStr"/>
     </row>
     <row r="43">
       <c r="A43" s="6" t="inlineStr">
@@ -16393,12 +16389,12 @@
       </c>
       <c r="B43" s="6" t="inlineStr">
         <is>
-          <t>Closing</t>
+          <t>Fix, lead line</t>
         </is>
       </c>
       <c r="C43" s="7" t="inlineStr">
         <is>
-          <t>Nothing at the front of the business needs attention until the back of it can breathe. Anything you do to bring in more work right now gets paid for by the customers you already have.</t>
+          <t>Make what you already have work properly, cut what isn't earning its capacity, then hire. In that order.</t>
         </is>
       </c>
       <c r="D43" s="7" t="inlineStr"/>
@@ -16412,16 +16408,20 @@
       </c>
       <c r="B44" s="6" t="inlineStr">
         <is>
-          <t>Fix, lead line</t>
+          <t>Fix action 1</t>
         </is>
       </c>
       <c r="C44" s="7" t="inlineStr">
         <is>
-          <t>You need more output from what you already have, or more capacity, before you go and win any more work.</t>
+          <t>Find the one step everything stalls at, and put the next day into streamlining that one step.</t>
         </is>
       </c>
       <c r="D44" s="7" t="inlineStr"/>
-      <c r="E44" s="8" t="inlineStr"/>
+      <c r="E44" s="8" t="inlineStr">
+        <is>
+          <t>always prints</t>
+        </is>
+      </c>
     </row>
     <row r="45">
       <c r="A45" s="6" t="inlineStr">
@@ -16431,18 +16431,18 @@
       </c>
       <c r="B45" s="6" t="inlineStr">
         <is>
-          <t>Fix action 1</t>
+          <t>Fix action 2</t>
         </is>
       </c>
       <c r="C45" s="7" t="inlineStr">
         <is>
-          <t>Find the one step everything queues behind, then put your next hour into that step and nothing else.</t>
+          <t>Write the five things that go wrong most often into one page checklists. Undocumented work is slow work.</t>
         </is>
       </c>
       <c r="D45" s="7" t="inlineStr"/>
       <c r="E45" s="8" t="inlineStr">
         <is>
-          <t>always prints</t>
+          <t>q46 is b/c/z</t>
         </is>
       </c>
     </row>
@@ -16454,18 +16454,18 @@
       </c>
       <c r="B46" s="6" t="inlineStr">
         <is>
-          <t>Fix action 2</t>
+          <t>Fix action 3</t>
         </is>
       </c>
       <c r="C46" s="7" t="inlineStr">
         <is>
-          <t>Write the five things that go wrong most often into one page checklists. Undocumented work is slow work.</t>
+          <t>Look at what your best people actually spent last week on. Anything that didn't need them is capacity you already have.</t>
         </is>
       </c>
       <c r="D46" s="7" t="inlineStr"/>
       <c r="E46" s="8" t="inlineStr">
         <is>
-          <t>q46 is b/c/z</t>
+          <t>always prints</t>
         </is>
       </c>
     </row>
@@ -16477,12 +16477,12 @@
       </c>
       <c r="B47" s="6" t="inlineStr">
         <is>
-          <t>Fix action 3</t>
+          <t>Fix action 4</t>
         </is>
       </c>
       <c r="C47" s="7" t="inlineStr">
         <is>
-          <t>Look at what your best people actually spent last week on. Anything that didn't need them is capacity you already have.</t>
+          <t>Cut the jobs that eat the most capacity for the least return.</t>
         </is>
       </c>
       <c r="D47" s="7" t="inlineStr"/>
@@ -16500,66 +16500,58 @@
       </c>
       <c r="B48" s="6" t="inlineStr">
         <is>
-          <t>Fix action 4</t>
+          <t>Fix action 5</t>
         </is>
       </c>
       <c r="C48" s="7" t="inlineStr">
         <is>
-          <t>Quote the lead time you actually deliver rather than the one you hope for. A blown promise costs a customer you'd already won.</t>
+          <t>Then hire more capacity into the roles that need it.</t>
         </is>
       </c>
       <c r="D48" s="7" t="inlineStr"/>
       <c r="E48" s="8" t="inlineStr">
         <is>
-          <t>q19 is c/d</t>
+          <t>always prints</t>
         </is>
       </c>
     </row>
     <row r="49">
       <c r="A49" s="6" t="inlineStr">
         <is>
-          <t>fulfilment</t>
+          <t>value</t>
         </is>
       </c>
       <c r="B49" s="6" t="inlineStr">
         <is>
-          <t>Fix action 5</t>
+          <t>Title</t>
         </is>
       </c>
       <c r="C49" s="7" t="inlineStr">
         <is>
-          <t>Work out which jobs eat the most capacity for the least return, and stop taking those until the queue clears.</t>
+          <t>You are {c} constrained</t>
         </is>
       </c>
       <c r="D49" s="7" t="inlineStr"/>
-      <c r="E49" s="8" t="inlineStr">
-        <is>
-          <t>always prints</t>
-        </is>
-      </c>
+      <c r="E49" s="8" t="inlineStr"/>
     </row>
     <row r="50">
       <c r="A50" s="6" t="inlineStr">
         <is>
-          <t>fulfilment</t>
+          <t>value</t>
         </is>
       </c>
       <c r="B50" s="6" t="inlineStr">
         <is>
-          <t>Fix action 6</t>
+          <t>Title, nothing failing</t>
         </is>
       </c>
       <c r="C50" s="7" t="inlineStr">
         <is>
-          <t>Add capacity last, once the steps above have been worked. Hiring multiplies whatever the process already does.</t>
+          <t>The tightest thing is {c}</t>
         </is>
       </c>
       <c r="D50" s="7" t="inlineStr"/>
-      <c r="E50" s="8" t="inlineStr">
-        <is>
-          <t>always prints</t>
-        </is>
-      </c>
+      <c r="E50" s="8" t="inlineStr"/>
     </row>
     <row r="51">
       <c r="A51" s="6" t="inlineStr">
@@ -16569,12 +16561,12 @@
       </c>
       <c r="B51" s="6" t="inlineStr">
         <is>
-          <t>Title</t>
+          <t>Opening</t>
         </is>
       </c>
       <c r="C51" s="7" t="inlineStr">
         <is>
-          <t>You are {c} constrained</t>
+          <t>Value here means what the customer perceives, and it has nothing to do with your pricing or your margin. They buy, then they either stop or start giving most of the work to somebody else.</t>
         </is>
       </c>
       <c r="D51" s="7" t="inlineStr"/>
@@ -16588,16 +16580,24 @@
       </c>
       <c r="B52" s="6" t="inlineStr">
         <is>
-          <t>Title, nothing failing</t>
+          <t>Evidence clause 1</t>
         </is>
       </c>
       <c r="C52" s="7" t="inlineStr">
         <is>
-          <t>The tightest thing is {c}</t>
-        </is>
-      </c>
-      <c r="D52" s="7" t="inlineStr"/>
-      <c r="E52" s="8" t="inlineStr"/>
+          <t>of the customers you had a year ago, {q21.band} still buy from you</t>
+        </is>
+      </c>
+      <c r="D52" s="7" t="inlineStr">
+        <is>
+          <t>of the customers you had a year ago, {q21.exact}% still buy from you</t>
+        </is>
+      </c>
+      <c r="E52" s="8" t="inlineStr">
+        <is>
+          <t>{q21.band}, {q21.exact}</t>
+        </is>
+      </c>
     </row>
     <row r="53">
       <c r="A53" s="6" t="inlineStr">
@@ -16607,16 +16607,24 @@
       </c>
       <c r="B53" s="6" t="inlineStr">
         <is>
-          <t>Opening</t>
+          <t>Evidence clause 2</t>
         </is>
       </c>
       <c r="C53" s="7" t="inlineStr">
         <is>
-          <t>Value here means what the customer perceives, and it has nothing to do with your pricing or your margin. They buy, then they either stop or start giving most of the work to somebody else.</t>
-        </is>
-      </c>
-      <c r="D53" s="7" t="inlineStr"/>
-      <c r="E53" s="8" t="inlineStr"/>
+          <t>you get {q57.band} of the work they put out</t>
+        </is>
+      </c>
+      <c r="D53" s="7" t="inlineStr">
+        <is>
+          <t>you get {q57.exact}% of the work they put out</t>
+        </is>
+      </c>
+      <c r="E53" s="8" t="inlineStr">
+        <is>
+          <t>{q57.band}, {q57.exact}</t>
+        </is>
+      </c>
     </row>
     <row r="54">
       <c r="A54" s="6" t="inlineStr">
@@ -16626,22 +16634,18 @@
       </c>
       <c r="B54" s="6" t="inlineStr">
         <is>
-          <t>Evidence clause 1</t>
+          <t>Evidence clause 3</t>
         </is>
       </c>
       <c r="C54" s="7" t="inlineStr">
         <is>
-          <t>of the customers you had a year ago, {q21.band} still buy from you</t>
-        </is>
-      </c>
-      <c r="D54" s="7" t="inlineStr">
-        <is>
-          <t>of the customers you had a year ago, {q21.exact}% still buy from you</t>
-        </is>
-      </c>
+          <t>they come back unprompted {q22.band}</t>
+        </is>
+      </c>
+      <c r="D54" s="7" t="inlineStr"/>
       <c r="E54" s="8" t="inlineStr">
         <is>
-          <t>{q21.band}, {q21.exact}</t>
+          <t>{q22.band}</t>
         </is>
       </c>
     </row>
@@ -16653,22 +16657,18 @@
       </c>
       <c r="B55" s="6" t="inlineStr">
         <is>
-          <t>Evidence clause 2</t>
+          <t>Evidence clause 4</t>
         </is>
       </c>
       <c r="C55" s="7" t="inlineStr">
         <is>
-          <t>you get {q57.band} of the work they put out</t>
-        </is>
-      </c>
-      <c r="D55" s="7" t="inlineStr">
-        <is>
-          <t>you get {q57.exact}% of the work they put out</t>
-        </is>
-      </c>
+          <t>referrals bring in {q23.band} of your new customers</t>
+        </is>
+      </c>
+      <c r="D55" s="7" t="inlineStr"/>
       <c r="E55" s="8" t="inlineStr">
         <is>
-          <t>{q57.band}, {q57.exact}</t>
+          <t>{q23.band}</t>
         </is>
       </c>
     </row>
@@ -16680,20 +16680,16 @@
       </c>
       <c r="B56" s="6" t="inlineStr">
         <is>
-          <t>Evidence clause 3</t>
+          <t>Closing</t>
         </is>
       </c>
       <c r="C56" s="7" t="inlineStr">
         <is>
-          <t>they come back unprompted {q22.band}</t>
+          <t>You're filling a leaky bucket. Every dollar going into finding new customers is currently paying to replace the ones walking out the other side, which is why the business feels busy and stays the same size.</t>
         </is>
       </c>
       <c r="D56" s="7" t="inlineStr"/>
-      <c r="E56" s="8" t="inlineStr">
-        <is>
-          <t>{q22.band}</t>
-        </is>
-      </c>
+      <c r="E56" s="8" t="inlineStr"/>
     </row>
     <row r="57">
       <c r="A57" s="6" t="inlineStr">
@@ -16703,20 +16699,16 @@
       </c>
       <c r="B57" s="6" t="inlineStr">
         <is>
-          <t>Evidence clause 4</t>
+          <t>Fix, lead line</t>
         </is>
       </c>
       <c r="C57" s="7" t="inlineStr">
         <is>
-          <t>referrals bring in {q23.band} of your new customers</t>
+          <t>You need to find out why customers leave or shrink, and fix that, before you spend another dollar finding new ones.</t>
         </is>
       </c>
       <c r="D57" s="7" t="inlineStr"/>
-      <c r="E57" s="8" t="inlineStr">
-        <is>
-          <t>{q23.band}</t>
-        </is>
-      </c>
+      <c r="E57" s="8" t="inlineStr"/>
     </row>
     <row r="58">
       <c r="A58" s="6" t="inlineStr">
@@ -16726,16 +16718,20 @@
       </c>
       <c r="B58" s="6" t="inlineStr">
         <is>
-          <t>Closing</t>
+          <t>Fix action 1</t>
         </is>
       </c>
       <c r="C58" s="7" t="inlineStr">
         <is>
-          <t>You're filling a leaky bucket. Every dollar going into finding new customers is currently paying to replace the ones walking out the other side, which is why the business feels busy and stays the same size.</t>
+          <t>Ring ten customers who stopped buying or cut back, and ask them straight. Not a survey. A phone call.</t>
         </is>
       </c>
       <c r="D58" s="7" t="inlineStr"/>
-      <c r="E58" s="8" t="inlineStr"/>
+      <c r="E58" s="8" t="inlineStr">
+        <is>
+          <t>always prints</t>
+        </is>
+      </c>
     </row>
     <row r="59">
       <c r="A59" s="6" t="inlineStr">
@@ -16745,16 +16741,20 @@
       </c>
       <c r="B59" s="6" t="inlineStr">
         <is>
-          <t>Fix, lead line</t>
+          <t>Fix action 2</t>
         </is>
       </c>
       <c r="C59" s="7" t="inlineStr">
         <is>
-          <t>You need to find out why customers leave or shrink, and fix that, before you spend another dollar finding new ones.</t>
+          <t>Ask your biggest customers what they give to somebody else, and why. That work already exists, you're just not getting it.</t>
         </is>
       </c>
       <c r="D59" s="7" t="inlineStr"/>
-      <c r="E59" s="8" t="inlineStr"/>
+      <c r="E59" s="8" t="inlineStr">
+        <is>
+          <t>q57 is c/d/e</t>
+        </is>
+      </c>
     </row>
     <row r="60">
       <c r="A60" s="6" t="inlineStr">
@@ -16764,12 +16764,12 @@
       </c>
       <c r="B60" s="6" t="inlineStr">
         <is>
-          <t>Fix action 1</t>
+          <t>Fix action 3</t>
         </is>
       </c>
       <c r="C60" s="7" t="inlineStr">
         <is>
-          <t>Ring ten customers who stopped buying or cut back, and ask them straight. Not a survey. A phone call.</t>
+          <t>Look hard at what happens in the first thirty days after somebody buys. That's the part of the experience you control most tightly.</t>
         </is>
       </c>
       <c r="D60" s="7" t="inlineStr"/>
@@ -16787,18 +16787,18 @@
       </c>
       <c r="B61" s="6" t="inlineStr">
         <is>
-          <t>Fix action 2</t>
+          <t>Fix action 4</t>
         </is>
       </c>
       <c r="C61" s="7" t="inlineStr">
         <is>
-          <t>Ask your biggest customers what they give to somebody else, and why. That work already exists, you're just not getting it.</t>
+          <t>Build one reason to come back that you initiate. A check in, or the next step offered before they go looking.</t>
         </is>
       </c>
       <c r="D61" s="7" t="inlineStr"/>
       <c r="E61" s="8" t="inlineStr">
         <is>
-          <t>q57 is c/d/e</t>
+          <t>always prints</t>
         </is>
       </c>
     </row>
@@ -16810,12 +16810,12 @@
       </c>
       <c r="B62" s="6" t="inlineStr">
         <is>
-          <t>Fix action 3</t>
+          <t>Fix action 5</t>
         </is>
       </c>
       <c r="C62" s="7" t="inlineStr">
         <is>
-          <t>Look hard at what happens in the first thirty days after somebody buys. That's the part of the experience you control most tightly.</t>
+          <t>Measure retention monthly, so a drop shows up while you can still do something about it.</t>
         </is>
       </c>
       <c r="D62" s="7" t="inlineStr"/>
@@ -16828,48 +16828,40 @@
     <row r="63">
       <c r="A63" s="6" t="inlineStr">
         <is>
-          <t>value</t>
+          <t>offer</t>
         </is>
       </c>
       <c r="B63" s="6" t="inlineStr">
         <is>
-          <t>Fix action 4</t>
+          <t>Title</t>
         </is>
       </c>
       <c r="C63" s="7" t="inlineStr">
         <is>
-          <t>Build one reason to come back that you initiate. A check in, or the next step offered before they go looking.</t>
+          <t>You are {c} constrained</t>
         </is>
       </c>
       <c r="D63" s="7" t="inlineStr"/>
-      <c r="E63" s="8" t="inlineStr">
-        <is>
-          <t>always prints</t>
-        </is>
-      </c>
+      <c r="E63" s="8" t="inlineStr"/>
     </row>
     <row r="64">
       <c r="A64" s="6" t="inlineStr">
         <is>
-          <t>value</t>
+          <t>offer</t>
         </is>
       </c>
       <c r="B64" s="6" t="inlineStr">
         <is>
-          <t>Fix action 5</t>
+          <t>Title, nothing failing</t>
         </is>
       </c>
       <c r="C64" s="7" t="inlineStr">
         <is>
-          <t>Measure retention monthly, so a drop shows up while you can still do something about it.</t>
+          <t>The tightest thing is {c}</t>
         </is>
       </c>
       <c r="D64" s="7" t="inlineStr"/>
-      <c r="E64" s="8" t="inlineStr">
-        <is>
-          <t>always prints</t>
-        </is>
-      </c>
+      <c r="E64" s="8" t="inlineStr"/>
     </row>
     <row r="65">
       <c r="A65" s="6" t="inlineStr">
@@ -16879,12 +16871,12 @@
       </c>
       <c r="B65" s="6" t="inlineStr">
         <is>
-          <t>Title</t>
+          <t>Opening sentence 1</t>
         </is>
       </c>
       <c r="C65" s="7" t="inlineStr">
         <is>
-          <t>You are {c} constrained</t>
+          <t>Enquiries arrive and they don't convert.</t>
         </is>
       </c>
       <c r="D65" s="7" t="inlineStr"/>
@@ -16898,12 +16890,12 @@
       </c>
       <c r="B66" s="6" t="inlineStr">
         <is>
-          <t>Title, nothing failing</t>
+          <t>Opening sentence 2</t>
         </is>
       </c>
       <c r="C66" s="7" t="inlineStr">
         <is>
-          <t>The tightest thing is {c}</t>
+          <t>That isn't a sales technique problem, it's what's on the table. Either the value in the offer doesn't justify the price you're asking, or there's something in the way of somebody saying yes.</t>
         </is>
       </c>
       <c r="D66" s="7" t="inlineStr"/>
@@ -16917,16 +16909,24 @@
       </c>
       <c r="B67" s="6" t="inlineStr">
         <is>
-          <t>Opening sentence 1</t>
+          <t>Evidence clause 1</t>
         </is>
       </c>
       <c r="C67" s="7" t="inlineStr">
         <is>
-          <t>Enquiries arrive and they don't convert.</t>
-        </is>
-      </c>
-      <c r="D67" s="7" t="inlineStr"/>
-      <c r="E67" s="8" t="inlineStr"/>
+          <t>your close rate sits {q26.band}</t>
+        </is>
+      </c>
+      <c r="D67" s="7" t="inlineStr">
+        <is>
+          <t>your close rate sits at {q26.exact}%</t>
+        </is>
+      </c>
+      <c r="E67" s="8" t="inlineStr">
+        <is>
+          <t>{q26.band}, {q26.exact}</t>
+        </is>
+      </c>
     </row>
     <row r="68">
       <c r="A68" s="6" t="inlineStr">
@@ -16936,16 +16936,20 @@
       </c>
       <c r="B68" s="6" t="inlineStr">
         <is>
-          <t>Opening sentence 2</t>
+          <t>Evidence clause 2</t>
         </is>
       </c>
       <c r="C68" s="7" t="inlineStr">
         <is>
-          <t>That isn't a sales technique problem, it's what's on the table. Either the value in the offer doesn't justify the price you're asking, or there's something in the way of somebody saying yes.</t>
+          <t>the most common reason you lose is {q27.band}</t>
         </is>
       </c>
       <c r="D68" s="7" t="inlineStr"/>
-      <c r="E68" s="8" t="inlineStr"/>
+      <c r="E68" s="8" t="inlineStr">
+        <is>
+          <t>{q27.band}</t>
+        </is>
+      </c>
     </row>
     <row r="69">
       <c r="A69" s="6" t="inlineStr">
@@ -16955,22 +16959,18 @@
       </c>
       <c r="B69" s="6" t="inlineStr">
         <is>
-          <t>Evidence clause 1</t>
+          <t>Evidence clause 3</t>
         </is>
       </c>
       <c r="C69" s="7" t="inlineStr">
         <is>
-          <t>your close rate sits {q26.band}</t>
-        </is>
-      </c>
-      <c r="D69" s="7" t="inlineStr">
-        <is>
-          <t>your close rate sits at {q26.exact}%</t>
-        </is>
-      </c>
+          <t>prospects come back on your quote asking what's included {q28.band}</t>
+        </is>
+      </c>
+      <c r="D69" s="7" t="inlineStr"/>
       <c r="E69" s="8" t="inlineStr">
         <is>
-          <t>{q26.band}, {q26.exact}</t>
+          <t>{q28.band}</t>
         </is>
       </c>
     </row>
@@ -16982,18 +16982,18 @@
       </c>
       <c r="B70" s="6" t="inlineStr">
         <is>
-          <t>Evidence clause 2</t>
+          <t>Evidence clause 4</t>
         </is>
       </c>
       <c r="C70" s="7" t="inlineStr">
         <is>
-          <t>the most common reason you lose is {q27.band}</t>
+          <t>they find out what you charge {q30.band}</t>
         </is>
       </c>
       <c r="D70" s="7" t="inlineStr"/>
       <c r="E70" s="8" t="inlineStr">
         <is>
-          <t>{q27.band}</t>
+          <t>{q30.band}</t>
         </is>
       </c>
     </row>
@@ -17005,20 +17005,16 @@
       </c>
       <c r="B71" s="6" t="inlineStr">
         <is>
-          <t>Evidence clause 3</t>
+          <t>Closing</t>
         </is>
       </c>
       <c r="C71" s="7" t="inlineStr">
         <is>
-          <t>prospects come back on your quote asking what's included {q28.band}</t>
+          <t>You don't fix this by dropping the price. You fix it by putting things into the offer that cost you very little and are worth real money to the buyer, and by removing whatever a prospect has to get over before they can say yes.</t>
         </is>
       </c>
       <c r="D71" s="7" t="inlineStr"/>
-      <c r="E71" s="8" t="inlineStr">
-        <is>
-          <t>{q28.band}</t>
-        </is>
-      </c>
+      <c r="E71" s="8" t="inlineStr"/>
     </row>
     <row r="72">
       <c r="A72" s="6" t="inlineStr">
@@ -17028,20 +17024,16 @@
       </c>
       <c r="B72" s="6" t="inlineStr">
         <is>
-          <t>Evidence clause 4</t>
+          <t>Fix, lead line</t>
         </is>
       </c>
       <c r="C72" s="7" t="inlineStr">
         <is>
-          <t>they find out what you charge {q30.band}</t>
+          <t>You need more value in the offer than the price is asking for, and the hurdles taken out of the way of somebody saying yes.</t>
         </is>
       </c>
       <c r="D72" s="7" t="inlineStr"/>
-      <c r="E72" s="8" t="inlineStr">
-        <is>
-          <t>{q30.band}</t>
-        </is>
-      </c>
+      <c r="E72" s="8" t="inlineStr"/>
     </row>
     <row r="73">
       <c r="A73" s="6" t="inlineStr">
@@ -17051,16 +17043,20 @@
       </c>
       <c r="B73" s="6" t="inlineStr">
         <is>
-          <t>Closing</t>
+          <t>Fix action 1</t>
         </is>
       </c>
       <c r="C73" s="7" t="inlineStr">
         <is>
-          <t>You don't fix this by dropping the price. You fix it by putting things into the offer that cost you very little and are worth real money to the buyer, and by removing whatever a prospect has to get over before they can say yes.</t>
+          <t>List everything you already do for a customer that isn't written into the offer. That's value nobody can see.</t>
         </is>
       </c>
       <c r="D73" s="7" t="inlineStr"/>
-      <c r="E73" s="8" t="inlineStr"/>
+      <c r="E73" s="8" t="inlineStr">
+        <is>
+          <t>always prints</t>
+        </is>
+      </c>
     </row>
     <row r="74">
       <c r="A74" s="6" t="inlineStr">
@@ -17070,16 +17066,20 @@
       </c>
       <c r="B74" s="6" t="inlineStr">
         <is>
-          <t>Fix, lead line</t>
+          <t>Fix action 2</t>
         </is>
       </c>
       <c r="C74" s="7" t="inlineStr">
         <is>
-          <t>You need more value in the offer than the price is asking for, and the hurdles taken out of the way of somebody saying yes.</t>
+          <t>Add two things that cost you close to nothing and are worth real money to the buyer. A guarantee, or something they would otherwise have to go and source themselves.</t>
         </is>
       </c>
       <c r="D74" s="7" t="inlineStr"/>
-      <c r="E74" s="8" t="inlineStr"/>
+      <c r="E74" s="8" t="inlineStr">
+        <is>
+          <t>always prints</t>
+        </is>
+      </c>
     </row>
     <row r="75">
       <c r="A75" s="6" t="inlineStr">
@@ -17089,18 +17089,18 @@
       </c>
       <c r="B75" s="6" t="inlineStr">
         <is>
-          <t>Fix action 1</t>
+          <t>Fix action 3</t>
         </is>
       </c>
       <c r="C75" s="7" t="inlineStr">
         <is>
-          <t>List everything you already do for a customer that isn't written into the offer. That's value nobody can see.</t>
+          <t>Write down every question a prospect asks after they get the quote, then answer all of them inside the quote itself.</t>
         </is>
       </c>
       <c r="D75" s="7" t="inlineStr"/>
       <c r="E75" s="8" t="inlineStr">
         <is>
-          <t>always prints</t>
+          <t>q28 is c/d</t>
         </is>
       </c>
     </row>
@@ -17112,18 +17112,18 @@
       </c>
       <c r="B76" s="6" t="inlineStr">
         <is>
-          <t>Fix action 2</t>
+          <t>Fix action 4</t>
         </is>
       </c>
       <c r="C76" s="7" t="inlineStr">
         <is>
-          <t>Add two things that cost you close to nothing and are worth real money to the buyer. A guarantee, or something they would otherwise have to go and source themselves.</t>
+          <t>Put a price or a range where they can see it. Making somebody wait for a number is a hurdle before they have even decided.</t>
         </is>
       </c>
       <c r="D76" s="7" t="inlineStr"/>
       <c r="E76" s="8" t="inlineStr">
         <is>
-          <t>always prints</t>
+          <t>q30 is c/d</t>
         </is>
       </c>
     </row>
@@ -17135,18 +17135,18 @@
       </c>
       <c r="B77" s="6" t="inlineStr">
         <is>
-          <t>Fix action 3</t>
+          <t>Fix action 5</t>
         </is>
       </c>
       <c r="C77" s="7" t="inlineStr">
         <is>
-          <t>Write down every question a prospect asks after they get the quote, then answer all of them inside the quote itself.</t>
+          <t>Sort your last twenty losses by reason and count them. If price keeps coming up, look at the value in the offer before you look at the number.</t>
         </is>
       </c>
       <c r="D77" s="7" t="inlineStr"/>
       <c r="E77" s="8" t="inlineStr">
         <is>
-          <t>q28 is c/d</t>
+          <t>always prints</t>
         </is>
       </c>
     </row>
@@ -17158,66 +17158,58 @@
       </c>
       <c r="B78" s="6" t="inlineStr">
         <is>
-          <t>Fix action 4</t>
+          <t>Fix action 6</t>
         </is>
       </c>
       <c r="C78" s="7" t="inlineStr">
         <is>
-          <t>Put a price or a range where they can see it. Making somebody wait for a number is a hurdle before they have even decided.</t>
+          <t>Test the new offer on the next ten enquiries before you change anything else.</t>
         </is>
       </c>
       <c r="D78" s="7" t="inlineStr"/>
       <c r="E78" s="8" t="inlineStr">
         <is>
-          <t>q30 is c/d</t>
+          <t>always prints</t>
         </is>
       </c>
     </row>
     <row r="79">
       <c r="A79" s="6" t="inlineStr">
         <is>
-          <t>offer</t>
+          <t>demand</t>
         </is>
       </c>
       <c r="B79" s="6" t="inlineStr">
         <is>
-          <t>Fix action 5</t>
+          <t>Title</t>
         </is>
       </c>
       <c r="C79" s="7" t="inlineStr">
         <is>
-          <t>Sort your last twenty losses by reason and count them. If price keeps coming up, look at the value in the offer before you look at the number.</t>
+          <t>You are {c} constrained</t>
         </is>
       </c>
       <c r="D79" s="7" t="inlineStr"/>
-      <c r="E79" s="8" t="inlineStr">
-        <is>
-          <t>always prints</t>
-        </is>
-      </c>
+      <c r="E79" s="8" t="inlineStr"/>
     </row>
     <row r="80">
       <c r="A80" s="6" t="inlineStr">
         <is>
-          <t>offer</t>
+          <t>demand</t>
         </is>
       </c>
       <c r="B80" s="6" t="inlineStr">
         <is>
-          <t>Fix action 6</t>
+          <t>Title, nothing failing</t>
         </is>
       </c>
       <c r="C80" s="7" t="inlineStr">
         <is>
-          <t>Test the new offer on the next ten enquiries before you change anything else.</t>
+          <t>The tightest thing is {c}</t>
         </is>
       </c>
       <c r="D80" s="7" t="inlineStr"/>
-      <c r="E80" s="8" t="inlineStr">
-        <is>
-          <t>always prints</t>
-        </is>
-      </c>
+      <c r="E80" s="8" t="inlineStr"/>
     </row>
     <row r="81">
       <c r="A81" s="6" t="inlineStr">
@@ -17227,12 +17219,12 @@
       </c>
       <c r="B81" s="6" t="inlineStr">
         <is>
-          <t>Title</t>
+          <t>Opening</t>
         </is>
       </c>
       <c r="C81" s="7" t="inlineStr">
         <is>
-          <t>You are {c} constrained</t>
+          <t>You've got capacity sitting idle and not enough people asking.</t>
         </is>
       </c>
       <c r="D81" s="7" t="inlineStr"/>
@@ -17246,16 +17238,24 @@
       </c>
       <c r="B82" s="6" t="inlineStr">
         <is>
-          <t>Title, nothing failing</t>
+          <t>Evidence clause 1</t>
         </is>
       </c>
       <c r="C82" s="7" t="inlineStr">
         <is>
-          <t>The tightest thing is {c}</t>
-        </is>
-      </c>
-      <c r="D82" s="7" t="inlineStr"/>
-      <c r="E82" s="8" t="inlineStr"/>
+          <t>enquiries run {q31.band}</t>
+        </is>
+      </c>
+      <c r="D82" s="7" t="inlineStr">
+        <is>
+          <t>enquiries run at about {q31.exact} a month</t>
+        </is>
+      </c>
+      <c r="E82" s="8" t="inlineStr">
+        <is>
+          <t>{q31.band}, {q31.exact}</t>
+        </is>
+      </c>
     </row>
     <row r="83">
       <c r="A83" s="6" t="inlineStr">
@@ -17265,16 +17265,20 @@
       </c>
       <c r="B83" s="6" t="inlineStr">
         <is>
-          <t>Opening</t>
+          <t>Evidence clause 2</t>
         </is>
       </c>
       <c r="C83" s="7" t="inlineStr">
         <is>
-          <t>You've got capacity sitting idle and not enough people asking.</t>
+          <t>volume has {q33.band} over the last year</t>
         </is>
       </c>
       <c r="D83" s="7" t="inlineStr"/>
-      <c r="E83" s="8" t="inlineStr"/>
+      <c r="E83" s="8" t="inlineStr">
+        <is>
+          <t>{q33.band}</t>
+        </is>
+      </c>
     </row>
     <row r="84">
       <c r="A84" s="6" t="inlineStr">
@@ -17284,22 +17288,18 @@
       </c>
       <c r="B84" s="6" t="inlineStr">
         <is>
-          <t>Evidence clause 1</t>
+          <t>Evidence clause 3</t>
         </is>
       </c>
       <c r="C84" s="7" t="inlineStr">
         <is>
-          <t>enquiries run {q31.band}</t>
-        </is>
-      </c>
-      <c r="D84" s="7" t="inlineStr">
-        <is>
-          <t>enquiries run at about {q31.exact} a month</t>
-        </is>
-      </c>
+          <t>{q35.band}</t>
+        </is>
+      </c>
+      <c r="D84" s="7" t="inlineStr"/>
       <c r="E84" s="8" t="inlineStr">
         <is>
-          <t>{q31.band}, {q31.exact}</t>
+          <t>{q35.band}</t>
         </is>
       </c>
     </row>
@@ -17311,20 +17311,16 @@
       </c>
       <c r="B85" s="6" t="inlineStr">
         <is>
-          <t>Evidence clause 2</t>
+          <t>Closing</t>
         </is>
       </c>
       <c r="C85" s="7" t="inlineStr">
         <is>
-          <t>volume has {q33.band} over the last year</t>
+          <t>You could take on more work tomorrow, which is what separates this from a delivery problem. Nothing downstream is broken. The business just isn't being fed, and it won't start feeding itself.</t>
         </is>
       </c>
       <c r="D85" s="7" t="inlineStr"/>
-      <c r="E85" s="8" t="inlineStr">
-        <is>
-          <t>{q33.band}</t>
-        </is>
-      </c>
+      <c r="E85" s="8" t="inlineStr"/>
     </row>
     <row r="86">
       <c r="A86" s="6" t="inlineStr">
@@ -17334,20 +17330,16 @@
       </c>
       <c r="B86" s="6" t="inlineStr">
         <is>
-          <t>Evidence clause 3</t>
+          <t>Fix, lead line</t>
         </is>
       </c>
       <c r="C86" s="7" t="inlineStr">
         <is>
-          <t>{q35.band}</t>
+          <t>You need one lead source running properly and consistently before you go anywhere near a second.</t>
         </is>
       </c>
       <c r="D86" s="7" t="inlineStr"/>
-      <c r="E86" s="8" t="inlineStr">
-        <is>
-          <t>{q35.band}</t>
-        </is>
-      </c>
+      <c r="E86" s="8" t="inlineStr"/>
     </row>
     <row r="87">
       <c r="A87" s="6" t="inlineStr">
@@ -17357,16 +17349,20 @@
       </c>
       <c r="B87" s="6" t="inlineStr">
         <is>
-          <t>Closing</t>
+          <t>Fix action 1</t>
         </is>
       </c>
       <c r="C87" s="7" t="inlineStr">
         <is>
-          <t>You could take on more work tomorrow, which is what separates this from a delivery problem. Nothing downstream is broken. The business just isn't being fed, and it won't start feeding itself.</t>
+          <t>Whatever you're doing to generate enquiries isn't running consistently. Start with the one thing you can do every week without fail.</t>
         </is>
       </c>
       <c r="D87" s="7" t="inlineStr"/>
-      <c r="E87" s="8" t="inlineStr"/>
+      <c r="E87" s="8" t="inlineStr">
+        <is>
+          <t>q35 is b/c</t>
+        </is>
+      </c>
     </row>
     <row r="88">
       <c r="A88" s="6" t="inlineStr">
@@ -17376,16 +17372,20 @@
       </c>
       <c r="B88" s="6" t="inlineStr">
         <is>
-          <t>Fix, lead line</t>
+          <t>Fix action 2</t>
         </is>
       </c>
       <c r="C88" s="7" t="inlineStr">
         <is>
-          <t>You need one lead source running properly and consistently before you go anywhere near a second.</t>
+          <t>Pick the lead source that already brings your best customers and put real weight behind it.</t>
         </is>
       </c>
       <c r="D88" s="7" t="inlineStr"/>
-      <c r="E88" s="8" t="inlineStr"/>
+      <c r="E88" s="8" t="inlineStr">
+        <is>
+          <t>always prints</t>
+        </is>
+      </c>
     </row>
     <row r="89">
       <c r="A89" s="6" t="inlineStr">
@@ -17395,18 +17395,18 @@
       </c>
       <c r="B89" s="6" t="inlineStr">
         <is>
-          <t>Fix action 1</t>
+          <t>Fix action 3</t>
         </is>
       </c>
       <c r="C89" s="7" t="inlineStr">
         <is>
-          <t>Whatever you're doing to generate enquiries isn't running consistently. Start with the one thing you can do every week without fail.</t>
+          <t>Go and ask for work. Outbound to the twenty businesses you'd most like to work with beats waiting on referrals.</t>
         </is>
       </c>
       <c r="D89" s="7" t="inlineStr"/>
       <c r="E89" s="8" t="inlineStr">
         <is>
-          <t>q35 is b/c</t>
+          <t>always prints</t>
         </is>
       </c>
     </row>
@@ -17418,18 +17418,18 @@
       </c>
       <c r="B90" s="6" t="inlineStr">
         <is>
-          <t>Fix action 2</t>
+          <t>Fix action 4</t>
         </is>
       </c>
       <c r="C90" s="7" t="inlineStr">
         <is>
-          <t>Pick the lead source that already brings your best customers and put real weight behind it.</t>
+          <t>Everything arrives through one lead source. Stand up a second before that one changes.</t>
         </is>
       </c>
       <c r="D90" s="7" t="inlineStr"/>
       <c r="E90" s="8" t="inlineStr">
         <is>
-          <t>always prints</t>
+          <t>q43 is c</t>
         </is>
       </c>
     </row>
@@ -17441,12 +17441,12 @@
       </c>
       <c r="B91" s="6" t="inlineStr">
         <is>
-          <t>Fix action 3</t>
+          <t>Fix action 5</t>
         </is>
       </c>
       <c r="C91" s="7" t="inlineStr">
         <is>
-          <t>Go and ask for work. Outbound to the twenty businesses you'd most like to work with beats waiting on referrals.</t>
+          <t>Ask every happy customer for one introduction.</t>
         </is>
       </c>
       <c r="D91" s="7" t="inlineStr"/>
@@ -17464,66 +17464,58 @@
       </c>
       <c r="B92" s="6" t="inlineStr">
         <is>
-          <t>Fix action 4</t>
+          <t>Fix action 6</t>
         </is>
       </c>
       <c r="C92" s="7" t="inlineStr">
         <is>
-          <t>Everything arrives through one lead source. Stand up a second before that one changes.</t>
+          <t>Give a lead source ninety days before you judge it. Anything shorter is guesswork.</t>
         </is>
       </c>
       <c r="D92" s="7" t="inlineStr"/>
       <c r="E92" s="8" t="inlineStr">
         <is>
-          <t>q43 is c</t>
+          <t>always prints</t>
         </is>
       </c>
     </row>
     <row r="93">
       <c r="A93" s="6" t="inlineStr">
         <is>
-          <t>demand</t>
+          <t>margin</t>
         </is>
       </c>
       <c r="B93" s="6" t="inlineStr">
         <is>
-          <t>Fix action 5</t>
+          <t>Title</t>
         </is>
       </c>
       <c r="C93" s="7" t="inlineStr">
         <is>
-          <t>Ask every happy customer for one introduction.</t>
+          <t>You are {c} constrained</t>
         </is>
       </c>
       <c r="D93" s="7" t="inlineStr"/>
-      <c r="E93" s="8" t="inlineStr">
-        <is>
-          <t>always prints</t>
-        </is>
-      </c>
+      <c r="E93" s="8" t="inlineStr"/>
     </row>
     <row r="94">
       <c r="A94" s="6" t="inlineStr">
         <is>
-          <t>demand</t>
+          <t>margin</t>
         </is>
       </c>
       <c r="B94" s="6" t="inlineStr">
         <is>
-          <t>Fix action 6</t>
+          <t>Title, nothing failing</t>
         </is>
       </c>
       <c r="C94" s="7" t="inlineStr">
         <is>
-          <t>Give a lead source ninety days before you judge it. Anything shorter is guesswork.</t>
+          <t>The tightest thing is {c}</t>
         </is>
       </c>
       <c r="D94" s="7" t="inlineStr"/>
-      <c r="E94" s="8" t="inlineStr">
-        <is>
-          <t>always prints</t>
-        </is>
-      </c>
+      <c r="E94" s="8" t="inlineStr"/>
     </row>
     <row r="95">
       <c r="A95" s="6" t="inlineStr">
@@ -17533,12 +17525,12 @@
       </c>
       <c r="B95" s="6" t="inlineStr">
         <is>
-          <t>Title</t>
+          <t>Opening</t>
         </is>
       </c>
       <c r="C95" s="7" t="inlineStr">
         <is>
-          <t>You are {c} constrained</t>
+          <t>You're full and busy, and there's nothing left at the end of it.</t>
         </is>
       </c>
       <c r="D95" s="7" t="inlineStr"/>
@@ -17552,16 +17544,24 @@
       </c>
       <c r="B96" s="6" t="inlineStr">
         <is>
-          <t>Title, nothing failing</t>
+          <t>Evidence clause 1</t>
         </is>
       </c>
       <c r="C96" s="7" t="inlineStr">
         <is>
-          <t>The tightest thing is {c}</t>
-        </is>
-      </c>
-      <c r="D96" s="7" t="inlineStr"/>
-      <c r="E96" s="8" t="inlineStr"/>
+          <t>what's left after direct costs sits {q36.band}</t>
+        </is>
+      </c>
+      <c r="D96" s="7" t="inlineStr">
+        <is>
+          <t>what's left after direct costs sits at {q36.exact}%</t>
+        </is>
+      </c>
+      <c r="E96" s="8" t="inlineStr">
+        <is>
+          <t>{q36.band}, {q36.exact}</t>
+        </is>
+      </c>
     </row>
     <row r="97">
       <c r="A97" s="6" t="inlineStr">
@@ -17571,16 +17571,24 @@
       </c>
       <c r="B97" s="6" t="inlineStr">
         <is>
-          <t>Opening</t>
+          <t>Evidence clause 2</t>
         </is>
       </c>
       <c r="C97" s="7" t="inlineStr">
         <is>
-          <t>You're full and busy, and there's nothing left at the end of it.</t>
-        </is>
-      </c>
-      <c r="D97" s="7" t="inlineStr"/>
-      <c r="E97" s="8" t="inlineStr"/>
+          <t>after everything it's {q37.band}</t>
+        </is>
+      </c>
+      <c r="D97" s="7" t="inlineStr">
+        <is>
+          <t>after everything it's {q37.exact}%</t>
+        </is>
+      </c>
+      <c r="E97" s="8" t="inlineStr">
+        <is>
+          <t>{q37.band}, {q37.exact}</t>
+        </is>
+      </c>
     </row>
     <row r="98">
       <c r="A98" s="6" t="inlineStr">
@@ -17590,22 +17598,18 @@
       </c>
       <c r="B98" s="6" t="inlineStr">
         <is>
-          <t>Evidence clause 1</t>
+          <t>Evidence clause 3</t>
         </is>
       </c>
       <c r="C98" s="7" t="inlineStr">
         <is>
-          <t>what's left after direct costs sits {q36.band}</t>
-        </is>
-      </c>
-      <c r="D98" s="7" t="inlineStr">
-        <is>
-          <t>what's left after direct costs sits at {q36.exact}%</t>
-        </is>
-      </c>
+          <t>{q38.band}</t>
+        </is>
+      </c>
+      <c r="D98" s="7" t="inlineStr"/>
       <c r="E98" s="8" t="inlineStr">
         <is>
-          <t>{q36.band}, {q36.exact}</t>
+          <t>{q38.band}</t>
         </is>
       </c>
     </row>
@@ -17617,22 +17621,18 @@
       </c>
       <c r="B99" s="6" t="inlineStr">
         <is>
-          <t>Evidence clause 2</t>
+          <t>Evidence clause 4</t>
         </is>
       </c>
       <c r="C99" s="7" t="inlineStr">
         <is>
-          <t>after everything it's {q37.band}</t>
-        </is>
-      </c>
-      <c r="D99" s="7" t="inlineStr">
-        <is>
-          <t>after everything it's {q37.exact}%</t>
-        </is>
-      </c>
+          <t>jobs run over what you quoted {q39.band}</t>
+        </is>
+      </c>
+      <c r="D99" s="7" t="inlineStr"/>
       <c r="E99" s="8" t="inlineStr">
         <is>
-          <t>{q37.band}, {q37.exact}</t>
+          <t>{q39.band}</t>
         </is>
       </c>
     </row>
@@ -17644,20 +17644,16 @@
       </c>
       <c r="B100" s="6" t="inlineStr">
         <is>
-          <t>Evidence clause 3</t>
+          <t>Closing</t>
         </is>
       </c>
       <c r="C100" s="7" t="inlineStr">
         <is>
-          <t>{q38.band}</t>
+          <t>Volume won't rescue this. At the margin you're running, more work gets you more of the same result and it arrives faster.</t>
         </is>
       </c>
       <c r="D100" s="7" t="inlineStr"/>
-      <c r="E100" s="8" t="inlineStr">
-        <is>
-          <t>{q38.band}</t>
-        </is>
-      </c>
+      <c r="E100" s="8" t="inlineStr"/>
     </row>
     <row r="101">
       <c r="A101" s="6" t="inlineStr">
@@ -17667,20 +17663,16 @@
       </c>
       <c r="B101" s="6" t="inlineStr">
         <is>
-          <t>Evidence clause 4</t>
+          <t>Fix, lead line</t>
         </is>
       </c>
       <c r="C101" s="7" t="inlineStr">
         <is>
-          <t>jobs run over what you quoted {q39.band}</t>
+          <t>You need to know what each job actually earns you before you change anything. A price rise can cost you customers as easily as it can fix the margin.</t>
         </is>
       </c>
       <c r="D101" s="7" t="inlineStr"/>
-      <c r="E101" s="8" t="inlineStr">
-        <is>
-          <t>{q39.band}</t>
-        </is>
-      </c>
+      <c r="E101" s="8" t="inlineStr"/>
     </row>
     <row r="102">
       <c r="A102" s="6" t="inlineStr">
@@ -17690,16 +17682,20 @@
       </c>
       <c r="B102" s="6" t="inlineStr">
         <is>
-          <t>Closing</t>
+          <t>Fix action 1</t>
         </is>
       </c>
       <c r="C102" s="7" t="inlineStr">
         <is>
-          <t>Volume won't rescue this. At the margin you're running, more work gets you more of the same result and it arrives faster.</t>
+          <t>Raise prices on new work now. Ten percent across the board, and watch what actually happens.</t>
         </is>
       </c>
       <c r="D102" s="7" t="inlineStr"/>
-      <c r="E102" s="8" t="inlineStr"/>
+      <c r="E102" s="8" t="inlineStr">
+        <is>
+          <t>q38 is c/d/e</t>
+        </is>
+      </c>
     </row>
     <row r="103">
       <c r="A103" s="6" t="inlineStr">
@@ -17709,16 +17705,20 @@
       </c>
       <c r="B103" s="6" t="inlineStr">
         <is>
-          <t>Fix, lead line</t>
+          <t>Fix action 2</t>
         </is>
       </c>
       <c r="C103" s="7" t="inlineStr">
         <is>
-          <t>You need to know what each job actually earns you before you change anything. A price rise can cost you customers as easily as it can fix the margin.</t>
+          <t>Work out what each job really costs, your own time included, then rank your last twenty by what was left.</t>
         </is>
       </c>
       <c r="D103" s="7" t="inlineStr"/>
-      <c r="E103" s="8" t="inlineStr"/>
+      <c r="E103" s="8" t="inlineStr">
+        <is>
+          <t>always prints</t>
+        </is>
+      </c>
     </row>
     <row r="104">
       <c r="A104" s="6" t="inlineStr">
@@ -17728,18 +17728,18 @@
       </c>
       <c r="B104" s="6" t="inlineStr">
         <is>
-          <t>Fix action 1</t>
+          <t>Fix action 3</t>
         </is>
       </c>
       <c r="C104" s="7" t="inlineStr">
         <is>
-          <t>Raise prices on new work now. Ten percent across the board, and watch what actually happens.</t>
+          <t>Quote a contingency into the jobs that historically run over. You already know which ones they are.</t>
         </is>
       </c>
       <c r="D104" s="7" t="inlineStr"/>
       <c r="E104" s="8" t="inlineStr">
         <is>
-          <t>q38 is c/d/e</t>
+          <t>q39 is c/d</t>
         </is>
       </c>
     </row>
@@ -17751,12 +17751,12 @@
       </c>
       <c r="B105" s="6" t="inlineStr">
         <is>
-          <t>Fix action 2</t>
+          <t>Fix action 4</t>
         </is>
       </c>
       <c r="C105" s="7" t="inlineStr">
         <is>
-          <t>Work out what each job really costs, your own time included, then rank your last twenty by what was left.</t>
+          <t>Find your worst three customers by margin, then reprice them or let them go.</t>
         </is>
       </c>
       <c r="D105" s="7" t="inlineStr"/>
@@ -17774,69 +17774,23 @@
       </c>
       <c r="B106" s="6" t="inlineStr">
         <is>
-          <t>Fix action 3</t>
+          <t>Fix action 5</t>
         </is>
       </c>
       <c r="C106" s="7" t="inlineStr">
         <is>
-          <t>Quote a contingency into the jobs that historically run over. You already know which ones they are.</t>
+          <t>Don't discount to win. A discount is the fastest way to buy work you'll resent delivering.</t>
         </is>
       </c>
       <c r="D106" s="7" t="inlineStr"/>
       <c r="E106" s="8" t="inlineStr">
         <is>
-          <t>q39 is c/d</t>
-        </is>
-      </c>
-    </row>
-    <row r="107">
-      <c r="A107" s="6" t="inlineStr">
-        <is>
-          <t>margin</t>
-        </is>
-      </c>
-      <c r="B107" s="6" t="inlineStr">
-        <is>
-          <t>Fix action 4</t>
-        </is>
-      </c>
-      <c r="C107" s="7" t="inlineStr">
-        <is>
-          <t>Find your worst three customers by margin, then reprice them or let them go.</t>
-        </is>
-      </c>
-      <c r="D107" s="7" t="inlineStr"/>
-      <c r="E107" s="8" t="inlineStr">
-        <is>
           <t>always prints</t>
         </is>
       </c>
     </row>
-    <row r="108">
-      <c r="A108" s="6" t="inlineStr">
-        <is>
-          <t>margin</t>
-        </is>
-      </c>
-      <c r="B108" s="6" t="inlineStr">
-        <is>
-          <t>Fix action 5</t>
-        </is>
-      </c>
-      <c r="C108" s="7" t="inlineStr">
-        <is>
-          <t>Don't discount to win. A discount is the fastest way to buy work you'll resent delivering.</t>
-        </is>
-      </c>
-      <c r="D108" s="7" t="inlineStr"/>
-      <c r="E108" s="8" t="inlineStr">
-        <is>
-          <t>always prints</t>
-        </is>
-      </c>
-    </row>
   </sheetData>
-  <autoFilter ref="A2:E108"/>
+  <autoFilter ref="A2:E106"/>
   <mergeCells count="1">
     <mergeCell ref="A1:E1"/>
   </mergeCells>
@@ -18404,7 +18358,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:C44"/>
+  <dimension ref="A1:C42"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="13" customWidth="1" min="1" max="1"/>
@@ -18626,17 +18580,17 @@
     <row r="14">
       <c r="A14" s="6" t="inlineStr">
         <is>
-          <t>talent</t>
+          <t>fulfilment</t>
         </is>
       </c>
       <c r="B14" s="6" t="inlineStr">
         <is>
-          <t>Item 5</t>
+          <t>Lead line</t>
         </is>
       </c>
       <c r="C14" s="7" t="inlineStr">
         <is>
-          <t>Don't redraw the org chart. What's missing is a person who doesn't exist, not a diagram.</t>
+          <t>Until you've done the above, leave these alone.</t>
         </is>
       </c>
     </row>
@@ -18648,12 +18602,12 @@
       </c>
       <c r="B15" s="6" t="inlineStr">
         <is>
-          <t>Lead line</t>
+          <t>Item 1</t>
         </is>
       </c>
       <c r="C15" s="7" t="inlineStr">
         <is>
-          <t>Until you can deliver what you've already sold, leave these alone.</t>
+          <t>Don't take on new customers until you've done the above.</t>
         </is>
       </c>
     </row>
@@ -18665,12 +18619,12 @@
       </c>
       <c r="B16" s="6" t="inlineStr">
         <is>
-          <t>Item 1</t>
+          <t>Item 2</t>
         </is>
       </c>
       <c r="C16" s="7" t="inlineStr">
         <is>
-          <t>Don't chase new customers. You'd be damaging the ones you have to serve the ones you win.</t>
+          <t>Don't start something new.</t>
         </is>
       </c>
     </row>
@@ -18682,12 +18636,12 @@
       </c>
       <c r="B17" s="6" t="inlineStr">
         <is>
-          <t>Item 2</t>
+          <t>Item 3</t>
         </is>
       </c>
       <c r="C17" s="7" t="inlineStr">
         <is>
-          <t>Don't increase marketing spend. Adding demand to a full pipeline is the classic accelerant.</t>
+          <t>Don't drop your prices.</t>
         </is>
       </c>
     </row>
@@ -18699,46 +18653,46 @@
       </c>
       <c r="B18" s="6" t="inlineStr">
         <is>
-          <t>Item 3</t>
+          <t>Item 4</t>
         </is>
       </c>
       <c r="C18" s="7" t="inlineStr">
         <is>
-          <t>Don't launch a new service line. New work is slow work while the process is still being learned.</t>
+          <t>Don't promise a shorter lead time to win a job.</t>
         </is>
       </c>
     </row>
     <row r="19">
       <c r="A19" s="6" t="inlineStr">
         <is>
-          <t>fulfilment</t>
+          <t>value</t>
         </is>
       </c>
       <c r="B19" s="6" t="inlineStr">
         <is>
-          <t>Item 4</t>
+          <t>Lead line</t>
         </is>
       </c>
       <c r="C19" s="7" t="inlineStr">
         <is>
-          <t>Don't drop your prices. You've got more demand than capacity, which is the one time raising them is easy.</t>
+          <t>Until customers stay, leave these alone.</t>
         </is>
       </c>
     </row>
     <row r="20">
       <c r="A20" s="6" t="inlineStr">
         <is>
-          <t>fulfilment</t>
+          <t>value</t>
         </is>
       </c>
       <c r="B20" s="6" t="inlineStr">
         <is>
-          <t>Item 5</t>
+          <t>Item 1</t>
         </is>
       </c>
       <c r="C20" s="7" t="inlineStr">
         <is>
-          <t>Don't promise a shorter lead time to win a job. That's where the quality problem starts.</t>
+          <t>Don't spend more on acquisition. You'd be paying to fill a bucket with a hole in it.</t>
         </is>
       </c>
     </row>
@@ -18750,12 +18704,12 @@
       </c>
       <c r="B21" s="6" t="inlineStr">
         <is>
-          <t>Lead line</t>
+          <t>Item 2</t>
         </is>
       </c>
       <c r="C21" s="7" t="inlineStr">
         <is>
-          <t>Until customers stay, leave these alone.</t>
+          <t>Don't raise prices. Value perception is already the problem.</t>
         </is>
       </c>
     </row>
@@ -18767,12 +18721,12 @@
       </c>
       <c r="B22" s="6" t="inlineStr">
         <is>
-          <t>Item 1</t>
+          <t>Item 3</t>
         </is>
       </c>
       <c r="C22" s="7" t="inlineStr">
         <is>
-          <t>Don't spend more on acquisition. You'd be paying to fill a bucket with a hole in it.</t>
+          <t>Don't add a new product for existing customers who aren't buying the current one.</t>
         </is>
       </c>
     </row>
@@ -18784,12 +18738,12 @@
       </c>
       <c r="B23" s="6" t="inlineStr">
         <is>
-          <t>Item 2</t>
+          <t>Item 4</t>
         </is>
       </c>
       <c r="C23" s="7" t="inlineStr">
         <is>
-          <t>Don't raise prices. Value perception is already the problem.</t>
+          <t>Don't expand into a new market. You'd take the retention problem with you.</t>
         </is>
       </c>
     </row>
@@ -18801,46 +18755,46 @@
       </c>
       <c r="B24" s="6" t="inlineStr">
         <is>
-          <t>Item 3</t>
+          <t>Item 5</t>
         </is>
       </c>
       <c r="C24" s="7" t="inlineStr">
         <is>
-          <t>Don't add a new product for existing customers who aren't buying the current one.</t>
+          <t>Don't run a loyalty programme. A discount doesn't fix a value gap, it confirms one.</t>
         </is>
       </c>
     </row>
     <row r="25">
       <c r="A25" s="6" t="inlineStr">
         <is>
-          <t>value</t>
+          <t>offer</t>
         </is>
       </c>
       <c r="B25" s="6" t="inlineStr">
         <is>
-          <t>Item 4</t>
+          <t>Lead line</t>
         </is>
       </c>
       <c r="C25" s="7" t="inlineStr">
         <is>
-          <t>Don't expand into a new market. You'd take the retention problem with you.</t>
+          <t>Until the offer lands, leave these alone.</t>
         </is>
       </c>
     </row>
     <row r="26">
       <c r="A26" s="6" t="inlineStr">
         <is>
-          <t>value</t>
+          <t>offer</t>
         </is>
       </c>
       <c r="B26" s="6" t="inlineStr">
         <is>
-          <t>Item 5</t>
+          <t>Item 1</t>
         </is>
       </c>
       <c r="C26" s="7" t="inlineStr">
         <is>
-          <t>Don't run a loyalty programme. A discount doesn't fix a value gap, it confirms one.</t>
+          <t>Don't buy more leads. You'd pay more money for the same conversion rate.</t>
         </is>
       </c>
     </row>
@@ -18852,12 +18806,12 @@
       </c>
       <c r="B27" s="6" t="inlineStr">
         <is>
-          <t>Lead line</t>
+          <t>Item 2</t>
         </is>
       </c>
       <c r="C27" s="7" t="inlineStr">
         <is>
-          <t>Until the offer lands, leave these alone.</t>
+          <t>Don't hire a salesperson. They'd fail against the same offer you're failing against.</t>
         </is>
       </c>
     </row>
@@ -18869,12 +18823,12 @@
       </c>
       <c r="B28" s="6" t="inlineStr">
         <is>
-          <t>Item 1</t>
+          <t>Item 3</t>
         </is>
       </c>
       <c r="C28" s="7" t="inlineStr">
         <is>
-          <t>Don't buy more leads. You'd pay more money for the same conversion rate.</t>
+          <t>Don't cut your price. Price is rarely the real reason, and you can't test it while the offer is unclear.</t>
         </is>
       </c>
     </row>
@@ -18886,12 +18840,12 @@
       </c>
       <c r="B29" s="6" t="inlineStr">
         <is>
-          <t>Item 2</t>
+          <t>Item 4</t>
         </is>
       </c>
       <c r="C29" s="7" t="inlineStr">
         <is>
-          <t>Don't hire a salesperson. They'd fail against the same offer you're failing against.</t>
+          <t>Don't add more options. More choice is part of why these deals are stalling.</t>
         </is>
       </c>
     </row>
@@ -18903,46 +18857,46 @@
       </c>
       <c r="B30" s="6" t="inlineStr">
         <is>
-          <t>Item 3</t>
+          <t>Item 5</t>
         </is>
       </c>
       <c r="C30" s="7" t="inlineStr">
         <is>
-          <t>Don't cut your price. Price is rarely the real reason, and you can't test it while the offer is unclear.</t>
+          <t>Don't rebrand. The words are the problem, not the logo.</t>
         </is>
       </c>
     </row>
     <row r="31">
       <c r="A31" s="6" t="inlineStr">
         <is>
-          <t>offer</t>
+          <t>demand</t>
         </is>
       </c>
       <c r="B31" s="6" t="inlineStr">
         <is>
-          <t>Item 4</t>
+          <t>Lead line</t>
         </is>
       </c>
       <c r="C31" s="7" t="inlineStr">
         <is>
-          <t>Don't add more options. More choice is part of why these deals are stalling.</t>
+          <t>Until enquiries lift, leave these alone.</t>
         </is>
       </c>
     </row>
     <row r="32">
       <c r="A32" s="6" t="inlineStr">
         <is>
-          <t>offer</t>
+          <t>demand</t>
         </is>
       </c>
       <c r="B32" s="6" t="inlineStr">
         <is>
-          <t>Item 5</t>
+          <t>Item 1</t>
         </is>
       </c>
       <c r="C32" s="7" t="inlineStr">
         <is>
-          <t>Don't rebrand. The words are the problem, not the logo.</t>
+          <t>Don't hire. You'd be adding capacity to capacity you already can't fill.</t>
         </is>
       </c>
     </row>
@@ -18954,12 +18908,12 @@
       </c>
       <c r="B33" s="6" t="inlineStr">
         <is>
-          <t>Lead line</t>
+          <t>Item 2</t>
         </is>
       </c>
       <c r="C33" s="7" t="inlineStr">
         <is>
-          <t>Until enquiries lift, leave these alone.</t>
+          <t>Don't build a new product. The one you have hasn't been shown to enough people.</t>
         </is>
       </c>
     </row>
@@ -18971,12 +18925,12 @@
       </c>
       <c r="B34" s="6" t="inlineStr">
         <is>
-          <t>Item 1</t>
+          <t>Item 3</t>
         </is>
       </c>
       <c r="C34" s="7" t="inlineStr">
         <is>
-          <t>Don't hire. You'd be adding capacity to capacity you already can't fill.</t>
+          <t>Don't cut prices to stimulate demand. It rarely moves volume, and it permanently resets what customers expect to pay.</t>
         </is>
       </c>
     </row>
@@ -18988,12 +18942,12 @@
       </c>
       <c r="B35" s="6" t="inlineStr">
         <is>
-          <t>Item 2</t>
+          <t>Item 4</t>
         </is>
       </c>
       <c r="C35" s="7" t="inlineStr">
         <is>
-          <t>Don't build a new product. The one you have hasn't been shown to enough people.</t>
+          <t>Don't spread across five channels at once. One channel run properly beats five run badly.</t>
         </is>
       </c>
     </row>
@@ -19005,46 +18959,46 @@
       </c>
       <c r="B36" s="6" t="inlineStr">
         <is>
-          <t>Item 3</t>
+          <t>Item 5</t>
         </is>
       </c>
       <c r="C36" s="7" t="inlineStr">
         <is>
-          <t>Don't cut prices to stimulate demand. It rarely moves volume, and it permanently resets what customers expect to pay.</t>
+          <t>Don't wait for referrals to pick back up. Referral volume follows the number of customers you have, and that's the number that's short.</t>
         </is>
       </c>
     </row>
     <row r="37">
       <c r="A37" s="6" t="inlineStr">
         <is>
-          <t>demand</t>
+          <t>margin</t>
         </is>
       </c>
       <c r="B37" s="6" t="inlineStr">
         <is>
-          <t>Item 4</t>
+          <t>Lead line</t>
         </is>
       </c>
       <c r="C37" s="7" t="inlineStr">
         <is>
-          <t>Don't spread across five channels at once. One channel run properly beats five run badly.</t>
+          <t>Until the margin moves, leave these alone.</t>
         </is>
       </c>
     </row>
     <row r="38">
       <c r="A38" s="6" t="inlineStr">
         <is>
-          <t>demand</t>
+          <t>margin</t>
         </is>
       </c>
       <c r="B38" s="6" t="inlineStr">
         <is>
-          <t>Item 5</t>
+          <t>Item 1</t>
         </is>
       </c>
       <c r="C38" s="7" t="inlineStr">
         <is>
-          <t>Don't wait for referrals to pick back up. Referral volume follows the number of customers you have, and that's the number that's short.</t>
+          <t>Don't chase volume. More work at this margin is more risk for the same money.</t>
         </is>
       </c>
     </row>
@@ -19056,12 +19010,12 @@
       </c>
       <c r="B39" s="6" t="inlineStr">
         <is>
-          <t>Lead line</t>
+          <t>Item 2</t>
         </is>
       </c>
       <c r="C39" s="7" t="inlineStr">
         <is>
-          <t>Until the margin moves, leave these alone.</t>
+          <t>Don't hire. Every head you add at this margin needs a lot of revenue standing behind it.</t>
         </is>
       </c>
     </row>
@@ -19073,12 +19027,12 @@
       </c>
       <c r="B40" s="6" t="inlineStr">
         <is>
-          <t>Item 1</t>
+          <t>Item 3</t>
         </is>
       </c>
       <c r="C40" s="7" t="inlineStr">
         <is>
-          <t>Don't chase volume. More work at this margin is more risk for the same money.</t>
+          <t>Don't take the big thin job because it's good for the brand. Reputation doesn't pay wages.</t>
         </is>
       </c>
     </row>
@@ -19090,12 +19044,12 @@
       </c>
       <c r="B41" s="6" t="inlineStr">
         <is>
-          <t>Item 2</t>
+          <t>Item 4</t>
         </is>
       </c>
       <c r="C41" s="7" t="inlineStr">
         <is>
-          <t>Don't hire. Every head you add at this margin needs a lot of revenue standing behind it.</t>
+          <t>Don't discount anything. There's nothing left to give away.</t>
         </is>
       </c>
     </row>
@@ -19107,51 +19061,17 @@
       </c>
       <c r="B42" s="6" t="inlineStr">
         <is>
-          <t>Item 3</t>
+          <t>Item 5</t>
         </is>
       </c>
       <c r="C42" s="7" t="inlineStr">
         <is>
-          <t>Don't take the big thin job because it's good for the brand. Reputation doesn't pay wages.</t>
-        </is>
-      </c>
-    </row>
-    <row r="43">
-      <c r="A43" s="6" t="inlineStr">
-        <is>
-          <t>margin</t>
-        </is>
-      </c>
-      <c r="B43" s="6" t="inlineStr">
-        <is>
-          <t>Item 4</t>
-        </is>
-      </c>
-      <c r="C43" s="7" t="inlineStr">
-        <is>
-          <t>Don't discount anything. There's nothing left to give away.</t>
-        </is>
-      </c>
-    </row>
-    <row r="44">
-      <c r="A44" s="6" t="inlineStr">
-        <is>
-          <t>margin</t>
-        </is>
-      </c>
-      <c r="B44" s="6" t="inlineStr">
-        <is>
-          <t>Item 5</t>
-        </is>
-      </c>
-      <c r="C44" s="7" t="inlineStr">
-        <is>
           <t>Don't invest in growth. Growing an unprofitable model makes it unprofitable faster.</t>
         </is>
       </c>
     </row>
   </sheetData>
-  <autoFilter ref="A2:C44"/>
+  <autoFilter ref="A2:C42"/>
   <mergeCells count="1">
     <mergeCell ref="A1:C1"/>
   </mergeCells>

</xml_diff>